<commit_message>
add 2 new calculator card and fix multi bug
</commit_message>
<xml_diff>
--- a/assets/data-source/data.xlsx
+++ b/assets/data-source/data.xlsx
@@ -1,27 +1,38 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Venus\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9DB75AE-4093-48F0-BEEF-8CFBF8C13DEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9231CA9A-1CF2-4A8C-B435-2E0082B2318E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="736" activeTab="1" xr2:uid="{2E6F1639-AB3B-4860-9C01-087F2448B9B1}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="23657" windowHeight="15394" tabRatio="736" activeTab="1" xr2:uid="{2E6F1639-AB3B-4860-9C01-087F2448B9B1}"/>
   </bookViews>
   <sheets>
     <sheet name="پایه سنوات طرح طبقه" sheetId="33" r:id="rId1"/>
     <sheet name="پایه سنوات عادی و داده ها" sheetId="34" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="111">
   <si>
     <t>پایه سنوات</t>
   </si>
@@ -93,15 +104,6 @@
   </si>
   <si>
     <t>حق تاهل</t>
-  </si>
-  <si>
-    <t xml:space="preserve">مبلغ عائله مندی به یک فرزند واجد شرایط </t>
-  </si>
-  <si>
-    <t>مبلغ حداقل عیدی ماهیانه</t>
-  </si>
-  <si>
-    <t>مبلغ حداکثر عیدی ماهیانه</t>
   </si>
   <si>
     <t>فرمول افزایش مزدی</t>
@@ -356,7 +358,13 @@
     <t>صبح  و شب یا عصر و شب 22.5%</t>
   </si>
   <si>
-    <t>پایه سنواتی  گذشته</t>
+    <t>مبلغ حداقل عیدی پاداش ماهیانه</t>
+  </si>
+  <si>
+    <t>مبلغ حداکثر عیدی پاداش  ماهیانه</t>
+  </si>
+  <si>
+    <t xml:space="preserve">مبلغ عائله مندی  یک فرزند واجد شرایط </t>
   </si>
 </sst>
 </file>
@@ -368,7 +376,7 @@
     <numFmt numFmtId="165" formatCode="0;[Red]0"/>
     <numFmt numFmtId="166" formatCode="0.000;[Red]0.000"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="14"/>
       <name val="B Nazanin"/>
@@ -987,17 +995,47 @@
     <xf numFmtId="0" fontId="10" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="10" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1026,47 +1064,17 @@
     <xf numFmtId="165" fontId="5" fillId="4" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="10" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1373,581 +1381,581 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F3FFB2F-BC88-43B7-B5AC-FC5BC58FCAEB}">
   <dimension ref="A1:DH348"/>
-  <sheetFormatPr defaultColWidth="14.4609375" defaultRowHeight="17.399999999999999"/>
+  <sheetFormatPr defaultColWidth="14.46484375" defaultRowHeight="25.75" x14ac:dyDescent="0.9"/>
   <cols>
-    <col min="1" max="1" width="14.4609375" style="37" customWidth="1"/>
-    <col min="2" max="16384" width="14.4609375" style="31"/>
+    <col min="1" max="1" width="14.46484375" style="37" customWidth="1"/>
+    <col min="2" max="16384" width="14.46484375" style="31"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:112" s="39" customFormat="1" ht="23.1" customHeight="1">
+    <row r="1" spans="1:112" s="39" customFormat="1" ht="23.15" customHeight="1" x14ac:dyDescent="0.9">
       <c r="A1" s="38" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="42">
+      <c r="B1" s="67">
         <v>1369</v>
       </c>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="42">
+      <c r="C1" s="68"/>
+      <c r="D1" s="68"/>
+      <c r="E1" s="67">
         <v>1370</v>
       </c>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="42">
+      <c r="F1" s="68"/>
+      <c r="G1" s="68"/>
+      <c r="H1" s="67">
         <v>1371</v>
       </c>
-      <c r="I1" s="43"/>
-      <c r="J1" s="43"/>
-      <c r="K1" s="42">
+      <c r="I1" s="68"/>
+      <c r="J1" s="68"/>
+      <c r="K1" s="67">
         <v>1372</v>
       </c>
-      <c r="L1" s="43"/>
-      <c r="M1" s="43"/>
-      <c r="N1" s="42">
+      <c r="L1" s="68"/>
+      <c r="M1" s="68"/>
+      <c r="N1" s="67">
         <v>1373</v>
       </c>
-      <c r="O1" s="43"/>
-      <c r="P1" s="43"/>
-      <c r="Q1" s="42">
+      <c r="O1" s="68"/>
+      <c r="P1" s="68"/>
+      <c r="Q1" s="67">
         <v>1374</v>
       </c>
-      <c r="R1" s="43"/>
-      <c r="S1" s="43"/>
-      <c r="T1" s="42">
+      <c r="R1" s="68"/>
+      <c r="S1" s="68"/>
+      <c r="T1" s="67">
         <v>1375</v>
       </c>
-      <c r="U1" s="43"/>
-      <c r="V1" s="43"/>
-      <c r="W1" s="42">
+      <c r="U1" s="68"/>
+      <c r="V1" s="68"/>
+      <c r="W1" s="67">
         <v>1376</v>
       </c>
-      <c r="X1" s="43"/>
-      <c r="Y1" s="43"/>
-      <c r="Z1" s="42">
+      <c r="X1" s="68"/>
+      <c r="Y1" s="68"/>
+      <c r="Z1" s="67">
         <v>1377</v>
       </c>
-      <c r="AA1" s="43"/>
-      <c r="AB1" s="43"/>
-      <c r="AC1" s="42">
+      <c r="AA1" s="68"/>
+      <c r="AB1" s="68"/>
+      <c r="AC1" s="67">
         <v>1378</v>
       </c>
-      <c r="AD1" s="43"/>
-      <c r="AE1" s="43"/>
-      <c r="AF1" s="42">
+      <c r="AD1" s="68"/>
+      <c r="AE1" s="68"/>
+      <c r="AF1" s="67">
         <v>1379</v>
       </c>
-      <c r="AG1" s="43"/>
-      <c r="AH1" s="43"/>
-      <c r="AI1" s="42">
+      <c r="AG1" s="68"/>
+      <c r="AH1" s="68"/>
+      <c r="AI1" s="67">
         <v>1380</v>
       </c>
-      <c r="AJ1" s="43"/>
-      <c r="AK1" s="43"/>
-      <c r="AL1" s="42">
+      <c r="AJ1" s="68"/>
+      <c r="AK1" s="68"/>
+      <c r="AL1" s="67">
         <v>1381</v>
       </c>
-      <c r="AM1" s="43"/>
-      <c r="AN1" s="43"/>
-      <c r="AO1" s="42">
+      <c r="AM1" s="68"/>
+      <c r="AN1" s="68"/>
+      <c r="AO1" s="67">
         <v>1382</v>
       </c>
-      <c r="AP1" s="43"/>
-      <c r="AQ1" s="43"/>
-      <c r="AR1" s="42">
+      <c r="AP1" s="68"/>
+      <c r="AQ1" s="68"/>
+      <c r="AR1" s="67">
         <v>1383</v>
       </c>
-      <c r="AS1" s="43"/>
-      <c r="AT1" s="43"/>
-      <c r="AU1" s="42">
+      <c r="AS1" s="68"/>
+      <c r="AT1" s="68"/>
+      <c r="AU1" s="67">
         <v>1384</v>
       </c>
-      <c r="AV1" s="43"/>
-      <c r="AW1" s="43"/>
-      <c r="AX1" s="42">
+      <c r="AV1" s="68"/>
+      <c r="AW1" s="68"/>
+      <c r="AX1" s="67">
         <v>1385</v>
       </c>
-      <c r="AY1" s="43"/>
-      <c r="AZ1" s="43"/>
-      <c r="BA1" s="42">
+      <c r="AY1" s="68"/>
+      <c r="AZ1" s="68"/>
+      <c r="BA1" s="67">
         <v>1386</v>
       </c>
-      <c r="BB1" s="43"/>
-      <c r="BC1" s="43"/>
-      <c r="BD1" s="42">
+      <c r="BB1" s="68"/>
+      <c r="BC1" s="68"/>
+      <c r="BD1" s="67">
         <v>1387</v>
       </c>
-      <c r="BE1" s="43"/>
-      <c r="BF1" s="43"/>
-      <c r="BG1" s="42">
+      <c r="BE1" s="68"/>
+      <c r="BF1" s="68"/>
+      <c r="BG1" s="67">
         <v>1388</v>
       </c>
-      <c r="BH1" s="43"/>
-      <c r="BI1" s="43"/>
-      <c r="BJ1" s="42">
+      <c r="BH1" s="68"/>
+      <c r="BI1" s="68"/>
+      <c r="BJ1" s="67">
         <v>1389</v>
       </c>
-      <c r="BK1" s="43"/>
-      <c r="BL1" s="43"/>
-      <c r="BM1" s="42">
+      <c r="BK1" s="68"/>
+      <c r="BL1" s="68"/>
+      <c r="BM1" s="67">
         <v>1390</v>
       </c>
-      <c r="BN1" s="43"/>
-      <c r="BO1" s="43"/>
-      <c r="BP1" s="42">
+      <c r="BN1" s="68"/>
+      <c r="BO1" s="68"/>
+      <c r="BP1" s="67">
         <v>1391</v>
       </c>
-      <c r="BQ1" s="43"/>
-      <c r="BR1" s="43"/>
-      <c r="BS1" s="42">
+      <c r="BQ1" s="68"/>
+      <c r="BR1" s="68"/>
+      <c r="BS1" s="67">
         <v>1392</v>
       </c>
-      <c r="BT1" s="43"/>
-      <c r="BU1" s="43"/>
-      <c r="BV1" s="42">
+      <c r="BT1" s="68"/>
+      <c r="BU1" s="68"/>
+      <c r="BV1" s="67">
         <v>1393</v>
       </c>
-      <c r="BW1" s="43"/>
-      <c r="BX1" s="43"/>
-      <c r="BY1" s="42">
+      <c r="BW1" s="68"/>
+      <c r="BX1" s="68"/>
+      <c r="BY1" s="67">
         <v>1394</v>
       </c>
-      <c r="BZ1" s="43"/>
-      <c r="CA1" s="43"/>
-      <c r="CB1" s="42">
+      <c r="BZ1" s="68"/>
+      <c r="CA1" s="68"/>
+      <c r="CB1" s="67">
         <v>1395</v>
       </c>
-      <c r="CC1" s="43"/>
-      <c r="CD1" s="43"/>
-      <c r="CE1" s="42">
+      <c r="CC1" s="68"/>
+      <c r="CD1" s="68"/>
+      <c r="CE1" s="67">
         <v>1396</v>
       </c>
-      <c r="CF1" s="43"/>
-      <c r="CG1" s="43"/>
-      <c r="CH1" s="42">
+      <c r="CF1" s="68"/>
+      <c r="CG1" s="68"/>
+      <c r="CH1" s="67">
         <v>1397</v>
       </c>
-      <c r="CI1" s="43"/>
-      <c r="CJ1" s="43"/>
-      <c r="CK1" s="42">
+      <c r="CI1" s="68"/>
+      <c r="CJ1" s="68"/>
+      <c r="CK1" s="67">
         <v>1398</v>
       </c>
-      <c r="CL1" s="43"/>
-      <c r="CM1" s="43"/>
-      <c r="CN1" s="42">
+      <c r="CL1" s="68"/>
+      <c r="CM1" s="68"/>
+      <c r="CN1" s="67">
         <v>1399</v>
       </c>
-      <c r="CO1" s="43"/>
-      <c r="CP1" s="43"/>
-      <c r="CQ1" s="42">
+      <c r="CO1" s="68"/>
+      <c r="CP1" s="68"/>
+      <c r="CQ1" s="67">
         <v>1400</v>
       </c>
-      <c r="CR1" s="43"/>
-      <c r="CS1" s="43"/>
-      <c r="CT1" s="42">
+      <c r="CR1" s="68"/>
+      <c r="CS1" s="68"/>
+      <c r="CT1" s="67">
         <v>1401</v>
       </c>
-      <c r="CU1" s="43"/>
-      <c r="CV1" s="43"/>
-      <c r="CW1" s="42">
+      <c r="CU1" s="68"/>
+      <c r="CV1" s="68"/>
+      <c r="CW1" s="67">
         <v>1402</v>
       </c>
-      <c r="CX1" s="43"/>
-      <c r="CY1" s="43"/>
-      <c r="CZ1" s="42">
+      <c r="CX1" s="68"/>
+      <c r="CY1" s="68"/>
+      <c r="CZ1" s="67">
         <v>1403</v>
       </c>
-      <c r="DA1" s="43"/>
-      <c r="DB1" s="43"/>
-      <c r="DC1" s="42">
+      <c r="DA1" s="68"/>
+      <c r="DB1" s="68"/>
+      <c r="DC1" s="67">
         <v>1404</v>
       </c>
-      <c r="DD1" s="43"/>
-      <c r="DE1" s="43"/>
-      <c r="DF1" s="42">
+      <c r="DD1" s="68"/>
+      <c r="DE1" s="68"/>
+      <c r="DF1" s="67">
         <v>1405</v>
       </c>
-      <c r="DG1" s="43"/>
-      <c r="DH1" s="43"/>
-    </row>
-    <row r="2" spans="1:112" s="41" customFormat="1" ht="31.35" customHeight="1">
+      <c r="DG1" s="68"/>
+      <c r="DH1" s="68"/>
+    </row>
+    <row r="2" spans="1:112" s="41" customFormat="1" ht="31.4" customHeight="1" x14ac:dyDescent="0.9">
       <c r="A2" s="40" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="44">
+      <c r="B2" s="65">
         <v>1.1399999999999999</v>
       </c>
-      <c r="C2" s="44"/>
-      <c r="D2" s="44"/>
-      <c r="E2" s="44">
+      <c r="C2" s="65"/>
+      <c r="D2" s="65"/>
+      <c r="E2" s="65">
         <v>1.1200000000000001</v>
       </c>
-      <c r="F2" s="44"/>
-      <c r="G2" s="44"/>
-      <c r="H2" s="44">
+      <c r="F2" s="65"/>
+      <c r="G2" s="65"/>
+      <c r="H2" s="65">
         <v>1.101</v>
       </c>
-      <c r="I2" s="44"/>
-      <c r="J2" s="44"/>
-      <c r="K2" s="44">
+      <c r="I2" s="65"/>
+      <c r="J2" s="65"/>
+      <c r="K2" s="65">
         <v>1.1299999999999999</v>
       </c>
-      <c r="L2" s="44"/>
-      <c r="M2" s="44"/>
-      <c r="N2" s="44">
+      <c r="L2" s="65"/>
+      <c r="M2" s="65"/>
+      <c r="N2" s="65">
         <v>1.1499999999999999</v>
       </c>
-      <c r="O2" s="44"/>
-      <c r="P2" s="44"/>
-      <c r="Q2" s="44">
+      <c r="O2" s="65"/>
+      <c r="P2" s="65"/>
+      <c r="Q2" s="65">
         <v>1.26</v>
       </c>
-      <c r="R2" s="44"/>
-      <c r="S2" s="44"/>
-      <c r="T2" s="44">
+      <c r="R2" s="65"/>
+      <c r="S2" s="65"/>
+      <c r="T2" s="65">
         <v>1.38</v>
       </c>
-      <c r="U2" s="44"/>
-      <c r="V2" s="44"/>
-      <c r="W2" s="44">
+      <c r="U2" s="65"/>
+      <c r="V2" s="65"/>
+      <c r="W2" s="65">
         <v>1.21</v>
       </c>
-      <c r="X2" s="44"/>
-      <c r="Y2" s="44"/>
-      <c r="Z2" s="44">
+      <c r="X2" s="65"/>
+      <c r="Y2" s="65"/>
+      <c r="Z2" s="65">
         <v>1.22</v>
       </c>
-      <c r="AA2" s="44"/>
-      <c r="AB2" s="44"/>
-      <c r="AC2" s="44">
+      <c r="AA2" s="65"/>
+      <c r="AB2" s="65"/>
+      <c r="AC2" s="65">
         <v>1.32</v>
       </c>
-      <c r="AD2" s="44"/>
-      <c r="AE2" s="44"/>
-      <c r="AF2" s="44">
+      <c r="AD2" s="65"/>
+      <c r="AE2" s="65"/>
+      <c r="AF2" s="65">
         <v>1.45</v>
       </c>
-      <c r="AG2" s="44"/>
-      <c r="AH2" s="44"/>
-      <c r="AI2" s="44">
+      <c r="AG2" s="65"/>
+      <c r="AH2" s="65"/>
+      <c r="AI2" s="65">
         <v>1.1200000000000001</v>
       </c>
-      <c r="AJ2" s="44"/>
-      <c r="AK2" s="44"/>
-      <c r="AL2" s="44">
+      <c r="AJ2" s="65"/>
+      <c r="AK2" s="65"/>
+      <c r="AL2" s="65">
         <v>1.17</v>
       </c>
-      <c r="AM2" s="44"/>
-      <c r="AN2" s="44"/>
-      <c r="AO2" s="44">
+      <c r="AM2" s="65"/>
+      <c r="AN2" s="65"/>
+      <c r="AO2" s="65">
         <v>1.1399999999999999</v>
       </c>
-      <c r="AP2" s="44"/>
-      <c r="AQ2" s="44"/>
-      <c r="AR2" s="44">
+      <c r="AP2" s="65"/>
+      <c r="AQ2" s="65"/>
+      <c r="AR2" s="65">
         <v>1.1200000000000001</v>
       </c>
-      <c r="AS2" s="44"/>
-      <c r="AT2" s="44"/>
-      <c r="AU2" s="44">
+      <c r="AS2" s="65"/>
+      <c r="AT2" s="65"/>
+      <c r="AU2" s="65">
         <v>1.101</v>
       </c>
-      <c r="AV2" s="44"/>
-      <c r="AW2" s="44"/>
-      <c r="AX2" s="44">
+      <c r="AV2" s="65"/>
+      <c r="AW2" s="65"/>
+      <c r="AX2" s="65">
         <v>1.1299999999999999</v>
       </c>
-      <c r="AY2" s="44"/>
-      <c r="AZ2" s="44"/>
-      <c r="BA2" s="44">
+      <c r="AY2" s="65"/>
+      <c r="AZ2" s="65"/>
+      <c r="BA2" s="65">
         <v>1.1499999999999999</v>
       </c>
-      <c r="BB2" s="44"/>
-      <c r="BC2" s="44"/>
-      <c r="BD2" s="44">
+      <c r="BB2" s="65"/>
+      <c r="BC2" s="65"/>
+      <c r="BD2" s="65">
         <v>1.26</v>
       </c>
-      <c r="BE2" s="44"/>
-      <c r="BF2" s="44"/>
-      <c r="BG2" s="44">
+      <c r="BE2" s="65"/>
+      <c r="BF2" s="65"/>
+      <c r="BG2" s="65">
         <v>1.38</v>
       </c>
-      <c r="BH2" s="44"/>
-      <c r="BI2" s="44"/>
-      <c r="BJ2" s="44">
+      <c r="BH2" s="65"/>
+      <c r="BI2" s="65"/>
+      <c r="BJ2" s="65">
         <v>1.21</v>
       </c>
-      <c r="BK2" s="44"/>
-      <c r="BL2" s="44"/>
-      <c r="BM2" s="44">
+      <c r="BK2" s="65"/>
+      <c r="BL2" s="65"/>
+      <c r="BM2" s="65">
         <v>1.22</v>
       </c>
-      <c r="BN2" s="44"/>
-      <c r="BO2" s="44"/>
-      <c r="BP2" s="44">
+      <c r="BN2" s="65"/>
+      <c r="BO2" s="65"/>
+      <c r="BP2" s="65">
         <v>1.1000000000000001</v>
       </c>
-      <c r="BQ2" s="44"/>
-      <c r="BR2" s="44"/>
-      <c r="BS2" s="44">
+      <c r="BQ2" s="65"/>
+      <c r="BR2" s="65"/>
+      <c r="BS2" s="65">
         <v>1.1000000000000001</v>
       </c>
-      <c r="BT2" s="44"/>
-      <c r="BU2" s="44"/>
-      <c r="BV2" s="44">
+      <c r="BT2" s="65"/>
+      <c r="BU2" s="65"/>
+      <c r="BV2" s="65">
         <v>1.1200000000000001</v>
       </c>
-      <c r="BW2" s="44"/>
-      <c r="BX2" s="44"/>
-      <c r="BY2" s="44">
+      <c r="BW2" s="65"/>
+      <c r="BX2" s="65"/>
+      <c r="BY2" s="65">
         <v>1.17</v>
       </c>
-      <c r="BZ2" s="44"/>
-      <c r="CA2" s="44"/>
-      <c r="CB2" s="44">
+      <c r="BZ2" s="65"/>
+      <c r="CA2" s="65"/>
+      <c r="CB2" s="65">
         <v>1.1399999999999999</v>
       </c>
-      <c r="CC2" s="44"/>
-      <c r="CD2" s="44"/>
-      <c r="CE2" s="44">
+      <c r="CC2" s="65"/>
+      <c r="CD2" s="65"/>
+      <c r="CE2" s="65">
         <v>1.1200000000000001</v>
       </c>
-      <c r="CF2" s="44"/>
-      <c r="CG2" s="44"/>
-      <c r="CH2" s="44">
+      <c r="CF2" s="65"/>
+      <c r="CG2" s="65"/>
+      <c r="CH2" s="65">
         <v>1.101</v>
       </c>
-      <c r="CI2" s="44"/>
-      <c r="CJ2" s="44"/>
-      <c r="CK2" s="44">
+      <c r="CI2" s="65"/>
+      <c r="CJ2" s="65"/>
+      <c r="CK2" s="65">
         <v>1.1299999999999999</v>
       </c>
-      <c r="CL2" s="44"/>
-      <c r="CM2" s="44"/>
-      <c r="CN2" s="44">
+      <c r="CL2" s="65"/>
+      <c r="CM2" s="65"/>
+      <c r="CN2" s="65">
         <v>1.1499999999999999</v>
       </c>
-      <c r="CO2" s="44"/>
-      <c r="CP2" s="44"/>
-      <c r="CQ2" s="44">
+      <c r="CO2" s="65"/>
+      <c r="CP2" s="65"/>
+      <c r="CQ2" s="65">
         <v>1.26</v>
       </c>
-      <c r="CR2" s="44"/>
-      <c r="CS2" s="44"/>
-      <c r="CT2" s="44">
+      <c r="CR2" s="65"/>
+      <c r="CS2" s="65"/>
+      <c r="CT2" s="65">
         <v>1.38</v>
       </c>
-      <c r="CU2" s="44"/>
-      <c r="CV2" s="44"/>
-      <c r="CW2" s="44">
+      <c r="CU2" s="65"/>
+      <c r="CV2" s="65"/>
+      <c r="CW2" s="65">
         <v>1.21</v>
       </c>
-      <c r="CX2" s="44"/>
-      <c r="CY2" s="44"/>
-      <c r="CZ2" s="44">
+      <c r="CX2" s="65"/>
+      <c r="CY2" s="65"/>
+      <c r="CZ2" s="65">
         <v>1.22</v>
       </c>
-      <c r="DA2" s="44"/>
-      <c r="DB2" s="44"/>
-      <c r="DC2" s="44">
+      <c r="DA2" s="65"/>
+      <c r="DB2" s="65"/>
+      <c r="DC2" s="65">
         <v>1.32</v>
       </c>
-      <c r="DD2" s="44"/>
-      <c r="DE2" s="44"/>
-      <c r="DF2" s="44">
+      <c r="DD2" s="65"/>
+      <c r="DE2" s="65"/>
+      <c r="DF2" s="65">
         <v>1.45</v>
       </c>
-      <c r="DG2" s="44"/>
-      <c r="DH2" s="44"/>
-    </row>
-    <row r="3" spans="1:112" s="41" customFormat="1" ht="40.799999999999997" customHeight="1">
+      <c r="DG2" s="65"/>
+      <c r="DH2" s="65"/>
+    </row>
+    <row r="3" spans="1:112" s="41" customFormat="1" ht="40.85" customHeight="1" x14ac:dyDescent="0.9">
       <c r="A3" s="40"/>
-      <c r="B3" s="44" t="s">
+      <c r="B3" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="45"/>
-      <c r="D3" s="45"/>
-      <c r="E3" s="44" t="s">
+      <c r="C3" s="66"/>
+      <c r="D3" s="66"/>
+      <c r="E3" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="F3" s="45"/>
-      <c r="G3" s="45"/>
-      <c r="H3" s="44" t="s">
+      <c r="F3" s="66"/>
+      <c r="G3" s="66"/>
+      <c r="H3" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="I3" s="45"/>
-      <c r="J3" s="45"/>
-      <c r="K3" s="44" t="s">
+      <c r="I3" s="66"/>
+      <c r="J3" s="66"/>
+      <c r="K3" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="L3" s="45"/>
-      <c r="M3" s="45"/>
-      <c r="N3" s="44" t="s">
+      <c r="L3" s="66"/>
+      <c r="M3" s="66"/>
+      <c r="N3" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="O3" s="45"/>
-      <c r="P3" s="45"/>
-      <c r="Q3" s="44" t="s">
+      <c r="O3" s="66"/>
+      <c r="P3" s="66"/>
+      <c r="Q3" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="R3" s="45"/>
-      <c r="S3" s="45"/>
-      <c r="T3" s="44" t="s">
+      <c r="R3" s="66"/>
+      <c r="S3" s="66"/>
+      <c r="T3" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="U3" s="45"/>
-      <c r="V3" s="45"/>
-      <c r="W3" s="44" t="s">
+      <c r="U3" s="66"/>
+      <c r="V3" s="66"/>
+      <c r="W3" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="X3" s="45"/>
-      <c r="Y3" s="45"/>
-      <c r="Z3" s="44" t="s">
+      <c r="X3" s="66"/>
+      <c r="Y3" s="66"/>
+      <c r="Z3" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="AA3" s="45"/>
-      <c r="AB3" s="45"/>
-      <c r="AC3" s="44" t="s">
+      <c r="AA3" s="66"/>
+      <c r="AB3" s="66"/>
+      <c r="AC3" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="AD3" s="45"/>
-      <c r="AE3" s="45"/>
-      <c r="AF3" s="44" t="s">
+      <c r="AD3" s="66"/>
+      <c r="AE3" s="66"/>
+      <c r="AF3" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="AG3" s="45"/>
-      <c r="AH3" s="45"/>
-      <c r="AI3" s="44" t="s">
+      <c r="AG3" s="66"/>
+      <c r="AH3" s="66"/>
+      <c r="AI3" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="AJ3" s="45"/>
-      <c r="AK3" s="45"/>
-      <c r="AL3" s="44" t="s">
+      <c r="AJ3" s="66"/>
+      <c r="AK3" s="66"/>
+      <c r="AL3" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="AM3" s="45"/>
-      <c r="AN3" s="45"/>
-      <c r="AO3" s="44" t="s">
+      <c r="AM3" s="66"/>
+      <c r="AN3" s="66"/>
+      <c r="AO3" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="AP3" s="45"/>
-      <c r="AQ3" s="45"/>
-      <c r="AR3" s="44" t="s">
+      <c r="AP3" s="66"/>
+      <c r="AQ3" s="66"/>
+      <c r="AR3" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="AS3" s="45"/>
-      <c r="AT3" s="45"/>
-      <c r="AU3" s="44" t="s">
+      <c r="AS3" s="66"/>
+      <c r="AT3" s="66"/>
+      <c r="AU3" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="AV3" s="45"/>
-      <c r="AW3" s="45"/>
-      <c r="AX3" s="44" t="s">
+      <c r="AV3" s="66"/>
+      <c r="AW3" s="66"/>
+      <c r="AX3" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="AY3" s="45"/>
-      <c r="AZ3" s="45"/>
-      <c r="BA3" s="44" t="s">
+      <c r="AY3" s="66"/>
+      <c r="AZ3" s="66"/>
+      <c r="BA3" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="BB3" s="45"/>
-      <c r="BC3" s="45"/>
-      <c r="BD3" s="44" t="s">
+      <c r="BB3" s="66"/>
+      <c r="BC3" s="66"/>
+      <c r="BD3" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="BE3" s="45"/>
-      <c r="BF3" s="45"/>
-      <c r="BG3" s="44" t="s">
+      <c r="BE3" s="66"/>
+      <c r="BF3" s="66"/>
+      <c r="BG3" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="BH3" s="45"/>
-      <c r="BI3" s="45"/>
-      <c r="BJ3" s="44" t="s">
+      <c r="BH3" s="66"/>
+      <c r="BI3" s="66"/>
+      <c r="BJ3" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="BK3" s="45"/>
-      <c r="BL3" s="45"/>
-      <c r="BM3" s="44" t="s">
+      <c r="BK3" s="66"/>
+      <c r="BL3" s="66"/>
+      <c r="BM3" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="BN3" s="45"/>
-      <c r="BO3" s="45"/>
-      <c r="BP3" s="44" t="s">
+      <c r="BN3" s="66"/>
+      <c r="BO3" s="66"/>
+      <c r="BP3" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="BQ3" s="45"/>
-      <c r="BR3" s="45"/>
-      <c r="BS3" s="44" t="s">
+      <c r="BQ3" s="66"/>
+      <c r="BR3" s="66"/>
+      <c r="BS3" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="BT3" s="45"/>
-      <c r="BU3" s="45"/>
-      <c r="BV3" s="44" t="s">
+      <c r="BT3" s="66"/>
+      <c r="BU3" s="66"/>
+      <c r="BV3" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="BW3" s="45"/>
-      <c r="BX3" s="45"/>
-      <c r="BY3" s="44" t="s">
+      <c r="BW3" s="66"/>
+      <c r="BX3" s="66"/>
+      <c r="BY3" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="BZ3" s="45"/>
-      <c r="CA3" s="45"/>
-      <c r="CB3" s="44" t="s">
+      <c r="BZ3" s="66"/>
+      <c r="CA3" s="66"/>
+      <c r="CB3" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="CC3" s="45"/>
-      <c r="CD3" s="45"/>
-      <c r="CE3" s="44" t="s">
+      <c r="CC3" s="66"/>
+      <c r="CD3" s="66"/>
+      <c r="CE3" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="CF3" s="45"/>
-      <c r="CG3" s="45"/>
-      <c r="CH3" s="44" t="s">
+      <c r="CF3" s="66"/>
+      <c r="CG3" s="66"/>
+      <c r="CH3" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="CI3" s="45"/>
-      <c r="CJ3" s="45"/>
-      <c r="CK3" s="44" t="s">
+      <c r="CI3" s="66"/>
+      <c r="CJ3" s="66"/>
+      <c r="CK3" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="CL3" s="45"/>
-      <c r="CM3" s="45"/>
-      <c r="CN3" s="44" t="s">
+      <c r="CL3" s="66"/>
+      <c r="CM3" s="66"/>
+      <c r="CN3" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="CO3" s="45"/>
-      <c r="CP3" s="45"/>
-      <c r="CQ3" s="44" t="s">
+      <c r="CO3" s="66"/>
+      <c r="CP3" s="66"/>
+      <c r="CQ3" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="CR3" s="45"/>
-      <c r="CS3" s="45"/>
-      <c r="CT3" s="44" t="s">
+      <c r="CR3" s="66"/>
+      <c r="CS3" s="66"/>
+      <c r="CT3" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="CU3" s="45"/>
-      <c r="CV3" s="45"/>
-      <c r="CW3" s="44" t="s">
+      <c r="CU3" s="66"/>
+      <c r="CV3" s="66"/>
+      <c r="CW3" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="CX3" s="45"/>
-      <c r="CY3" s="45"/>
-      <c r="CZ3" s="44" t="s">
+      <c r="CX3" s="66"/>
+      <c r="CY3" s="66"/>
+      <c r="CZ3" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="DA3" s="45"/>
-      <c r="DB3" s="45"/>
-      <c r="DC3" s="44" t="s">
+      <c r="DA3" s="66"/>
+      <c r="DB3" s="66"/>
+      <c r="DC3" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="DD3" s="45"/>
-      <c r="DE3" s="45"/>
-      <c r="DF3" s="44" t="s">
+      <c r="DD3" s="66"/>
+      <c r="DE3" s="66"/>
+      <c r="DF3" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="DG3" s="45"/>
-      <c r="DH3" s="45"/>
-    </row>
-    <row r="4" spans="1:112" s="27" customFormat="1" ht="40.799999999999997" customHeight="1">
+      <c r="DG3" s="66"/>
+      <c r="DH3" s="66"/>
+    </row>
+    <row r="4" spans="1:112" s="27" customFormat="1" ht="40.85" customHeight="1" x14ac:dyDescent="0.9">
       <c r="A4" s="32" t="s">
         <v>5</v>
       </c>
@@ -2283,7 +2291,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:112" s="35" customFormat="1" ht="27" customHeight="1">
+    <row r="5" spans="1:112" s="35" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.9">
       <c r="A5" s="33">
         <v>1</v>
       </c>
@@ -2700,7 +2708,7 @@
         <v>289017092.6656388</v>
       </c>
     </row>
-    <row r="6" spans="1:112">
+    <row r="6" spans="1:112" x14ac:dyDescent="0.9">
       <c r="A6" s="34">
         <v>2</v>
       </c>
@@ -3121,7 +3129,7 @@
         <v>289904014.05304569</v>
       </c>
     </row>
-    <row r="7" spans="1:112">
+    <row r="7" spans="1:112" x14ac:dyDescent="0.9">
       <c r="A7" s="34">
         <v>3</v>
       </c>
@@ -3542,7 +3550,7 @@
         <v>289957907.69702905</v>
       </c>
     </row>
-    <row r="8" spans="1:112">
+    <row r="8" spans="1:112" x14ac:dyDescent="0.9">
       <c r="A8" s="34">
         <v>4</v>
       </c>
@@ -3963,7 +3971,7 @@
         <v>290011801.34101248</v>
       </c>
     </row>
-    <row r="9" spans="1:112">
+    <row r="9" spans="1:112" x14ac:dyDescent="0.9">
       <c r="A9" s="34">
         <v>5</v>
       </c>
@@ -4384,7 +4392,7 @@
         <v>290065694.9849959</v>
       </c>
     </row>
-    <row r="10" spans="1:112">
+    <row r="10" spans="1:112" x14ac:dyDescent="0.9">
       <c r="A10" s="34">
         <v>6</v>
       </c>
@@ -4805,7 +4813,7 @@
         <v>290119588.62897927</v>
       </c>
     </row>
-    <row r="11" spans="1:112">
+    <row r="11" spans="1:112" x14ac:dyDescent="0.9">
       <c r="A11" s="34">
         <v>7</v>
       </c>
@@ -5226,7 +5234,7 @@
         <v>290173482.27296269</v>
       </c>
     </row>
-    <row r="12" spans="1:112">
+    <row r="12" spans="1:112" x14ac:dyDescent="0.9">
       <c r="A12" s="34">
         <v>8</v>
       </c>
@@ -5647,7 +5655,7 @@
         <v>290227375.91694611</v>
       </c>
     </row>
-    <row r="13" spans="1:112">
+    <row r="13" spans="1:112" x14ac:dyDescent="0.9">
       <c r="A13" s="34">
         <v>9</v>
       </c>
@@ -6068,7 +6076,7 @@
         <v>290281269.56092954</v>
       </c>
     </row>
-    <row r="14" spans="1:112">
+    <row r="14" spans="1:112" x14ac:dyDescent="0.9">
       <c r="A14" s="34">
         <v>10</v>
       </c>
@@ -6489,7 +6497,7 @@
         <v>290335163.2049129</v>
       </c>
     </row>
-    <row r="15" spans="1:112">
+    <row r="15" spans="1:112" x14ac:dyDescent="0.9">
       <c r="A15" s="34">
         <v>11</v>
       </c>
@@ -6910,7 +6918,7 @@
         <v>290389056.84889632</v>
       </c>
     </row>
-    <row r="16" spans="1:112">
+    <row r="16" spans="1:112" x14ac:dyDescent="0.9">
       <c r="A16" s="34">
         <v>12</v>
       </c>
@@ -7331,7 +7339,7 @@
         <v>290484847.68082577</v>
       </c>
     </row>
-    <row r="17" spans="1:112">
+    <row r="17" spans="1:112" x14ac:dyDescent="0.9">
       <c r="A17" s="34">
         <v>13</v>
       </c>
@@ -7752,7 +7760,7 @@
         <v>290591515.58007014</v>
       </c>
     </row>
-    <row r="18" spans="1:112">
+    <row r="18" spans="1:112" x14ac:dyDescent="0.9">
       <c r="A18" s="34">
         <v>14</v>
       </c>
@@ -8173,7 +8181,7 @@
         <v>290698183.47931457</v>
       </c>
     </row>
-    <row r="19" spans="1:112">
+    <row r="19" spans="1:112" x14ac:dyDescent="0.9">
       <c r="A19" s="34">
         <v>15</v>
       </c>
@@ -8594,7 +8602,7 @@
         <v>290804851.37855899</v>
       </c>
     </row>
-    <row r="20" spans="1:112">
+    <row r="20" spans="1:112" x14ac:dyDescent="0.9">
       <c r="A20" s="34">
         <v>16</v>
       </c>
@@ -9015,7 +9023,7 @@
         <v>290911519.27780336</v>
       </c>
     </row>
-    <row r="21" spans="1:112">
+    <row r="21" spans="1:112" x14ac:dyDescent="0.9">
       <c r="A21" s="34">
         <v>17</v>
       </c>
@@ -9436,7 +9444,7 @@
         <v>291018187.17704779</v>
       </c>
     </row>
-    <row r="22" spans="1:112">
+    <row r="22" spans="1:112" x14ac:dyDescent="0.9">
       <c r="A22" s="34">
         <v>18</v>
       </c>
@@ -9857,7 +9865,7 @@
         <v>291113105.22166628</v>
       </c>
     </row>
-    <row r="23" spans="1:112">
+    <row r="23" spans="1:112" x14ac:dyDescent="0.9">
       <c r="A23" s="34">
         <v>19</v>
       </c>
@@ -10278,7 +10286,7 @@
         <v>291231522.97553647</v>
       </c>
     </row>
-    <row r="24" spans="1:112">
+    <row r="24" spans="1:112" x14ac:dyDescent="0.9">
       <c r="A24" s="34">
         <v>20</v>
       </c>
@@ -10699,335 +10707,400 @@
         <v>291338190.87478095</v>
       </c>
     </row>
-    <row r="33" s="31" customFormat="1"/>
-    <row r="34" s="31" customFormat="1"/>
-    <row r="35" s="31" customFormat="1"/>
-    <row r="36" s="31" customFormat="1"/>
-    <row r="37" s="31" customFormat="1"/>
-    <row r="38" s="31" customFormat="1"/>
-    <row r="39" s="31" customFormat="1"/>
-    <row r="40" s="31" customFormat="1"/>
-    <row r="41" s="31" customFormat="1"/>
-    <row r="42" s="31" customFormat="1"/>
-    <row r="43" s="31" customFormat="1"/>
-    <row r="44" s="31" customFormat="1"/>
-    <row r="45" s="31" customFormat="1"/>
-    <row r="46" s="31" customFormat="1"/>
-    <row r="47" s="31" customFormat="1"/>
-    <row r="48" s="31" customFormat="1"/>
-    <row r="49" s="31" customFormat="1"/>
-    <row r="50" s="31" customFormat="1"/>
-    <row r="51" s="31" customFormat="1"/>
-    <row r="52" s="31" customFormat="1"/>
-    <row r="53" s="31" customFormat="1"/>
-    <row r="54" s="31" customFormat="1"/>
-    <row r="55" s="31" customFormat="1"/>
-    <row r="56" s="31" customFormat="1"/>
-    <row r="57" s="31" customFormat="1"/>
-    <row r="58" s="31" customFormat="1"/>
-    <row r="59" s="31" customFormat="1"/>
-    <row r="60" s="31" customFormat="1"/>
-    <row r="61" s="31" customFormat="1"/>
-    <row r="62" s="31" customFormat="1"/>
-    <row r="63" s="31" customFormat="1"/>
-    <row r="64" s="31" customFormat="1"/>
-    <row r="65" s="31" customFormat="1"/>
-    <row r="66" s="31" customFormat="1"/>
-    <row r="67" s="31" customFormat="1"/>
-    <row r="68" s="31" customFormat="1"/>
-    <row r="69" s="31" customFormat="1"/>
-    <row r="70" s="31" customFormat="1"/>
-    <row r="71" s="31" customFormat="1"/>
-    <row r="72" s="31" customFormat="1"/>
-    <row r="73" s="31" customFormat="1"/>
-    <row r="74" s="31" customFormat="1"/>
-    <row r="75" s="31" customFormat="1"/>
-    <row r="76" s="31" customFormat="1"/>
-    <row r="77" s="31" customFormat="1"/>
-    <row r="78" s="31" customFormat="1"/>
-    <row r="79" s="31" customFormat="1"/>
-    <row r="80" s="31" customFormat="1"/>
-    <row r="81" s="31" customFormat="1"/>
-    <row r="82" s="31" customFormat="1"/>
-    <row r="83" s="31" customFormat="1"/>
-    <row r="84" s="31" customFormat="1"/>
-    <row r="85" s="31" customFormat="1"/>
-    <row r="86" s="31" customFormat="1"/>
-    <row r="87" s="31" customFormat="1"/>
-    <row r="88" s="31" customFormat="1"/>
-    <row r="89" s="31" customFormat="1"/>
-    <row r="90" s="31" customFormat="1"/>
-    <row r="91" s="31" customFormat="1"/>
-    <row r="92" s="31" customFormat="1"/>
-    <row r="93" s="31" customFormat="1"/>
-    <row r="94" s="31" customFormat="1"/>
-    <row r="95" s="31" customFormat="1"/>
-    <row r="96" s="31" customFormat="1"/>
-    <row r="97" s="31" customFormat="1"/>
-    <row r="98" s="31" customFormat="1"/>
-    <row r="99" s="31" customFormat="1"/>
-    <row r="100" s="31" customFormat="1"/>
-    <row r="101" s="31" customFormat="1"/>
-    <row r="102" s="31" customFormat="1"/>
-    <row r="103" s="31" customFormat="1"/>
-    <row r="104" s="31" customFormat="1"/>
-    <row r="105" s="31" customFormat="1"/>
-    <row r="106" s="31" customFormat="1"/>
-    <row r="107" s="31" customFormat="1"/>
-    <row r="108" s="31" customFormat="1"/>
-    <row r="109" s="31" customFormat="1"/>
-    <row r="110" s="31" customFormat="1"/>
-    <row r="111" s="31" customFormat="1"/>
-    <row r="112" s="31" customFormat="1"/>
-    <row r="113" s="31" customFormat="1"/>
-    <row r="114" s="31" customFormat="1"/>
-    <row r="115" s="31" customFormat="1"/>
-    <row r="116" s="31" customFormat="1"/>
-    <row r="117" s="31" customFormat="1"/>
-    <row r="118" s="31" customFormat="1"/>
-    <row r="119" s="31" customFormat="1"/>
-    <row r="120" s="31" customFormat="1"/>
-    <row r="121" s="31" customFormat="1"/>
-    <row r="122" s="31" customFormat="1"/>
-    <row r="123" s="31" customFormat="1"/>
-    <row r="124" s="31" customFormat="1"/>
-    <row r="125" s="31" customFormat="1"/>
-    <row r="126" s="31" customFormat="1"/>
-    <row r="127" s="31" customFormat="1"/>
-    <row r="128" s="31" customFormat="1"/>
-    <row r="129" s="31" customFormat="1"/>
-    <row r="130" s="31" customFormat="1"/>
-    <row r="131" s="31" customFormat="1"/>
-    <row r="132" s="31" customFormat="1"/>
-    <row r="133" s="31" customFormat="1"/>
-    <row r="134" s="31" customFormat="1"/>
-    <row r="135" s="31" customFormat="1"/>
-    <row r="136" s="31" customFormat="1"/>
-    <row r="137" s="31" customFormat="1"/>
-    <row r="138" s="31" customFormat="1"/>
-    <row r="139" s="31" customFormat="1"/>
-    <row r="140" s="31" customFormat="1"/>
-    <row r="141" s="31" customFormat="1"/>
-    <row r="142" s="31" customFormat="1"/>
-    <row r="143" s="31" customFormat="1"/>
-    <row r="144" s="31" customFormat="1"/>
-    <row r="145" s="31" customFormat="1"/>
-    <row r="146" s="31" customFormat="1"/>
-    <row r="147" s="31" customFormat="1"/>
-    <row r="148" s="31" customFormat="1"/>
-    <row r="149" s="31" customFormat="1"/>
-    <row r="150" s="31" customFormat="1"/>
-    <row r="151" s="31" customFormat="1"/>
-    <row r="152" s="31" customFormat="1"/>
-    <row r="153" s="31" customFormat="1"/>
-    <row r="154" s="31" customFormat="1"/>
-    <row r="155" s="31" customFormat="1"/>
-    <row r="156" s="31" customFormat="1"/>
-    <row r="157" s="31" customFormat="1"/>
-    <row r="158" s="31" customFormat="1"/>
-    <row r="159" s="31" customFormat="1"/>
-    <row r="160" s="31" customFormat="1"/>
-    <row r="161" s="31" customFormat="1"/>
-    <row r="162" s="31" customFormat="1"/>
-    <row r="163" s="31" customFormat="1"/>
-    <row r="164" s="31" customFormat="1"/>
-    <row r="165" s="31" customFormat="1"/>
-    <row r="166" s="31" customFormat="1"/>
-    <row r="167" s="31" customFormat="1"/>
-    <row r="168" s="31" customFormat="1"/>
-    <row r="169" s="31" customFormat="1"/>
-    <row r="170" s="31" customFormat="1"/>
-    <row r="171" s="31" customFormat="1"/>
-    <row r="172" s="31" customFormat="1"/>
-    <row r="173" s="31" customFormat="1"/>
-    <row r="174" s="31" customFormat="1"/>
-    <row r="175" s="31" customFormat="1"/>
-    <row r="176" s="31" customFormat="1"/>
-    <row r="177" s="31" customFormat="1"/>
-    <row r="178" s="31" customFormat="1"/>
-    <row r="179" s="31" customFormat="1"/>
-    <row r="180" s="31" customFormat="1"/>
-    <row r="181" s="31" customFormat="1"/>
-    <row r="182" s="31" customFormat="1"/>
-    <row r="183" s="31" customFormat="1"/>
-    <row r="184" s="31" customFormat="1"/>
-    <row r="185" s="31" customFormat="1"/>
-    <row r="186" s="31" customFormat="1"/>
-    <row r="187" s="31" customFormat="1"/>
-    <row r="188" s="31" customFormat="1"/>
-    <row r="189" s="31" customFormat="1"/>
-    <row r="190" s="31" customFormat="1"/>
-    <row r="191" s="31" customFormat="1"/>
-    <row r="192" s="31" customFormat="1"/>
-    <row r="193" s="31" customFormat="1"/>
-    <row r="194" s="31" customFormat="1"/>
-    <row r="195" s="31" customFormat="1"/>
-    <row r="196" s="31" customFormat="1"/>
-    <row r="197" s="31" customFormat="1"/>
-    <row r="198" s="31" customFormat="1"/>
-    <row r="199" s="31" customFormat="1"/>
-    <row r="200" s="31" customFormat="1"/>
-    <row r="201" s="31" customFormat="1"/>
-    <row r="202" s="31" customFormat="1"/>
-    <row r="203" s="31" customFormat="1"/>
-    <row r="204" s="31" customFormat="1"/>
-    <row r="205" s="31" customFormat="1"/>
-    <row r="206" s="31" customFormat="1"/>
-    <row r="207" s="31" customFormat="1"/>
-    <row r="208" s="31" customFormat="1"/>
-    <row r="209" s="31" customFormat="1"/>
-    <row r="210" s="31" customFormat="1"/>
-    <row r="211" s="31" customFormat="1"/>
-    <row r="212" s="31" customFormat="1"/>
-    <row r="213" s="31" customFormat="1"/>
-    <row r="214" s="31" customFormat="1"/>
-    <row r="215" s="31" customFormat="1"/>
-    <row r="216" s="31" customFormat="1"/>
-    <row r="217" s="31" customFormat="1"/>
-    <row r="218" s="31" customFormat="1"/>
-    <row r="219" s="31" customFormat="1"/>
-    <row r="220" s="31" customFormat="1"/>
-    <row r="221" s="31" customFormat="1"/>
-    <row r="222" s="31" customFormat="1"/>
-    <row r="223" s="31" customFormat="1"/>
-    <row r="224" s="31" customFormat="1"/>
-    <row r="225" s="31" customFormat="1"/>
-    <row r="226" s="31" customFormat="1"/>
-    <row r="227" s="31" customFormat="1"/>
-    <row r="228" s="31" customFormat="1"/>
-    <row r="229" s="31" customFormat="1"/>
-    <row r="230" s="31" customFormat="1"/>
-    <row r="231" s="31" customFormat="1"/>
-    <row r="232" s="31" customFormat="1"/>
-    <row r="233" s="31" customFormat="1"/>
-    <row r="234" s="31" customFormat="1"/>
-    <row r="235" s="31" customFormat="1"/>
-    <row r="236" s="31" customFormat="1"/>
-    <row r="237" s="31" customFormat="1"/>
-    <row r="238" s="31" customFormat="1"/>
-    <row r="239" s="31" customFormat="1"/>
-    <row r="240" s="31" customFormat="1"/>
-    <row r="241" s="31" customFormat="1"/>
-    <row r="242" s="31" customFormat="1"/>
-    <row r="243" s="31" customFormat="1"/>
-    <row r="244" s="31" customFormat="1"/>
-    <row r="245" s="31" customFormat="1"/>
-    <row r="246" s="31" customFormat="1"/>
-    <row r="247" s="31" customFormat="1"/>
-    <row r="248" s="31" customFormat="1"/>
-    <row r="249" s="31" customFormat="1"/>
-    <row r="250" s="31" customFormat="1"/>
-    <row r="251" s="31" customFormat="1"/>
-    <row r="252" s="31" customFormat="1"/>
-    <row r="253" s="31" customFormat="1"/>
-    <row r="254" s="31" customFormat="1"/>
-    <row r="255" s="31" customFormat="1"/>
-    <row r="256" s="31" customFormat="1"/>
-    <row r="257" s="31" customFormat="1"/>
-    <row r="258" s="31" customFormat="1"/>
-    <row r="259" s="31" customFormat="1"/>
-    <row r="260" s="31" customFormat="1"/>
-    <row r="261" s="31" customFormat="1"/>
-    <row r="262" s="31" customFormat="1"/>
-    <row r="263" s="31" customFormat="1"/>
-    <row r="264" s="31" customFormat="1"/>
-    <row r="265" s="31" customFormat="1"/>
-    <row r="266" s="31" customFormat="1"/>
-    <row r="267" s="31" customFormat="1"/>
-    <row r="268" s="31" customFormat="1"/>
-    <row r="269" s="31" customFormat="1"/>
-    <row r="270" s="31" customFormat="1"/>
-    <row r="271" s="31" customFormat="1"/>
-    <row r="272" s="31" customFormat="1"/>
-    <row r="273" s="31" customFormat="1"/>
-    <row r="274" s="31" customFormat="1"/>
-    <row r="275" s="31" customFormat="1"/>
-    <row r="276" s="31" customFormat="1"/>
-    <row r="277" s="31" customFormat="1"/>
-    <row r="278" s="31" customFormat="1"/>
-    <row r="279" s="31" customFormat="1"/>
-    <row r="280" s="31" customFormat="1"/>
-    <row r="281" s="31" customFormat="1"/>
-    <row r="282" s="31" customFormat="1"/>
-    <row r="283" s="31" customFormat="1"/>
-    <row r="284" s="31" customFormat="1"/>
-    <row r="285" s="31" customFormat="1"/>
-    <row r="286" s="31" customFormat="1"/>
-    <row r="287" s="31" customFormat="1"/>
-    <row r="288" s="31" customFormat="1"/>
-    <row r="289" s="31" customFormat="1"/>
-    <row r="290" s="31" customFormat="1"/>
-    <row r="291" s="31" customFormat="1"/>
-    <row r="292" s="31" customFormat="1"/>
-    <row r="293" s="31" customFormat="1"/>
-    <row r="294" s="31" customFormat="1"/>
-    <row r="295" s="31" customFormat="1"/>
-    <row r="296" s="31" customFormat="1"/>
-    <row r="297" s="31" customFormat="1"/>
-    <row r="298" s="31" customFormat="1"/>
-    <row r="299" s="31" customFormat="1"/>
-    <row r="300" s="31" customFormat="1"/>
-    <row r="301" s="31" customFormat="1"/>
-    <row r="302" s="31" customFormat="1"/>
-    <row r="303" s="31" customFormat="1"/>
-    <row r="304" s="31" customFormat="1"/>
-    <row r="305" s="31" customFormat="1"/>
-    <row r="306" s="31" customFormat="1"/>
-    <row r="307" s="31" customFormat="1"/>
-    <row r="308" s="31" customFormat="1"/>
-    <row r="309" s="31" customFormat="1"/>
-    <row r="310" s="31" customFormat="1"/>
-    <row r="311" s="31" customFormat="1"/>
-    <row r="312" s="31" customFormat="1"/>
-    <row r="313" s="31" customFormat="1"/>
-    <row r="314" s="31" customFormat="1"/>
-    <row r="315" s="31" customFormat="1"/>
-    <row r="316" s="31" customFormat="1"/>
-    <row r="317" s="31" customFormat="1"/>
-    <row r="318" s="31" customFormat="1"/>
-    <row r="319" s="31" customFormat="1"/>
-    <row r="320" s="31" customFormat="1"/>
-    <row r="321" s="31" customFormat="1"/>
-    <row r="322" s="31" customFormat="1"/>
-    <row r="323" s="31" customFormat="1"/>
-    <row r="324" s="31" customFormat="1"/>
-    <row r="325" s="31" customFormat="1"/>
-    <row r="326" s="31" customFormat="1"/>
-    <row r="327" s="31" customFormat="1"/>
-    <row r="328" s="31" customFormat="1"/>
-    <row r="329" s="31" customFormat="1"/>
-    <row r="330" s="31" customFormat="1"/>
-    <row r="331" s="31" customFormat="1"/>
-    <row r="332" s="31" customFormat="1"/>
-    <row r="333" s="31" customFormat="1"/>
-    <row r="334" s="31" customFormat="1"/>
-    <row r="335" s="31" customFormat="1"/>
-    <row r="336" s="31" customFormat="1"/>
-    <row r="337" s="31" customFormat="1"/>
-    <row r="338" s="31" customFormat="1"/>
-    <row r="339" s="31" customFormat="1"/>
-    <row r="340" s="31" customFormat="1"/>
-    <row r="341" s="31" customFormat="1"/>
-    <row r="342" s="31" customFormat="1"/>
-    <row r="343" s="31" customFormat="1"/>
-    <row r="344" s="31" customFormat="1"/>
-    <row r="345" s="31" customFormat="1"/>
-    <row r="346" s="31" customFormat="1"/>
-    <row r="347" s="31" customFormat="1"/>
-    <row r="348" s="31" customFormat="1"/>
+    <row r="33" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="34" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="35" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="36" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="37" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="38" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="39" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="40" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="41" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="42" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="43" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="44" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="45" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="46" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="47" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="48" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="49" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="50" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="51" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="52" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="53" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="54" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="55" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="56" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="57" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="58" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="59" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="60" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="61" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="62" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="63" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="64" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="65" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="66" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="67" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="68" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="69" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="70" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="71" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="72" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="73" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="74" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="75" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="76" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="77" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="78" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="79" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="80" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="81" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="82" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="83" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="84" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="85" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="86" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="87" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="88" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="89" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="90" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="91" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="92" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="93" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="94" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="95" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="96" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="97" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="98" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="99" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="100" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="101" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="102" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="103" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="104" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="105" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="106" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="107" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="108" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="109" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="110" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="111" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="112" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="113" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="114" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="115" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="116" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="117" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="118" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="119" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="120" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="121" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="122" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="123" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="124" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="125" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="126" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="127" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="128" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="129" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="130" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="131" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="132" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="133" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="134" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="135" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="136" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="137" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="138" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="139" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="140" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="141" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="142" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="143" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="144" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="145" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="146" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="147" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="148" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="149" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="150" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="151" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="152" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="153" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="154" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="155" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="156" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="157" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="158" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="159" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="160" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="161" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="162" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="163" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="164" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="165" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="166" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="167" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="168" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="169" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="170" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="171" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="172" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="173" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="174" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="175" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="176" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="177" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="178" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="179" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="180" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="181" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="182" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="183" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="184" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="185" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="186" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="187" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="188" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="189" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="190" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="191" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="192" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="193" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="194" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="195" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="196" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="197" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="198" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="199" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="200" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="201" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="202" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="203" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="204" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="205" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="206" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="207" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="208" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="209" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="210" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="211" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="212" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="213" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="214" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="215" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="216" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="217" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="218" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="219" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="220" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="221" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="222" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="223" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="224" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="225" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="226" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="227" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="228" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="229" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="230" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="231" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="232" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="233" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="234" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="235" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="236" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="237" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="238" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="239" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="240" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="241" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="242" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="243" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="244" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="245" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="246" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="247" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="248" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="249" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="250" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="251" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="252" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="253" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="254" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="255" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="256" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="257" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="258" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="259" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="260" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="261" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="262" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="263" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="264" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="265" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="266" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="267" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="268" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="269" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="270" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="271" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="272" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="273" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="274" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="275" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="276" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="277" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="278" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="279" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="280" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="281" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="282" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="283" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="284" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="285" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="286" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="287" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="288" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="289" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="290" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="291" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="292" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="293" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="294" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="295" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="296" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="297" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="298" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="299" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="300" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="301" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="302" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="303" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="304" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="305" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="306" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="307" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="308" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="309" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="310" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="311" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="312" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="313" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="314" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="315" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="316" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="317" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="318" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="319" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="320" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="321" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="322" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="323" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="324" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="325" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="326" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="327" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="328" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="329" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="330" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="331" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="332" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="333" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="334" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="335" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="336" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="337" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="338" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="339" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="340" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="341" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="342" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="343" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="344" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="345" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="346" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="347" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="348" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
   </sheetData>
   <mergeCells count="111">
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="E3:G3"/>
-    <mergeCell ref="Z3:AB3"/>
-    <mergeCell ref="AC3:AE3"/>
-    <mergeCell ref="AF3:AH3"/>
-    <mergeCell ref="H3:J3"/>
-    <mergeCell ref="K3:M3"/>
-    <mergeCell ref="N3:P3"/>
-    <mergeCell ref="Q3:S3"/>
-    <mergeCell ref="T3:V3"/>
-    <mergeCell ref="W3:Y3"/>
+    <mergeCell ref="DF1:DH1"/>
+    <mergeCell ref="DF2:DH2"/>
+    <mergeCell ref="BY3:CA3"/>
+    <mergeCell ref="AI1:AK1"/>
+    <mergeCell ref="AL1:AN1"/>
+    <mergeCell ref="CN1:CP1"/>
+    <mergeCell ref="CQ1:CS1"/>
+    <mergeCell ref="AO1:AQ1"/>
+    <mergeCell ref="AR1:AT1"/>
+    <mergeCell ref="DC3:DE3"/>
+    <mergeCell ref="CZ1:DB1"/>
+    <mergeCell ref="DC1:DE1"/>
+    <mergeCell ref="CW1:CY1"/>
+    <mergeCell ref="CT2:CV2"/>
+    <mergeCell ref="CT1:CV1"/>
+    <mergeCell ref="CW2:CY2"/>
+    <mergeCell ref="CE1:CG1"/>
+    <mergeCell ref="CH1:CJ1"/>
+    <mergeCell ref="CK1:CM1"/>
+    <mergeCell ref="CT3:CV3"/>
+    <mergeCell ref="CW3:CY3"/>
+    <mergeCell ref="CZ3:DB3"/>
+    <mergeCell ref="CN3:CP3"/>
+    <mergeCell ref="BS3:BU3"/>
+    <mergeCell ref="DF3:DH3"/>
+    <mergeCell ref="BS2:BU2"/>
+    <mergeCell ref="BV2:BX2"/>
+    <mergeCell ref="BY2:CA2"/>
+    <mergeCell ref="CB2:CD2"/>
+    <mergeCell ref="CE2:CG2"/>
+    <mergeCell ref="CH2:CJ2"/>
+    <mergeCell ref="CK2:CM2"/>
+    <mergeCell ref="CN2:CP2"/>
+    <mergeCell ref="CQ2:CS2"/>
+    <mergeCell ref="CZ2:DB2"/>
+    <mergeCell ref="DC2:DE2"/>
+    <mergeCell ref="CE3:CG3"/>
+    <mergeCell ref="CH3:CJ3"/>
+    <mergeCell ref="CK3:CM3"/>
+    <mergeCell ref="CQ3:CS3"/>
+    <mergeCell ref="CB3:CD3"/>
+    <mergeCell ref="BV1:BX1"/>
+    <mergeCell ref="AU1:AW1"/>
+    <mergeCell ref="AX1:AZ1"/>
+    <mergeCell ref="BA1:BC1"/>
+    <mergeCell ref="BD1:BF1"/>
+    <mergeCell ref="BG1:BI1"/>
+    <mergeCell ref="BJ1:BL1"/>
+    <mergeCell ref="AU3:AW3"/>
+    <mergeCell ref="AX3:AZ3"/>
+    <mergeCell ref="BA3:BC3"/>
+    <mergeCell ref="BD3:BF3"/>
+    <mergeCell ref="BY1:CA1"/>
+    <mergeCell ref="Q2:S2"/>
+    <mergeCell ref="N1:P1"/>
+    <mergeCell ref="Q1:S1"/>
+    <mergeCell ref="T1:V1"/>
+    <mergeCell ref="T2:V2"/>
+    <mergeCell ref="BP1:BR1"/>
+    <mergeCell ref="BP2:BR2"/>
+    <mergeCell ref="BP3:BR3"/>
+    <mergeCell ref="BG3:BI3"/>
+    <mergeCell ref="BJ3:BL3"/>
+    <mergeCell ref="BM3:BO3"/>
+    <mergeCell ref="AI3:AK3"/>
+    <mergeCell ref="AL3:AN3"/>
+    <mergeCell ref="AO3:AQ3"/>
+    <mergeCell ref="AR3:AT3"/>
+    <mergeCell ref="BM1:BO1"/>
+    <mergeCell ref="BJ2:BL2"/>
+    <mergeCell ref="BM2:BO2"/>
+    <mergeCell ref="AX2:AZ2"/>
+    <mergeCell ref="BA2:BC2"/>
+    <mergeCell ref="BD2:BF2"/>
+    <mergeCell ref="BV3:BX3"/>
+    <mergeCell ref="BS1:BU1"/>
     <mergeCell ref="CB1:CD1"/>
     <mergeCell ref="B1:D1"/>
     <mergeCell ref="E1:G1"/>
@@ -11052,82 +11125,17 @@
     <mergeCell ref="AO2:AQ2"/>
     <mergeCell ref="AR2:AT2"/>
     <mergeCell ref="AU2:AW2"/>
-    <mergeCell ref="BY1:CA1"/>
-    <mergeCell ref="Q2:S2"/>
-    <mergeCell ref="N1:P1"/>
-    <mergeCell ref="Q1:S1"/>
-    <mergeCell ref="T1:V1"/>
-    <mergeCell ref="T2:V2"/>
-    <mergeCell ref="BP1:BR1"/>
-    <mergeCell ref="BP2:BR2"/>
-    <mergeCell ref="BP3:BR3"/>
-    <mergeCell ref="BG3:BI3"/>
-    <mergeCell ref="BJ3:BL3"/>
-    <mergeCell ref="BM3:BO3"/>
-    <mergeCell ref="AI3:AK3"/>
-    <mergeCell ref="AL3:AN3"/>
-    <mergeCell ref="AO3:AQ3"/>
-    <mergeCell ref="AR3:AT3"/>
-    <mergeCell ref="BM1:BO1"/>
-    <mergeCell ref="BJ2:BL2"/>
-    <mergeCell ref="BM2:BO2"/>
-    <mergeCell ref="AX2:AZ2"/>
-    <mergeCell ref="BA2:BC2"/>
-    <mergeCell ref="BD2:BF2"/>
-    <mergeCell ref="BV3:BX3"/>
-    <mergeCell ref="BS1:BU1"/>
-    <mergeCell ref="BV1:BX1"/>
-    <mergeCell ref="AU1:AW1"/>
-    <mergeCell ref="AX1:AZ1"/>
-    <mergeCell ref="BA1:BC1"/>
-    <mergeCell ref="BD1:BF1"/>
-    <mergeCell ref="BG1:BI1"/>
-    <mergeCell ref="BJ1:BL1"/>
-    <mergeCell ref="AU3:AW3"/>
-    <mergeCell ref="AX3:AZ3"/>
-    <mergeCell ref="BA3:BC3"/>
-    <mergeCell ref="BD3:BF3"/>
-    <mergeCell ref="DF3:DH3"/>
-    <mergeCell ref="BS2:BU2"/>
-    <mergeCell ref="BV2:BX2"/>
-    <mergeCell ref="BY2:CA2"/>
-    <mergeCell ref="CB2:CD2"/>
-    <mergeCell ref="CE2:CG2"/>
-    <mergeCell ref="CH2:CJ2"/>
-    <mergeCell ref="CK2:CM2"/>
-    <mergeCell ref="CN2:CP2"/>
-    <mergeCell ref="CQ2:CS2"/>
-    <mergeCell ref="CZ2:DB2"/>
-    <mergeCell ref="DC2:DE2"/>
-    <mergeCell ref="CE3:CG3"/>
-    <mergeCell ref="CH3:CJ3"/>
-    <mergeCell ref="CK3:CM3"/>
-    <mergeCell ref="CQ3:CS3"/>
-    <mergeCell ref="CB3:CD3"/>
-    <mergeCell ref="DF1:DH1"/>
-    <mergeCell ref="DF2:DH2"/>
-    <mergeCell ref="BY3:CA3"/>
-    <mergeCell ref="AI1:AK1"/>
-    <mergeCell ref="AL1:AN1"/>
-    <mergeCell ref="CN1:CP1"/>
-    <mergeCell ref="CQ1:CS1"/>
-    <mergeCell ref="AO1:AQ1"/>
-    <mergeCell ref="AR1:AT1"/>
-    <mergeCell ref="DC3:DE3"/>
-    <mergeCell ref="CZ1:DB1"/>
-    <mergeCell ref="DC1:DE1"/>
-    <mergeCell ref="CW1:CY1"/>
-    <mergeCell ref="CT2:CV2"/>
-    <mergeCell ref="CT1:CV1"/>
-    <mergeCell ref="CW2:CY2"/>
-    <mergeCell ref="CE1:CG1"/>
-    <mergeCell ref="CH1:CJ1"/>
-    <mergeCell ref="CK1:CM1"/>
-    <mergeCell ref="CT3:CV3"/>
-    <mergeCell ref="CW3:CY3"/>
-    <mergeCell ref="CZ3:DB3"/>
-    <mergeCell ref="CN3:CP3"/>
-    <mergeCell ref="BS3:BU3"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="E3:G3"/>
+    <mergeCell ref="Z3:AB3"/>
+    <mergeCell ref="AC3:AE3"/>
+    <mergeCell ref="AF3:AH3"/>
+    <mergeCell ref="H3:J3"/>
+    <mergeCell ref="K3:M3"/>
+    <mergeCell ref="N3:P3"/>
+    <mergeCell ref="Q3:S3"/>
+    <mergeCell ref="T3:V3"/>
+    <mergeCell ref="W3:Y3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -11137,108 +11145,108 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D65A848-DDAF-4F6A-8445-D8E58599F91D}">
   <dimension ref="A1:AM197"/>
-  <sheetFormatPr defaultColWidth="12" defaultRowHeight="15" thickTop="1" thickBottom="1"/>
+  <sheetFormatPr defaultColWidth="12" defaultRowHeight="23.6" thickTop="1" thickBottom="1" x14ac:dyDescent="0.95"/>
   <cols>
-    <col min="1" max="2" width="8.15234375" style="14" customWidth="1"/>
-    <col min="3" max="3" width="6.69140625" style="14" customWidth="1"/>
-    <col min="4" max="4" width="9.23046875" style="14" customWidth="1"/>
-    <col min="5" max="5" width="12.23046875" style="14" customWidth="1"/>
+    <col min="1" max="2" width="8.1328125" style="14" customWidth="1"/>
+    <col min="3" max="3" width="6.73046875" style="14" customWidth="1"/>
+    <col min="4" max="4" width="9.19921875" style="14" customWidth="1"/>
+    <col min="5" max="5" width="12.19921875" style="14" customWidth="1"/>
     <col min="6" max="8" width="12" style="14"/>
     <col min="9" max="9" width="12" style="25"/>
     <col min="10" max="12" width="12" style="14"/>
     <col min="13" max="13" width="12" style="20"/>
     <col min="14" max="15" width="12" style="14"/>
-    <col min="16" max="18" width="20.23046875" style="14" customWidth="1"/>
-    <col min="19" max="19" width="14.69140625" style="14" customWidth="1"/>
+    <col min="16" max="18" width="20.19921875" style="14" customWidth="1"/>
+    <col min="19" max="19" width="14.6640625" style="14" customWidth="1"/>
     <col min="20" max="20" width="12" style="14"/>
-    <col min="21" max="21" width="20.23046875" style="20" customWidth="1"/>
-    <col min="22" max="22" width="18.15234375" style="14" customWidth="1"/>
-    <col min="23" max="23" width="20.23046875" style="14" customWidth="1"/>
-    <col min="24" max="24" width="19.4609375" style="26" customWidth="1"/>
-    <col min="25" max="26" width="18.3828125" style="14" customWidth="1"/>
-    <col min="27" max="27" width="26.15234375" style="14" customWidth="1"/>
+    <col min="21" max="21" width="20.19921875" style="20" customWidth="1"/>
+    <col min="22" max="22" width="18.1328125" style="14" customWidth="1"/>
+    <col min="23" max="23" width="20.19921875" style="14" customWidth="1"/>
+    <col min="24" max="24" width="19.46484375" style="26" customWidth="1"/>
+    <col min="25" max="26" width="18.3984375" style="14" customWidth="1"/>
+    <col min="27" max="27" width="26.1328125" style="14" customWidth="1"/>
     <col min="28" max="28" width="25" style="14" customWidth="1"/>
     <col min="29" max="30" width="12" style="14"/>
     <col min="31" max="39" width="12" style="15"/>
     <col min="40" max="16384" width="12" style="14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:39" s="1" customFormat="1" ht="72" customHeight="1" thickBot="1">
-      <c r="A1" s="55" t="s">
+    <row r="1" spans="1:39" s="1" customFormat="1" ht="72" customHeight="1" thickBot="1" x14ac:dyDescent="0.95">
+      <c r="A1" s="42" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="55" t="s">
+      <c r="B1" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="55" t="s">
-        <v>106</v>
-      </c>
-      <c r="D1" s="55" t="s">
+      <c r="C1" s="42" t="s">
+        <v>103</v>
+      </c>
+      <c r="D1" s="42" t="s">
         <v>9</v>
       </c>
-      <c r="E1" s="55" t="s">
-        <v>107</v>
-      </c>
-      <c r="F1" s="55" t="s">
+      <c r="E1" s="42" t="s">
+        <v>104</v>
+      </c>
+      <c r="F1" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="G1" s="55" t="s">
+      <c r="G1" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="H1" s="55" t="s">
+      <c r="H1" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="I1" s="67" t="s">
+      <c r="I1" s="46" t="s">
         <v>13</v>
       </c>
-      <c r="J1" s="55" t="s">
-        <v>111</v>
-      </c>
-      <c r="K1" s="55" t="s">
+      <c r="J1" s="42" t="s">
+        <v>14</v>
+      </c>
+      <c r="K1" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="L1" s="65" t="s">
+      <c r="L1" s="44" t="s">
         <v>16</v>
       </c>
-      <c r="M1" s="55" t="s">
+      <c r="M1" s="42" t="s">
         <v>17</v>
       </c>
-      <c r="N1" s="55" t="s">
+      <c r="N1" s="42" t="s">
         <v>18</v>
       </c>
-      <c r="O1" s="55" t="s">
+      <c r="O1" s="42" t="s">
         <v>19</v>
       </c>
-      <c r="P1" s="62" t="s">
+      <c r="P1" s="53" t="s">
         <v>20</v>
       </c>
-      <c r="Q1" s="63"/>
-      <c r="R1" s="64"/>
-      <c r="S1" s="57" t="s">
+      <c r="Q1" s="54"/>
+      <c r="R1" s="55"/>
+      <c r="S1" s="48" t="s">
         <v>21</v>
       </c>
-      <c r="T1" s="58"/>
-      <c r="U1" s="57" t="s">
+      <c r="T1" s="49"/>
+      <c r="U1" s="48" t="s">
         <v>22</v>
       </c>
-      <c r="V1" s="59"/>
-      <c r="W1" s="60" t="s">
+      <c r="V1" s="50"/>
+      <c r="W1" s="51" t="s">
         <v>23</v>
       </c>
-      <c r="X1" s="55" t="s">
+      <c r="X1" s="42" t="s">
+        <v>110</v>
+      </c>
+      <c r="Y1" s="42" t="s">
+        <v>108</v>
+      </c>
+      <c r="Z1" s="51" t="s">
+        <v>109</v>
+      </c>
+      <c r="AA1" s="42" t="s">
         <v>24</v>
       </c>
-      <c r="Y1" s="55" t="s">
+      <c r="AB1" s="42" t="s">
         <v>25</v>
-      </c>
-      <c r="Z1" s="60" t="s">
-        <v>26</v>
-      </c>
-      <c r="AA1" s="55" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="55" t="s">
-        <v>28</v>
       </c>
       <c r="AE1" s="2"/>
       <c r="AF1" s="2"/>
@@ -11250,57 +11258,57 @@
       <c r="AL1" s="2"/>
       <c r="AM1" s="2"/>
     </row>
-    <row r="2" spans="1:39" s="1" customFormat="1" ht="48" customHeight="1" thickBot="1">
-      <c r="A2" s="56"/>
-      <c r="B2" s="56"/>
-      <c r="C2" s="56"/>
-      <c r="D2" s="56"/>
-      <c r="E2" s="56"/>
-      <c r="F2" s="56"/>
-      <c r="G2" s="56"/>
-      <c r="H2" s="56"/>
-      <c r="I2" s="68" t="s">
+    <row r="2" spans="1:39" s="1" customFormat="1" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.95">
+      <c r="A2" s="43"/>
+      <c r="B2" s="43"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="43"/>
+      <c r="G2" s="43"/>
+      <c r="H2" s="43"/>
+      <c r="I2" s="47" t="s">
         <v>13</v>
       </c>
-      <c r="J2" s="56" t="s">
+      <c r="J2" s="43" t="s">
         <v>14</v>
       </c>
-      <c r="K2" s="56" t="s">
+      <c r="K2" s="43" t="s">
         <v>15</v>
       </c>
-      <c r="L2" s="66" t="s">
-        <v>29</v>
-      </c>
-      <c r="M2" s="56"/>
-      <c r="N2" s="56"/>
-      <c r="O2" s="56"/>
+      <c r="L2" s="45" t="s">
+        <v>26</v>
+      </c>
+      <c r="M2" s="43"/>
+      <c r="N2" s="43"/>
+      <c r="O2" s="43"/>
       <c r="P2" s="3" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="S2" s="4" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="T2" s="4" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="U2" s="3" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="V2" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="W2" s="61"/>
-      <c r="X2" s="56"/>
-      <c r="Y2" s="56"/>
-      <c r="Z2" s="61"/>
-      <c r="AA2" s="56"/>
-      <c r="AB2" s="56"/>
+        <v>28</v>
+      </c>
+      <c r="W2" s="52"/>
+      <c r="X2" s="43"/>
+      <c r="Y2" s="43"/>
+      <c r="Z2" s="52"/>
+      <c r="AA2" s="43"/>
+      <c r="AB2" s="43"/>
       <c r="AE2" s="2"/>
       <c r="AF2" s="2"/>
       <c r="AG2" s="2"/>
@@ -11311,7 +11319,7 @@
       <c r="AL2" s="2"/>
       <c r="AM2" s="2"/>
     </row>
-    <row r="3" spans="1:39" s="1" customFormat="1" ht="42" customHeight="1" thickBot="1">
+    <row r="3" spans="1:39" s="1" customFormat="1" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A3" s="5">
         <v>1369</v>
       </c>
@@ -11389,10 +11397,10 @@
         <v>7500</v>
       </c>
       <c r="AA3" s="11" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="AB3" s="11" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="AE3" s="2"/>
       <c r="AF3" s="2"/>
@@ -11404,7 +11412,7 @@
       <c r="AL3" s="2"/>
       <c r="AM3" s="2"/>
     </row>
-    <row r="4" spans="1:39" s="1" customFormat="1" ht="38.25" customHeight="1" thickTop="1" thickBot="1">
+    <row r="4" spans="1:39" s="1" customFormat="1" ht="38.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A4" s="5">
         <v>1370</v>
       </c>
@@ -11482,10 +11490,10 @@
         <v>12503</v>
       </c>
       <c r="AA4" s="12" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="AB4" s="13" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="AE4" s="2"/>
       <c r="AF4" s="2"/>
@@ -11497,7 +11505,7 @@
       <c r="AL4" s="2"/>
       <c r="AM4" s="2"/>
     </row>
-    <row r="5" spans="1:39" s="1" customFormat="1" ht="38.25" customHeight="1" thickTop="1" thickBot="1">
+    <row r="5" spans="1:39" s="1" customFormat="1" ht="38.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A5" s="5">
         <v>1371</v>
       </c>
@@ -11575,10 +11583,10 @@
         <v>17003</v>
       </c>
       <c r="AA5" s="12" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="AB5" s="13" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="AE5" s="2"/>
       <c r="AF5" s="2"/>
@@ -11590,7 +11598,7 @@
       <c r="AL5" s="2"/>
       <c r="AM5" s="2"/>
     </row>
-    <row r="6" spans="1:39" s="1" customFormat="1" ht="38.25" customHeight="1" thickTop="1" thickBot="1">
+    <row r="6" spans="1:39" s="1" customFormat="1" ht="38.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A6" s="5">
         <v>1372</v>
       </c>
@@ -11668,10 +11676,10 @@
         <v>22455</v>
       </c>
       <c r="AA6" s="12" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="AB6" s="13" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="AE6" s="2"/>
       <c r="AF6" s="2"/>
@@ -11683,7 +11691,7 @@
       <c r="AL6" s="2"/>
       <c r="AM6" s="2"/>
     </row>
-    <row r="7" spans="1:39" s="1" customFormat="1" ht="38.25" customHeight="1" thickTop="1" thickBot="1">
+    <row r="7" spans="1:39" s="1" customFormat="1" ht="38.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A7" s="5">
         <v>1373</v>
       </c>
@@ -11761,10 +11769,10 @@
         <v>29205</v>
       </c>
       <c r="AA7" s="12" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="AB7" s="13" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="AE7" s="2"/>
       <c r="AF7" s="2"/>
@@ -11776,7 +11784,7 @@
       <c r="AL7" s="2"/>
       <c r="AM7" s="2"/>
     </row>
-    <row r="8" spans="1:39" s="1" customFormat="1" ht="38.25" customHeight="1" thickTop="1" thickBot="1">
+    <row r="8" spans="1:39" s="1" customFormat="1" ht="38.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A8" s="5">
         <v>1374</v>
       </c>
@@ -11854,10 +11862,10 @@
         <v>39998</v>
       </c>
       <c r="AA8" s="12" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="AB8" s="13" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="AE8" s="2"/>
       <c r="AF8" s="2"/>
@@ -11869,7 +11877,7 @@
       <c r="AL8" s="2"/>
       <c r="AM8" s="2"/>
     </row>
-    <row r="9" spans="1:39" s="1" customFormat="1" ht="38.25" customHeight="1" thickTop="1" thickBot="1">
+    <row r="9" spans="1:39" s="1" customFormat="1" ht="38.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A9" s="5">
         <v>1375</v>
       </c>
@@ -11947,10 +11955,10 @@
         <v>51803</v>
       </c>
       <c r="AA9" s="12" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="AB9" s="13" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="AE9" s="2"/>
       <c r="AF9" s="2"/>
@@ -11962,7 +11970,7 @@
       <c r="AL9" s="2"/>
       <c r="AM9" s="2"/>
     </row>
-    <row r="10" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
+    <row r="10" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A10" s="5">
         <v>1376</v>
       </c>
@@ -12040,13 +12048,13 @@
         <v>63615</v>
       </c>
       <c r="AA10" s="12" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="AB10" s="13" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="11" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="11" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A11" s="5">
         <v>1377</v>
       </c>
@@ -12124,13 +12132,13 @@
         <v>75383</v>
       </c>
       <c r="AA11" s="12" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="AB11" s="13" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="12" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="12" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A12" s="5">
         <v>1378</v>
       </c>
@@ -12208,13 +12216,13 @@
         <v>90458</v>
       </c>
       <c r="AA12" s="12" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="AB12" s="13" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="13" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="13" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A13" s="5">
         <v>1379</v>
       </c>
@@ -12292,13 +12300,13 @@
         <v>114503</v>
       </c>
       <c r="AA13" s="12" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="AB13" s="13" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="14" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="14" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A14" s="5">
         <v>1380</v>
       </c>
@@ -12376,13 +12384,13 @@
         <v>141975</v>
       </c>
       <c r="AA14" s="12" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="AB14" s="13" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="15" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="15" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A15" s="5">
         <v>1381</v>
       </c>
@@ -12460,13 +12468,13 @@
         <v>174615</v>
       </c>
       <c r="AA15" s="12" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="AB15" s="13" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="16" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="16" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A16" s="5">
         <v>1382</v>
       </c>
@@ -12544,13 +12552,13 @@
         <v>213345</v>
       </c>
       <c r="AA16" s="12" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="AB16" s="13" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="17" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="17" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A17" s="5">
         <v>1383</v>
       </c>
@@ -12628,13 +12636,13 @@
         <v>266505</v>
       </c>
       <c r="AA17" s="12" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="AB17" s="13" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="18" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="18" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A18" s="5">
         <v>1384</v>
       </c>
@@ -12712,13 +12720,13 @@
         <v>306480</v>
       </c>
       <c r="AA18" s="12" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="AB18" s="13" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="19" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="19" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A19" s="5">
         <v>1385</v>
       </c>
@@ -12796,13 +12804,13 @@
         <v>375000</v>
       </c>
       <c r="AA19" s="12" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="AB19" s="13" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="20" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="20" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A20" s="5">
         <v>1386</v>
       </c>
@@ -12880,13 +12888,13 @@
         <v>457500</v>
       </c>
       <c r="AA20" s="12" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="AB20" s="13" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="21" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="21" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A21" s="5">
         <v>1387</v>
       </c>
@@ -12906,7 +12914,7 @@
         <v>78</v>
       </c>
       <c r="G21" s="7">
-        <v>2104</v>
+        <v>2111</v>
       </c>
       <c r="H21" s="7">
         <v>73200</v>
@@ -12964,13 +12972,13 @@
         <v>549000</v>
       </c>
       <c r="AA21" s="12" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="AB21" s="13" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="22" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="22" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A22" s="5">
         <v>1388</v>
       </c>
@@ -13048,13 +13056,13 @@
         <v>658800</v>
       </c>
       <c r="AA22" s="12" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="AB22" s="13" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="23" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="23" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A23" s="5">
         <v>1389</v>
       </c>
@@ -13132,13 +13140,13 @@
         <v>757500</v>
       </c>
       <c r="AA23" s="12" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="AB23" s="13" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="24" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="24" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A24" s="5">
         <v>1390</v>
       </c>
@@ -13216,13 +13224,13 @@
         <v>825750</v>
       </c>
       <c r="AA24" s="12" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="AB24" s="13" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="25" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="25" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A25" s="5">
         <v>1391</v>
       </c>
@@ -13242,7 +13250,7 @@
         <v>73</v>
       </c>
       <c r="G25" s="7">
-        <v>2140</v>
+        <v>2148</v>
       </c>
       <c r="H25" s="7">
         <v>129900</v>
@@ -13300,14 +13308,14 @@
         <v>974250</v>
       </c>
       <c r="AA25" s="12" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="AB25" s="13" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="26" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
-      <c r="A26" s="46">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="26" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
+      <c r="A26" s="56">
         <v>1392</v>
       </c>
       <c r="B26" s="6">
@@ -13384,14 +13392,14 @@
         <v>1217813</v>
       </c>
       <c r="AA26" s="12" t="s">
-        <v>78</v>
-      </c>
-      <c r="AB26" s="46" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="27" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
-      <c r="A27" s="47"/>
+        <v>75</v>
+      </c>
+      <c r="AB26" s="56" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="27" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
+      <c r="A27" s="57"/>
       <c r="B27" s="6">
         <v>8</v>
       </c>
@@ -13466,11 +13474,11 @@
         <v>1217813</v>
       </c>
       <c r="AA27" s="12" t="s">
-        <v>78</v>
-      </c>
-      <c r="AB27" s="47"/>
-    </row>
-    <row r="28" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
+        <v>75</v>
+      </c>
+      <c r="AB27" s="57"/>
+    </row>
+    <row r="28" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A28" s="5">
         <v>1393</v>
       </c>
@@ -13548,13 +13556,13 @@
         <v>1522275</v>
       </c>
       <c r="AA28" s="12" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="AB28" s="13" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="29" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="29" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A29" s="5">
         <v>1394</v>
       </c>
@@ -13632,14 +13640,14 @@
         <v>1781063</v>
       </c>
       <c r="AA29" s="12" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="AB29" s="13" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="30" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
-      <c r="A30" s="48">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="30" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
+      <c r="A30" s="58">
         <v>1395</v>
       </c>
       <c r="B30" s="6">
@@ -13716,14 +13724,14 @@
         <v>2030415</v>
       </c>
       <c r="AA30" s="12" t="s">
-        <v>84</v>
-      </c>
-      <c r="AB30" s="50" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="31" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
-      <c r="A31" s="49"/>
+        <v>81</v>
+      </c>
+      <c r="AB30" s="60" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="31" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
+      <c r="A31" s="59"/>
       <c r="B31" s="6">
         <v>6</v>
       </c>
@@ -13798,11 +13806,11 @@
         <v>2030415</v>
       </c>
       <c r="AA31" s="12" t="s">
-        <v>84</v>
-      </c>
-      <c r="AB31" s="51"/>
-    </row>
-    <row r="32" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
+        <v>81</v>
+      </c>
+      <c r="AB31" s="61"/>
+    </row>
+    <row r="32" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A32" s="5">
         <v>1396</v>
       </c>
@@ -13880,13 +13888,13 @@
         <v>2324828</v>
       </c>
       <c r="AA32" s="12" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="AB32" s="13" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="33" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="33" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A33" s="5">
         <v>1397</v>
       </c>
@@ -13964,13 +13972,13 @@
         <v>2778173</v>
       </c>
       <c r="AA33" s="12" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="AB33" s="13" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="34" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="34" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A34" s="5">
         <v>1398</v>
       </c>
@@ -14048,14 +14056,14 @@
         <v>3792203</v>
       </c>
       <c r="AA34" s="12" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AB34" s="13" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="35" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
-      <c r="A35" s="52">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="35" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
+      <c r="A35" s="62">
         <v>1399</v>
       </c>
       <c r="B35" s="6">
@@ -14132,14 +14140,14 @@
         <v>4588568</v>
       </c>
       <c r="AA35" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="AB35" s="54" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="36" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
-      <c r="A36" s="53"/>
+        <v>89</v>
+      </c>
+      <c r="AB35" s="64" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="36" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
+      <c r="A36" s="63"/>
       <c r="B36" s="6">
         <v>9</v>
       </c>
@@ -14214,11 +14222,11 @@
         <v>4776068</v>
       </c>
       <c r="AA36" s="12" t="s">
-        <v>94</v>
-      </c>
-      <c r="AB36" s="51"/>
-    </row>
-    <row r="37" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
+        <v>91</v>
+      </c>
+      <c r="AB36" s="61"/>
+    </row>
+    <row r="37" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A37" s="5">
         <v>1400</v>
       </c>
@@ -14296,13 +14304,13 @@
         <v>6638738</v>
       </c>
       <c r="AA37" s="12" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AB37" s="13" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="38" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="38" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A38" s="5">
         <v>1401</v>
       </c>
@@ -14380,13 +14388,13 @@
         <v>10449375</v>
       </c>
       <c r="AA38" s="12" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="AB38" s="13" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="39" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="39" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A39" s="5">
         <v>1402</v>
       </c>
@@ -14464,13 +14472,13 @@
         <v>13270710</v>
       </c>
       <c r="AA39" s="12" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="AB39" s="13" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="40" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="40" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A40" s="5">
         <v>1403</v>
       </c>
@@ -14490,7 +14498,7 @@
         <v>77</v>
       </c>
       <c r="G40" s="7">
-        <v>2111</v>
+        <v>2118</v>
       </c>
       <c r="H40" s="7">
         <v>2388728</v>
@@ -14550,13 +14558,13 @@
         <v>17915460</v>
       </c>
       <c r="AA40" s="12" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="AB40" s="13" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="41" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="41" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A41" s="5">
         <v>1404</v>
       </c>
@@ -14636,13 +14644,13 @@
         <v>25977420</v>
       </c>
       <c r="AA41" s="12" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="AB41" s="13" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="42" spans="1:39" s="24" customFormat="1" ht="45.75" customHeight="1" thickTop="1" thickBot="1">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="42" spans="1:39" s="24" customFormat="1" ht="45.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A42" s="5">
         <v>1405</v>
       </c>
@@ -14722,10 +14730,10 @@
         <v>41563875</v>
       </c>
       <c r="AA42" s="12" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="AB42" s="12" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="AC42" s="22"/>
       <c r="AD42" s="22"/>
@@ -14739,7 +14747,7 @@
       <c r="AL42" s="23"/>
       <c r="AM42" s="23"/>
     </row>
-    <row r="43" spans="1:39" ht="13.8">
+    <row r="43" spans="1:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="M43" s="14"/>
       <c r="S43" s="15"/>
       <c r="T43" s="15"/>
@@ -14759,7 +14767,7 @@
       <c r="AL43" s="14"/>
       <c r="AM43" s="14"/>
     </row>
-    <row r="44" spans="1:39" ht="13.8">
+    <row r="44" spans="1:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="M44" s="14"/>
       <c r="S44" s="15"/>
       <c r="T44" s="15"/>
@@ -14779,7 +14787,7 @@
       <c r="AL44" s="14"/>
       <c r="AM44" s="14"/>
     </row>
-    <row r="45" spans="1:39" ht="13.8">
+    <row r="45" spans="1:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="M45" s="14"/>
       <c r="S45" s="15"/>
       <c r="T45" s="15"/>
@@ -14799,7 +14807,7 @@
       <c r="AL45" s="14"/>
       <c r="AM45" s="14"/>
     </row>
-    <row r="46" spans="1:39" ht="13.8">
+    <row r="46" spans="1:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="M46" s="14"/>
       <c r="S46" s="15"/>
       <c r="T46" s="15"/>
@@ -14819,7 +14827,7 @@
       <c r="AL46" s="14"/>
       <c r="AM46" s="14"/>
     </row>
-    <row r="47" spans="1:39" ht="13.8">
+    <row r="47" spans="1:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="M47" s="14"/>
       <c r="S47" s="15"/>
       <c r="T47" s="15"/>
@@ -14839,7 +14847,7 @@
       <c r="AL47" s="14"/>
       <c r="AM47" s="14"/>
     </row>
-    <row r="48" spans="1:39" ht="13.8">
+    <row r="48" spans="1:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="M48" s="14"/>
       <c r="S48" s="15"/>
       <c r="T48" s="15"/>
@@ -14859,7 +14867,7 @@
       <c r="AL48" s="14"/>
       <c r="AM48" s="14"/>
     </row>
-    <row r="49" spans="13:39" ht="13.8">
+    <row r="49" spans="13:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="M49" s="14"/>
       <c r="S49" s="15"/>
       <c r="T49" s="15"/>
@@ -14879,7 +14887,7 @@
       <c r="AL49" s="14"/>
       <c r="AM49" s="14"/>
     </row>
-    <row r="50" spans="13:39" ht="13.8">
+    <row r="50" spans="13:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="M50" s="14"/>
       <c r="S50" s="15"/>
       <c r="T50" s="15"/>
@@ -14897,7 +14905,7 @@
       <c r="AL50" s="14"/>
       <c r="AM50" s="14"/>
     </row>
-    <row r="51" spans="13:39" ht="13.8">
+    <row r="51" spans="13:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="M51" s="14"/>
       <c r="S51" s="15"/>
       <c r="T51" s="15"/>
@@ -14917,7 +14925,7 @@
       <c r="AL51" s="14"/>
       <c r="AM51" s="14"/>
     </row>
-    <row r="52" spans="13:39" ht="13.8">
+    <row r="52" spans="13:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="M52" s="14"/>
       <c r="S52" s="15"/>
       <c r="T52" s="15"/>
@@ -14937,7 +14945,7 @@
       <c r="AL52" s="14"/>
       <c r="AM52" s="14"/>
     </row>
-    <row r="53" spans="13:39" ht="13.8">
+    <row r="53" spans="13:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="M53" s="14"/>
       <c r="S53" s="15"/>
       <c r="T53" s="15"/>
@@ -14957,7 +14965,7 @@
       <c r="AL53" s="14"/>
       <c r="AM53" s="14"/>
     </row>
-    <row r="54" spans="13:39" ht="13.8">
+    <row r="54" spans="13:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="M54" s="14"/>
       <c r="S54" s="15"/>
       <c r="T54" s="15"/>
@@ -14977,7 +14985,7 @@
       <c r="AL54" s="14"/>
       <c r="AM54" s="14"/>
     </row>
-    <row r="55" spans="13:39" ht="13.8">
+    <row r="55" spans="13:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="M55" s="14"/>
       <c r="S55" s="15"/>
       <c r="T55" s="15"/>
@@ -14997,7 +15005,7 @@
       <c r="AL55" s="14"/>
       <c r="AM55" s="14"/>
     </row>
-    <row r="56" spans="13:39" ht="13.8">
+    <row r="56" spans="13:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="M56" s="14"/>
       <c r="S56" s="15"/>
       <c r="T56" s="15"/>
@@ -15017,7 +15025,7 @@
       <c r="AL56" s="14"/>
       <c r="AM56" s="14"/>
     </row>
-    <row r="57" spans="13:39" ht="13.8">
+    <row r="57" spans="13:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="M57" s="14"/>
       <c r="S57" s="15"/>
       <c r="T57" s="15"/>
@@ -15037,7 +15045,7 @@
       <c r="AL57" s="14"/>
       <c r="AM57" s="14"/>
     </row>
-    <row r="58" spans="13:39" ht="13.8">
+    <row r="58" spans="13:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="M58" s="14"/>
       <c r="S58" s="15"/>
       <c r="T58" s="15"/>
@@ -15057,7 +15065,7 @@
       <c r="AL58" s="14"/>
       <c r="AM58" s="14"/>
     </row>
-    <row r="59" spans="13:39" ht="13.8">
+    <row r="59" spans="13:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="M59" s="14"/>
       <c r="S59" s="15"/>
       <c r="T59" s="15"/>
@@ -15077,7 +15085,7 @@
       <c r="AL59" s="14"/>
       <c r="AM59" s="14"/>
     </row>
-    <row r="60" spans="13:39" ht="13.8">
+    <row r="60" spans="13:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="M60" s="14"/>
       <c r="S60" s="15"/>
       <c r="T60" s="15"/>
@@ -15097,7 +15105,7 @@
       <c r="AL60" s="14"/>
       <c r="AM60" s="14"/>
     </row>
-    <row r="61" spans="13:39" ht="13.8">
+    <row r="61" spans="13:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="M61" s="14"/>
       <c r="S61" s="15"/>
       <c r="T61" s="15"/>
@@ -15117,7 +15125,7 @@
       <c r="AL61" s="14"/>
       <c r="AM61" s="14"/>
     </row>
-    <row r="62" spans="13:39" ht="13.8">
+    <row r="62" spans="13:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S62" s="15"/>
       <c r="T62" s="15"/>
       <c r="U62" s="15"/>
@@ -15136,7 +15144,7 @@
       <c r="AL62" s="14"/>
       <c r="AM62" s="14"/>
     </row>
-    <row r="63" spans="13:39" ht="13.8">
+    <row r="63" spans="13:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S63" s="15"/>
       <c r="T63" s="15"/>
       <c r="U63" s="15"/>
@@ -15155,7 +15163,7 @@
       <c r="AL63" s="14"/>
       <c r="AM63" s="14"/>
     </row>
-    <row r="64" spans="13:39" ht="13.8">
+    <row r="64" spans="13:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S64" s="15"/>
       <c r="T64" s="15"/>
       <c r="U64" s="15"/>
@@ -15174,7 +15182,7 @@
       <c r="AL64" s="14"/>
       <c r="AM64" s="14"/>
     </row>
-    <row r="65" spans="19:39" ht="13.8">
+    <row r="65" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S65" s="15"/>
       <c r="T65" s="15"/>
       <c r="U65" s="15"/>
@@ -15193,7 +15201,7 @@
       <c r="AL65" s="14"/>
       <c r="AM65" s="14"/>
     </row>
-    <row r="66" spans="19:39" ht="13.8">
+    <row r="66" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S66" s="15"/>
       <c r="T66" s="15"/>
       <c r="U66" s="15"/>
@@ -15212,7 +15220,7 @@
       <c r="AL66" s="14"/>
       <c r="AM66" s="14"/>
     </row>
-    <row r="67" spans="19:39" ht="13.8">
+    <row r="67" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S67" s="15"/>
       <c r="T67" s="15"/>
       <c r="U67" s="15"/>
@@ -15231,7 +15239,7 @@
       <c r="AL67" s="14"/>
       <c r="AM67" s="14"/>
     </row>
-    <row r="68" spans="19:39" ht="13.8">
+    <row r="68" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S68" s="15"/>
       <c r="T68" s="15"/>
       <c r="U68" s="15"/>
@@ -15250,7 +15258,7 @@
       <c r="AL68" s="14"/>
       <c r="AM68" s="14"/>
     </row>
-    <row r="69" spans="19:39" ht="13.8">
+    <row r="69" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S69" s="15"/>
       <c r="T69" s="15"/>
       <c r="U69" s="15"/>
@@ -15269,7 +15277,7 @@
       <c r="AL69" s="14"/>
       <c r="AM69" s="14"/>
     </row>
-    <row r="70" spans="19:39" ht="13.8">
+    <row r="70" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S70" s="15"/>
       <c r="T70" s="15"/>
       <c r="U70" s="15"/>
@@ -15288,7 +15296,7 @@
       <c r="AL70" s="14"/>
       <c r="AM70" s="14"/>
     </row>
-    <row r="71" spans="19:39" ht="13.8">
+    <row r="71" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S71" s="15"/>
       <c r="T71" s="15"/>
       <c r="U71" s="15"/>
@@ -15307,7 +15315,7 @@
       <c r="AL71" s="14"/>
       <c r="AM71" s="14"/>
     </row>
-    <row r="72" spans="19:39" ht="13.8">
+    <row r="72" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S72" s="15"/>
       <c r="T72" s="15"/>
       <c r="U72" s="15"/>
@@ -15326,7 +15334,7 @@
       <c r="AL72" s="14"/>
       <c r="AM72" s="14"/>
     </row>
-    <row r="73" spans="19:39" ht="13.8">
+    <row r="73" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S73" s="15"/>
       <c r="T73" s="15"/>
       <c r="U73" s="15"/>
@@ -15345,7 +15353,7 @@
       <c r="AL73" s="14"/>
       <c r="AM73" s="14"/>
     </row>
-    <row r="74" spans="19:39" ht="13.8">
+    <row r="74" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S74" s="15"/>
       <c r="T74" s="15"/>
       <c r="U74" s="15"/>
@@ -15364,7 +15372,7 @@
       <c r="AL74" s="14"/>
       <c r="AM74" s="14"/>
     </row>
-    <row r="75" spans="19:39" ht="13.8">
+    <row r="75" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S75" s="15"/>
       <c r="T75" s="15"/>
       <c r="U75" s="15"/>
@@ -15383,7 +15391,7 @@
       <c r="AL75" s="14"/>
       <c r="AM75" s="14"/>
     </row>
-    <row r="76" spans="19:39" ht="13.8">
+    <row r="76" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S76" s="15"/>
       <c r="T76" s="15"/>
       <c r="U76" s="15"/>
@@ -15402,7 +15410,7 @@
       <c r="AL76" s="14"/>
       <c r="AM76" s="14"/>
     </row>
-    <row r="77" spans="19:39" ht="13.8">
+    <row r="77" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S77" s="15"/>
       <c r="T77" s="15"/>
       <c r="U77" s="15"/>
@@ -15421,7 +15429,7 @@
       <c r="AL77" s="14"/>
       <c r="AM77" s="14"/>
     </row>
-    <row r="78" spans="19:39" ht="13.8">
+    <row r="78" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S78" s="15"/>
       <c r="T78" s="15"/>
       <c r="U78" s="15"/>
@@ -15440,7 +15448,7 @@
       <c r="AL78" s="14"/>
       <c r="AM78" s="14"/>
     </row>
-    <row r="79" spans="19:39" ht="13.8">
+    <row r="79" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S79" s="15"/>
       <c r="T79" s="15"/>
       <c r="U79" s="15"/>
@@ -15459,7 +15467,7 @@
       <c r="AL79" s="14"/>
       <c r="AM79" s="14"/>
     </row>
-    <row r="80" spans="19:39" ht="13.8">
+    <row r="80" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S80" s="15"/>
       <c r="T80" s="15"/>
       <c r="U80" s="15"/>
@@ -15478,7 +15486,7 @@
       <c r="AL80" s="14"/>
       <c r="AM80" s="14"/>
     </row>
-    <row r="81" spans="19:39" ht="13.8">
+    <row r="81" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S81" s="15"/>
       <c r="T81" s="15"/>
       <c r="U81" s="15"/>
@@ -15497,7 +15505,7 @@
       <c r="AL81" s="14"/>
       <c r="AM81" s="14"/>
     </row>
-    <row r="82" spans="19:39" ht="13.8">
+    <row r="82" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S82" s="15"/>
       <c r="T82" s="15"/>
       <c r="U82" s="15"/>
@@ -15516,7 +15524,7 @@
       <c r="AL82" s="14"/>
       <c r="AM82" s="14"/>
     </row>
-    <row r="83" spans="19:39" ht="13.8">
+    <row r="83" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S83" s="15"/>
       <c r="T83" s="15"/>
       <c r="U83" s="15"/>
@@ -15535,7 +15543,7 @@
       <c r="AL83" s="14"/>
       <c r="AM83" s="14"/>
     </row>
-    <row r="84" spans="19:39" ht="13.8">
+    <row r="84" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S84" s="15"/>
       <c r="T84" s="15"/>
       <c r="U84" s="15"/>
@@ -15554,7 +15562,7 @@
       <c r="AL84" s="14"/>
       <c r="AM84" s="14"/>
     </row>
-    <row r="85" spans="19:39" ht="13.8">
+    <row r="85" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S85" s="15"/>
       <c r="T85" s="15"/>
       <c r="U85" s="15"/>
@@ -15573,7 +15581,7 @@
       <c r="AL85" s="14"/>
       <c r="AM85" s="14"/>
     </row>
-    <row r="86" spans="19:39" ht="13.8">
+    <row r="86" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S86" s="15"/>
       <c r="T86" s="15"/>
       <c r="U86" s="15"/>
@@ -15592,7 +15600,7 @@
       <c r="AL86" s="14"/>
       <c r="AM86" s="14"/>
     </row>
-    <row r="87" spans="19:39" ht="13.8">
+    <row r="87" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S87" s="15"/>
       <c r="T87" s="15"/>
       <c r="U87" s="15"/>
@@ -15611,7 +15619,7 @@
       <c r="AL87" s="14"/>
       <c r="AM87" s="14"/>
     </row>
-    <row r="88" spans="19:39" ht="13.8">
+    <row r="88" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S88" s="15"/>
       <c r="T88" s="15"/>
       <c r="U88" s="15"/>
@@ -15630,7 +15638,7 @@
       <c r="AL88" s="14"/>
       <c r="AM88" s="14"/>
     </row>
-    <row r="89" spans="19:39" ht="13.8">
+    <row r="89" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S89" s="15"/>
       <c r="T89" s="15"/>
       <c r="U89" s="15"/>
@@ -15649,7 +15657,7 @@
       <c r="AL89" s="14"/>
       <c r="AM89" s="14"/>
     </row>
-    <row r="90" spans="19:39" ht="13.8">
+    <row r="90" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S90" s="15"/>
       <c r="T90" s="15"/>
       <c r="U90" s="15"/>
@@ -15668,7 +15676,7 @@
       <c r="AL90" s="14"/>
       <c r="AM90" s="14"/>
     </row>
-    <row r="91" spans="19:39" ht="13.8">
+    <row r="91" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S91" s="15"/>
       <c r="T91" s="15"/>
       <c r="U91" s="15"/>
@@ -15687,7 +15695,7 @@
       <c r="AL91" s="14"/>
       <c r="AM91" s="14"/>
     </row>
-    <row r="92" spans="19:39" ht="13.8">
+    <row r="92" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S92" s="15"/>
       <c r="T92" s="15"/>
       <c r="U92" s="15"/>
@@ -15706,7 +15714,7 @@
       <c r="AL92" s="14"/>
       <c r="AM92" s="14"/>
     </row>
-    <row r="93" spans="19:39" ht="13.8">
+    <row r="93" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S93" s="15"/>
       <c r="T93" s="15"/>
       <c r="U93" s="15"/>
@@ -15725,7 +15733,7 @@
       <c r="AL93" s="14"/>
       <c r="AM93" s="14"/>
     </row>
-    <row r="94" spans="19:39" ht="13.8">
+    <row r="94" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S94" s="15"/>
       <c r="T94" s="15"/>
       <c r="U94" s="15"/>
@@ -15744,7 +15752,7 @@
       <c r="AL94" s="14"/>
       <c r="AM94" s="14"/>
     </row>
-    <row r="95" spans="19:39" ht="13.8">
+    <row r="95" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S95" s="15"/>
       <c r="T95" s="15"/>
       <c r="U95" s="15"/>
@@ -15763,7 +15771,7 @@
       <c r="AL95" s="14"/>
       <c r="AM95" s="14"/>
     </row>
-    <row r="96" spans="19:39" ht="13.8">
+    <row r="96" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S96" s="15"/>
       <c r="T96" s="15"/>
       <c r="U96" s="15"/>
@@ -15782,7 +15790,7 @@
       <c r="AL96" s="14"/>
       <c r="AM96" s="14"/>
     </row>
-    <row r="97" spans="19:39" ht="13.8">
+    <row r="97" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S97" s="15"/>
       <c r="T97" s="15"/>
       <c r="U97" s="15"/>
@@ -15801,7 +15809,7 @@
       <c r="AL97" s="14"/>
       <c r="AM97" s="14"/>
     </row>
-    <row r="98" spans="19:39" ht="13.8">
+    <row r="98" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S98" s="15"/>
       <c r="T98" s="15"/>
       <c r="U98" s="15"/>
@@ -15820,7 +15828,7 @@
       <c r="AL98" s="14"/>
       <c r="AM98" s="14"/>
     </row>
-    <row r="99" spans="19:39" ht="13.8">
+    <row r="99" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S99" s="15"/>
       <c r="T99" s="15"/>
       <c r="U99" s="15"/>
@@ -15839,7 +15847,7 @@
       <c r="AL99" s="14"/>
       <c r="AM99" s="14"/>
     </row>
-    <row r="100" spans="19:39" ht="13.8">
+    <row r="100" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S100" s="15"/>
       <c r="T100" s="15"/>
       <c r="U100" s="15"/>
@@ -15858,7 +15866,7 @@
       <c r="AL100" s="14"/>
       <c r="AM100" s="14"/>
     </row>
-    <row r="101" spans="19:39" ht="13.8">
+    <row r="101" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S101" s="15"/>
       <c r="T101" s="15"/>
       <c r="U101" s="15"/>
@@ -15877,7 +15885,7 @@
       <c r="AL101" s="14"/>
       <c r="AM101" s="14"/>
     </row>
-    <row r="102" spans="19:39" ht="13.8">
+    <row r="102" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S102" s="15"/>
       <c r="T102" s="15"/>
       <c r="U102" s="15"/>
@@ -15896,7 +15904,7 @@
       <c r="AL102" s="14"/>
       <c r="AM102" s="14"/>
     </row>
-    <row r="103" spans="19:39" ht="13.8">
+    <row r="103" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S103" s="15"/>
       <c r="T103" s="15"/>
       <c r="U103" s="15"/>
@@ -15915,7 +15923,7 @@
       <c r="AL103" s="14"/>
       <c r="AM103" s="14"/>
     </row>
-    <row r="104" spans="19:39" ht="13.8">
+    <row r="104" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S104" s="15"/>
       <c r="T104" s="15"/>
       <c r="U104" s="15"/>
@@ -15934,7 +15942,7 @@
       <c r="AL104" s="14"/>
       <c r="AM104" s="14"/>
     </row>
-    <row r="105" spans="19:39" ht="13.8">
+    <row r="105" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S105" s="15"/>
       <c r="T105" s="15"/>
       <c r="U105" s="15"/>
@@ -15953,7 +15961,7 @@
       <c r="AL105" s="14"/>
       <c r="AM105" s="14"/>
     </row>
-    <row r="106" spans="19:39" ht="13.8">
+    <row r="106" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S106" s="15"/>
       <c r="T106" s="15"/>
       <c r="U106" s="15"/>
@@ -15972,7 +15980,7 @@
       <c r="AL106" s="14"/>
       <c r="AM106" s="14"/>
     </row>
-    <row r="107" spans="19:39" ht="13.8">
+    <row r="107" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S107" s="15"/>
       <c r="T107" s="15"/>
       <c r="U107" s="15"/>
@@ -15991,7 +15999,7 @@
       <c r="AL107" s="14"/>
       <c r="AM107" s="14"/>
     </row>
-    <row r="108" spans="19:39" ht="13.8">
+    <row r="108" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S108" s="15"/>
       <c r="T108" s="15"/>
       <c r="U108" s="15"/>
@@ -16010,7 +16018,7 @@
       <c r="AL108" s="14"/>
       <c r="AM108" s="14"/>
     </row>
-    <row r="109" spans="19:39" ht="13.8">
+    <row r="109" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S109" s="15"/>
       <c r="T109" s="15"/>
       <c r="U109" s="15"/>
@@ -16029,7 +16037,7 @@
       <c r="AL109" s="14"/>
       <c r="AM109" s="14"/>
     </row>
-    <row r="110" spans="19:39" ht="13.8">
+    <row r="110" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S110" s="15"/>
       <c r="T110" s="15"/>
       <c r="U110" s="15"/>
@@ -16048,7 +16056,7 @@
       <c r="AL110" s="14"/>
       <c r="AM110" s="14"/>
     </row>
-    <row r="111" spans="19:39" ht="13.8">
+    <row r="111" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S111" s="15"/>
       <c r="T111" s="15"/>
       <c r="U111" s="15"/>
@@ -16067,7 +16075,7 @@
       <c r="AL111" s="14"/>
       <c r="AM111" s="14"/>
     </row>
-    <row r="112" spans="19:39" ht="13.8">
+    <row r="112" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S112" s="15"/>
       <c r="T112" s="15"/>
       <c r="U112" s="15"/>
@@ -16086,7 +16094,7 @@
       <c r="AL112" s="14"/>
       <c r="AM112" s="14"/>
     </row>
-    <row r="113" spans="19:39" ht="13.8">
+    <row r="113" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S113" s="15"/>
       <c r="T113" s="15"/>
       <c r="U113" s="15"/>
@@ -16105,7 +16113,7 @@
       <c r="AL113" s="14"/>
       <c r="AM113" s="14"/>
     </row>
-    <row r="114" spans="19:39" ht="13.8">
+    <row r="114" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S114" s="15"/>
       <c r="T114" s="15"/>
       <c r="U114" s="15"/>
@@ -16124,7 +16132,7 @@
       <c r="AL114" s="14"/>
       <c r="AM114" s="14"/>
     </row>
-    <row r="115" spans="19:39" ht="13.8">
+    <row r="115" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S115" s="15"/>
       <c r="T115" s="15"/>
       <c r="U115" s="15"/>
@@ -16143,7 +16151,7 @@
       <c r="AL115" s="14"/>
       <c r="AM115" s="14"/>
     </row>
-    <row r="116" spans="19:39" ht="13.8">
+    <row r="116" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S116" s="15"/>
       <c r="T116" s="15"/>
       <c r="U116" s="15"/>
@@ -16162,7 +16170,7 @@
       <c r="AL116" s="14"/>
       <c r="AM116" s="14"/>
     </row>
-    <row r="117" spans="19:39" ht="13.8">
+    <row r="117" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S117" s="15"/>
       <c r="T117" s="15"/>
       <c r="U117" s="15"/>
@@ -16181,7 +16189,7 @@
       <c r="AL117" s="14"/>
       <c r="AM117" s="14"/>
     </row>
-    <row r="118" spans="19:39" ht="13.8">
+    <row r="118" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S118" s="15"/>
       <c r="T118" s="15"/>
       <c r="U118" s="15"/>
@@ -16200,7 +16208,7 @@
       <c r="AL118" s="14"/>
       <c r="AM118" s="14"/>
     </row>
-    <row r="119" spans="19:39" ht="13.8">
+    <row r="119" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S119" s="15"/>
       <c r="T119" s="15"/>
       <c r="U119" s="15"/>
@@ -16219,7 +16227,7 @@
       <c r="AL119" s="14"/>
       <c r="AM119" s="14"/>
     </row>
-    <row r="120" spans="19:39" ht="13.8">
+    <row r="120" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S120" s="15"/>
       <c r="T120" s="15"/>
       <c r="U120" s="15"/>
@@ -16238,7 +16246,7 @@
       <c r="AL120" s="14"/>
       <c r="AM120" s="14"/>
     </row>
-    <row r="121" spans="19:39" ht="13.8">
+    <row r="121" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S121" s="15"/>
       <c r="T121" s="15"/>
       <c r="U121" s="15"/>
@@ -16257,7 +16265,7 @@
       <c r="AL121" s="14"/>
       <c r="AM121" s="14"/>
     </row>
-    <row r="122" spans="19:39" ht="13.8">
+    <row r="122" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S122" s="15"/>
       <c r="T122" s="15"/>
       <c r="U122" s="15"/>
@@ -16276,7 +16284,7 @@
       <c r="AL122" s="14"/>
       <c r="AM122" s="14"/>
     </row>
-    <row r="123" spans="19:39" ht="13.8">
+    <row r="123" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S123" s="15"/>
       <c r="T123" s="15"/>
       <c r="U123" s="15"/>
@@ -16295,7 +16303,7 @@
       <c r="AL123" s="14"/>
       <c r="AM123" s="14"/>
     </row>
-    <row r="124" spans="19:39" ht="13.8">
+    <row r="124" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S124" s="15"/>
       <c r="T124" s="15"/>
       <c r="U124" s="15"/>
@@ -16314,7 +16322,7 @@
       <c r="AL124" s="14"/>
       <c r="AM124" s="14"/>
     </row>
-    <row r="125" spans="19:39" ht="13.8">
+    <row r="125" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S125" s="15"/>
       <c r="T125" s="15"/>
       <c r="U125" s="15"/>
@@ -16333,7 +16341,7 @@
       <c r="AL125" s="14"/>
       <c r="AM125" s="14"/>
     </row>
-    <row r="126" spans="19:39" ht="13.8">
+    <row r="126" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S126" s="15"/>
       <c r="T126" s="15"/>
       <c r="U126" s="15"/>
@@ -16352,7 +16360,7 @@
       <c r="AL126" s="14"/>
       <c r="AM126" s="14"/>
     </row>
-    <row r="127" spans="19:39" ht="13.8">
+    <row r="127" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S127" s="15"/>
       <c r="T127" s="15"/>
       <c r="U127" s="15"/>
@@ -16371,7 +16379,7 @@
       <c r="AL127" s="14"/>
       <c r="AM127" s="14"/>
     </row>
-    <row r="128" spans="19:39" ht="13.8">
+    <row r="128" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S128" s="15"/>
       <c r="T128" s="15"/>
       <c r="U128" s="15"/>
@@ -16390,7 +16398,7 @@
       <c r="AL128" s="14"/>
       <c r="AM128" s="14"/>
     </row>
-    <row r="129" spans="19:39" ht="13.8">
+    <row r="129" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S129" s="15"/>
       <c r="T129" s="15"/>
       <c r="U129" s="15"/>
@@ -16409,7 +16417,7 @@
       <c r="AL129" s="14"/>
       <c r="AM129" s="14"/>
     </row>
-    <row r="130" spans="19:39" ht="13.8">
+    <row r="130" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S130" s="15"/>
       <c r="T130" s="15"/>
       <c r="U130" s="15"/>
@@ -16428,7 +16436,7 @@
       <c r="AL130" s="14"/>
       <c r="AM130" s="14"/>
     </row>
-    <row r="131" spans="19:39" ht="13.8">
+    <row r="131" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S131" s="15"/>
       <c r="T131" s="15"/>
       <c r="U131" s="15"/>
@@ -16447,7 +16455,7 @@
       <c r="AL131" s="14"/>
       <c r="AM131" s="14"/>
     </row>
-    <row r="132" spans="19:39" ht="13.8">
+    <row r="132" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S132" s="15"/>
       <c r="T132" s="15"/>
       <c r="U132" s="15"/>
@@ -16466,7 +16474,7 @@
       <c r="AL132" s="14"/>
       <c r="AM132" s="14"/>
     </row>
-    <row r="133" spans="19:39" ht="13.8">
+    <row r="133" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S133" s="15"/>
       <c r="T133" s="15"/>
       <c r="U133" s="15"/>
@@ -16485,7 +16493,7 @@
       <c r="AL133" s="14"/>
       <c r="AM133" s="14"/>
     </row>
-    <row r="134" spans="19:39" ht="13.8">
+    <row r="134" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S134" s="15"/>
       <c r="T134" s="15"/>
       <c r="U134" s="15"/>
@@ -16504,7 +16512,7 @@
       <c r="AL134" s="14"/>
       <c r="AM134" s="14"/>
     </row>
-    <row r="135" spans="19:39" ht="13.8">
+    <row r="135" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S135" s="15"/>
       <c r="T135" s="15"/>
       <c r="U135" s="15"/>
@@ -16523,7 +16531,7 @@
       <c r="AL135" s="14"/>
       <c r="AM135" s="14"/>
     </row>
-    <row r="136" spans="19:39" ht="13.8">
+    <row r="136" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S136" s="15"/>
       <c r="T136" s="15"/>
       <c r="U136" s="15"/>
@@ -16542,7 +16550,7 @@
       <c r="AL136" s="14"/>
       <c r="AM136" s="14"/>
     </row>
-    <row r="137" spans="19:39" ht="13.8">
+    <row r="137" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S137" s="15"/>
       <c r="T137" s="15"/>
       <c r="U137" s="15"/>
@@ -16561,7 +16569,7 @@
       <c r="AL137" s="14"/>
       <c r="AM137" s="14"/>
     </row>
-    <row r="138" spans="19:39" ht="13.8">
+    <row r="138" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S138" s="15"/>
       <c r="T138" s="15"/>
       <c r="U138" s="15"/>
@@ -16580,7 +16588,7 @@
       <c r="AL138" s="14"/>
       <c r="AM138" s="14"/>
     </row>
-    <row r="139" spans="19:39" ht="13.8">
+    <row r="139" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S139" s="15"/>
       <c r="T139" s="15"/>
       <c r="U139" s="15"/>
@@ -16599,7 +16607,7 @@
       <c r="AL139" s="14"/>
       <c r="AM139" s="14"/>
     </row>
-    <row r="140" spans="19:39" ht="13.8">
+    <row r="140" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S140" s="15"/>
       <c r="T140" s="15"/>
       <c r="U140" s="15"/>
@@ -16618,7 +16626,7 @@
       <c r="AL140" s="14"/>
       <c r="AM140" s="14"/>
     </row>
-    <row r="141" spans="19:39" ht="13.8">
+    <row r="141" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S141" s="15"/>
       <c r="T141" s="15"/>
       <c r="U141" s="15"/>
@@ -16637,7 +16645,7 @@
       <c r="AL141" s="14"/>
       <c r="AM141" s="14"/>
     </row>
-    <row r="142" spans="19:39" ht="13.8">
+    <row r="142" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S142" s="15"/>
       <c r="T142" s="15"/>
       <c r="U142" s="15"/>
@@ -16656,7 +16664,7 @@
       <c r="AL142" s="14"/>
       <c r="AM142" s="14"/>
     </row>
-    <row r="143" spans="19:39" ht="13.8">
+    <row r="143" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S143" s="15"/>
       <c r="T143" s="15"/>
       <c r="U143" s="15"/>
@@ -16675,7 +16683,7 @@
       <c r="AL143" s="14"/>
       <c r="AM143" s="14"/>
     </row>
-    <row r="144" spans="19:39" ht="13.8">
+    <row r="144" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S144" s="15"/>
       <c r="T144" s="15"/>
       <c r="U144" s="15"/>
@@ -16694,7 +16702,7 @@
       <c r="AL144" s="14"/>
       <c r="AM144" s="14"/>
     </row>
-    <row r="145" spans="19:39" ht="13.8">
+    <row r="145" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S145" s="15"/>
       <c r="T145" s="15"/>
       <c r="U145" s="15"/>
@@ -16713,7 +16721,7 @@
       <c r="AL145" s="14"/>
       <c r="AM145" s="14"/>
     </row>
-    <row r="146" spans="19:39" ht="13.8">
+    <row r="146" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S146" s="15"/>
       <c r="T146" s="15"/>
       <c r="U146" s="15"/>
@@ -16732,7 +16740,7 @@
       <c r="AL146" s="14"/>
       <c r="AM146" s="14"/>
     </row>
-    <row r="147" spans="19:39" ht="13.8">
+    <row r="147" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S147" s="15"/>
       <c r="T147" s="15"/>
       <c r="U147" s="15"/>
@@ -16751,7 +16759,7 @@
       <c r="AL147" s="14"/>
       <c r="AM147" s="14"/>
     </row>
-    <row r="148" spans="19:39" ht="13.8">
+    <row r="148" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S148" s="15"/>
       <c r="T148" s="15"/>
       <c r="U148" s="15"/>
@@ -16770,7 +16778,7 @@
       <c r="AL148" s="14"/>
       <c r="AM148" s="14"/>
     </row>
-    <row r="149" spans="19:39" ht="13.8">
+    <row r="149" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S149" s="15"/>
       <c r="T149" s="15"/>
       <c r="U149" s="15"/>
@@ -16789,7 +16797,7 @@
       <c r="AL149" s="14"/>
       <c r="AM149" s="14"/>
     </row>
-    <row r="150" spans="19:39" ht="13.8">
+    <row r="150" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S150" s="15"/>
       <c r="T150" s="15"/>
       <c r="U150" s="15"/>
@@ -16808,7 +16816,7 @@
       <c r="AL150" s="14"/>
       <c r="AM150" s="14"/>
     </row>
-    <row r="151" spans="19:39" ht="13.8">
+    <row r="151" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S151" s="15"/>
       <c r="T151" s="15"/>
       <c r="U151" s="15"/>
@@ -16827,7 +16835,7 @@
       <c r="AL151" s="14"/>
       <c r="AM151" s="14"/>
     </row>
-    <row r="152" spans="19:39" ht="13.8">
+    <row r="152" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S152" s="15"/>
       <c r="T152" s="15"/>
       <c r="U152" s="15"/>
@@ -16846,7 +16854,7 @@
       <c r="AL152" s="14"/>
       <c r="AM152" s="14"/>
     </row>
-    <row r="153" spans="19:39" ht="13.8">
+    <row r="153" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S153" s="15"/>
       <c r="T153" s="15"/>
       <c r="U153" s="15"/>
@@ -16865,7 +16873,7 @@
       <c r="AL153" s="14"/>
       <c r="AM153" s="14"/>
     </row>
-    <row r="154" spans="19:39" ht="13.8">
+    <row r="154" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S154" s="15"/>
       <c r="T154" s="15"/>
       <c r="U154" s="15"/>
@@ -16884,7 +16892,7 @@
       <c r="AL154" s="14"/>
       <c r="AM154" s="14"/>
     </row>
-    <row r="155" spans="19:39" ht="13.8">
+    <row r="155" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S155" s="15"/>
       <c r="T155" s="15"/>
       <c r="U155" s="15"/>
@@ -16903,7 +16911,7 @@
       <c r="AL155" s="14"/>
       <c r="AM155" s="14"/>
     </row>
-    <row r="156" spans="19:39" ht="13.8">
+    <row r="156" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S156" s="15"/>
       <c r="T156" s="15"/>
       <c r="U156" s="15"/>
@@ -16922,7 +16930,7 @@
       <c r="AL156" s="14"/>
       <c r="AM156" s="14"/>
     </row>
-    <row r="157" spans="19:39" ht="13.8">
+    <row r="157" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S157" s="15"/>
       <c r="T157" s="15"/>
       <c r="U157" s="15"/>
@@ -16941,7 +16949,7 @@
       <c r="AL157" s="14"/>
       <c r="AM157" s="14"/>
     </row>
-    <row r="158" spans="19:39" ht="13.8">
+    <row r="158" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S158" s="15"/>
       <c r="T158" s="15"/>
       <c r="U158" s="15"/>
@@ -16960,7 +16968,7 @@
       <c r="AL158" s="14"/>
       <c r="AM158" s="14"/>
     </row>
-    <row r="159" spans="19:39" ht="13.8">
+    <row r="159" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S159" s="15"/>
       <c r="T159" s="15"/>
       <c r="U159" s="15"/>
@@ -16979,7 +16987,7 @@
       <c r="AL159" s="14"/>
       <c r="AM159" s="14"/>
     </row>
-    <row r="160" spans="19:39" ht="13.8">
+    <row r="160" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S160" s="15"/>
       <c r="T160" s="15"/>
       <c r="U160" s="15"/>
@@ -16998,7 +17006,7 @@
       <c r="AL160" s="14"/>
       <c r="AM160" s="14"/>
     </row>
-    <row r="161" spans="19:39" ht="13.8">
+    <row r="161" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S161" s="15"/>
       <c r="T161" s="15"/>
       <c r="U161" s="15"/>
@@ -17017,7 +17025,7 @@
       <c r="AL161" s="14"/>
       <c r="AM161" s="14"/>
     </row>
-    <row r="162" spans="19:39" ht="13.8">
+    <row r="162" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S162" s="15"/>
       <c r="T162" s="15"/>
       <c r="U162" s="15"/>
@@ -17036,7 +17044,7 @@
       <c r="AL162" s="14"/>
       <c r="AM162" s="14"/>
     </row>
-    <row r="163" spans="19:39" ht="13.8">
+    <row r="163" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S163" s="15"/>
       <c r="T163" s="15"/>
       <c r="U163" s="15"/>
@@ -17055,7 +17063,7 @@
       <c r="AL163" s="14"/>
       <c r="AM163" s="14"/>
     </row>
-    <row r="164" spans="19:39" ht="13.8">
+    <row r="164" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S164" s="15"/>
       <c r="T164" s="15"/>
       <c r="U164" s="15"/>
@@ -17074,7 +17082,7 @@
       <c r="AL164" s="14"/>
       <c r="AM164" s="14"/>
     </row>
-    <row r="165" spans="19:39" ht="13.8">
+    <row r="165" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S165" s="15"/>
       <c r="T165" s="15"/>
       <c r="U165" s="15"/>
@@ -17093,7 +17101,7 @@
       <c r="AL165" s="14"/>
       <c r="AM165" s="14"/>
     </row>
-    <row r="166" spans="19:39" ht="13.8">
+    <row r="166" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S166" s="15"/>
       <c r="T166" s="15"/>
       <c r="U166" s="15"/>
@@ -17112,7 +17120,7 @@
       <c r="AL166" s="14"/>
       <c r="AM166" s="14"/>
     </row>
-    <row r="167" spans="19:39" ht="13.8">
+    <row r="167" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S167" s="15"/>
       <c r="T167" s="15"/>
       <c r="U167" s="15"/>
@@ -17131,7 +17139,7 @@
       <c r="AL167" s="14"/>
       <c r="AM167" s="14"/>
     </row>
-    <row r="168" spans="19:39" ht="13.8">
+    <row r="168" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S168" s="15"/>
       <c r="T168" s="15"/>
       <c r="U168" s="15"/>
@@ -17150,7 +17158,7 @@
       <c r="AL168" s="14"/>
       <c r="AM168" s="14"/>
     </row>
-    <row r="169" spans="19:39" ht="13.8">
+    <row r="169" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S169" s="15"/>
       <c r="T169" s="15"/>
       <c r="U169" s="15"/>
@@ -17169,7 +17177,7 @@
       <c r="AL169" s="14"/>
       <c r="AM169" s="14"/>
     </row>
-    <row r="170" spans="19:39" ht="13.8">
+    <row r="170" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S170" s="15"/>
       <c r="T170" s="15"/>
       <c r="U170" s="15"/>
@@ -17188,7 +17196,7 @@
       <c r="AL170" s="14"/>
       <c r="AM170" s="14"/>
     </row>
-    <row r="171" spans="19:39" ht="13.8">
+    <row r="171" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S171" s="15"/>
       <c r="T171" s="15"/>
       <c r="U171" s="15"/>
@@ -17207,7 +17215,7 @@
       <c r="AL171" s="14"/>
       <c r="AM171" s="14"/>
     </row>
-    <row r="172" spans="19:39" ht="13.8">
+    <row r="172" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S172" s="15"/>
       <c r="T172" s="15"/>
       <c r="U172" s="15"/>
@@ -17226,7 +17234,7 @@
       <c r="AL172" s="14"/>
       <c r="AM172" s="14"/>
     </row>
-    <row r="173" spans="19:39" ht="13.8">
+    <row r="173" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S173" s="15"/>
       <c r="T173" s="15"/>
       <c r="U173" s="15"/>
@@ -17245,7 +17253,7 @@
       <c r="AL173" s="14"/>
       <c r="AM173" s="14"/>
     </row>
-    <row r="174" spans="19:39" ht="13.8">
+    <row r="174" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S174" s="15"/>
       <c r="T174" s="15"/>
       <c r="U174" s="15"/>
@@ -17264,7 +17272,7 @@
       <c r="AL174" s="14"/>
       <c r="AM174" s="14"/>
     </row>
-    <row r="175" spans="19:39" ht="13.8">
+    <row r="175" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S175" s="15"/>
       <c r="T175" s="15"/>
       <c r="U175" s="15"/>
@@ -17283,7 +17291,7 @@
       <c r="AL175" s="14"/>
       <c r="AM175" s="14"/>
     </row>
-    <row r="176" spans="19:39" ht="13.8">
+    <row r="176" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S176" s="15"/>
       <c r="T176" s="15"/>
       <c r="U176" s="15"/>
@@ -17302,7 +17310,7 @@
       <c r="AL176" s="14"/>
       <c r="AM176" s="14"/>
     </row>
-    <row r="177" spans="19:39" ht="13.8">
+    <row r="177" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S177" s="15"/>
       <c r="T177" s="15"/>
       <c r="U177" s="15"/>
@@ -17321,7 +17329,7 @@
       <c r="AL177" s="14"/>
       <c r="AM177" s="14"/>
     </row>
-    <row r="178" spans="19:39" ht="13.8">
+    <row r="178" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S178" s="15"/>
       <c r="T178" s="15"/>
       <c r="U178" s="15"/>
@@ -17340,7 +17348,7 @@
       <c r="AL178" s="14"/>
       <c r="AM178" s="14"/>
     </row>
-    <row r="179" spans="19:39" ht="13.8">
+    <row r="179" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S179" s="15"/>
       <c r="T179" s="15"/>
       <c r="U179" s="15"/>
@@ -17359,7 +17367,7 @@
       <c r="AL179" s="14"/>
       <c r="AM179" s="14"/>
     </row>
-    <row r="180" spans="19:39" ht="13.8">
+    <row r="180" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S180" s="15"/>
       <c r="T180" s="15"/>
       <c r="U180" s="15"/>
@@ -17378,7 +17386,7 @@
       <c r="AL180" s="14"/>
       <c r="AM180" s="14"/>
     </row>
-    <row r="181" spans="19:39" ht="13.8">
+    <row r="181" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S181" s="15"/>
       <c r="T181" s="15"/>
       <c r="U181" s="15"/>
@@ -17397,7 +17405,7 @@
       <c r="AL181" s="14"/>
       <c r="AM181" s="14"/>
     </row>
-    <row r="182" spans="19:39" ht="13.8">
+    <row r="182" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S182" s="15"/>
       <c r="T182" s="15"/>
       <c r="U182" s="15"/>
@@ -17416,7 +17424,7 @@
       <c r="AL182" s="14"/>
       <c r="AM182" s="14"/>
     </row>
-    <row r="183" spans="19:39" ht="13.8">
+    <row r="183" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S183" s="15"/>
       <c r="T183" s="15"/>
       <c r="U183" s="15"/>
@@ -17435,7 +17443,7 @@
       <c r="AL183" s="14"/>
       <c r="AM183" s="14"/>
     </row>
-    <row r="184" spans="19:39" ht="13.8">
+    <row r="184" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S184" s="15"/>
       <c r="T184" s="15"/>
       <c r="U184" s="15"/>
@@ -17454,7 +17462,7 @@
       <c r="AL184" s="14"/>
       <c r="AM184" s="14"/>
     </row>
-    <row r="185" spans="19:39" ht="13.8">
+    <row r="185" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S185" s="15"/>
       <c r="T185" s="15"/>
       <c r="U185" s="15"/>
@@ -17473,7 +17481,7 @@
       <c r="AL185" s="14"/>
       <c r="AM185" s="14"/>
     </row>
-    <row r="186" spans="19:39" ht="13.8">
+    <row r="186" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S186" s="15"/>
       <c r="T186" s="15"/>
       <c r="U186" s="15"/>
@@ -17492,7 +17500,7 @@
       <c r="AL186" s="14"/>
       <c r="AM186" s="14"/>
     </row>
-    <row r="187" spans="19:39" ht="13.8">
+    <row r="187" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S187" s="15"/>
       <c r="T187" s="15"/>
       <c r="U187" s="15"/>
@@ -17511,7 +17519,7 @@
       <c r="AL187" s="14"/>
       <c r="AM187" s="14"/>
     </row>
-    <row r="188" spans="19:39" ht="13.8">
+    <row r="188" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S188" s="15"/>
       <c r="T188" s="15"/>
       <c r="U188" s="15"/>
@@ -17530,7 +17538,7 @@
       <c r="AL188" s="14"/>
       <c r="AM188" s="14"/>
     </row>
-    <row r="189" spans="19:39" ht="13.8">
+    <row r="189" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S189" s="15"/>
       <c r="T189" s="15"/>
       <c r="U189" s="15"/>
@@ -17549,7 +17557,7 @@
       <c r="AL189" s="14"/>
       <c r="AM189" s="14"/>
     </row>
-    <row r="190" spans="19:39" ht="13.8">
+    <row r="190" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S190" s="15"/>
       <c r="T190" s="15"/>
       <c r="U190" s="15"/>
@@ -17568,7 +17576,7 @@
       <c r="AL190" s="14"/>
       <c r="AM190" s="14"/>
     </row>
-    <row r="191" spans="19:39" ht="13.8">
+    <row r="191" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S191" s="15"/>
       <c r="T191" s="15"/>
       <c r="U191" s="15"/>
@@ -17587,7 +17595,7 @@
       <c r="AL191" s="14"/>
       <c r="AM191" s="14"/>
     </row>
-    <row r="192" spans="19:39" ht="13.8">
+    <row r="192" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S192" s="15"/>
       <c r="T192" s="15"/>
       <c r="U192" s="15"/>
@@ -17606,7 +17614,7 @@
       <c r="AL192" s="14"/>
       <c r="AM192" s="14"/>
     </row>
-    <row r="193" spans="19:39" ht="13.8">
+    <row r="193" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S193" s="15"/>
       <c r="T193" s="15"/>
       <c r="U193" s="15"/>
@@ -17625,7 +17633,7 @@
       <c r="AL193" s="14"/>
       <c r="AM193" s="14"/>
     </row>
-    <row r="194" spans="19:39" ht="13.8">
+    <row r="194" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S194" s="15"/>
       <c r="T194" s="15"/>
       <c r="U194" s="15"/>
@@ -17644,7 +17652,7 @@
       <c r="AL194" s="14"/>
       <c r="AM194" s="14"/>
     </row>
-    <row r="195" spans="19:39" ht="13.8">
+    <row r="195" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S195" s="15"/>
       <c r="T195" s="15"/>
       <c r="U195" s="15"/>
@@ -17663,7 +17671,7 @@
       <c r="AL195" s="14"/>
       <c r="AM195" s="14"/>
     </row>
-    <row r="196" spans="19:39" ht="13.8">
+    <row r="196" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
       <c r="S196" s="15"/>
       <c r="T196" s="15"/>
       <c r="U196" s="15"/>
@@ -17682,7 +17690,7 @@
       <c r="AL196" s="14"/>
       <c r="AM196" s="14"/>
     </row>
-    <row r="197" spans="19:39" ht="14.4" thickBot="1">
+    <row r="197" spans="19:39" ht="23.15" thickBot="1" x14ac:dyDescent="0.95">
       <c r="S197" s="15"/>
       <c r="T197" s="15"/>
       <c r="U197" s="15"/>
@@ -17703,18 +17711,12 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="K1:K2"/>
-    <mergeCell ref="L1:L2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="G1:G2"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="I1:I2"/>
-    <mergeCell ref="J1:J2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="AB26:AB27"/>
+    <mergeCell ref="A30:A31"/>
+    <mergeCell ref="AB30:AB31"/>
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="AB35:AB36"/>
     <mergeCell ref="AB1:AB2"/>
     <mergeCell ref="M1:M2"/>
     <mergeCell ref="N1:N2"/>
@@ -17727,12 +17729,18 @@
     <mergeCell ref="Z1:Z2"/>
     <mergeCell ref="AA1:AA2"/>
     <mergeCell ref="P1:R1"/>
-    <mergeCell ref="A26:A27"/>
-    <mergeCell ref="AB26:AB27"/>
-    <mergeCell ref="A30:A31"/>
-    <mergeCell ref="AB30:AB31"/>
-    <mergeCell ref="A35:A36"/>
-    <mergeCell ref="AB35:AB36"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="K1:K2"/>
+    <mergeCell ref="L1:L2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="I1:I2"/>
+    <mergeCell ref="J1:J2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
update and optimization cards
</commit_message>
<xml_diff>
--- a/assets/data-source/data.xlsx
+++ b/assets/data-source/data.xlsx
@@ -1,38 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Venus\Desktop\PahnavarKar\assets\data-source\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9231CA9A-1CF2-4A8C-B435-2E0082B2318E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2704CEFB-7758-4BEF-B314-1E6471F7F886}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="23657" windowHeight="15394" tabRatio="736" activeTab="1" xr2:uid="{2E6F1639-AB3B-4860-9C01-087F2448B9B1}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="736" activeTab="1" xr2:uid="{2E6F1639-AB3B-4860-9C01-087F2448B9B1}"/>
   </bookViews>
   <sheets>
     <sheet name="پایه سنوات طرح طبقه" sheetId="33" r:id="rId1"/>
     <sheet name="پایه سنوات عادی و داده ها" sheetId="34" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="181029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="110">
   <si>
     <t>پایه سنوات</t>
   </si>
@@ -80,9 +69,6 @@
   </si>
   <si>
     <t>پایه سنواتی جاری</t>
-  </si>
-  <si>
-    <t>پایه سنوات استحقاقی</t>
   </si>
   <si>
     <t>مبلغ اضافه كاری یک ساعت</t>
@@ -376,7 +362,7 @@
     <numFmt numFmtId="165" formatCode="0;[Red]0"/>
     <numFmt numFmtId="166" formatCode="0.000;[Red]0.000"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="11">
     <font>
       <sz val="14"/>
       <name val="B Nazanin"/>
@@ -995,6 +981,18 @@
     <xf numFmtId="0" fontId="10" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="2" fontId="10" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="3" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1063,18 +1061,6 @@
     </xf>
     <xf numFmtId="165" fontId="5" fillId="4" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="10" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1381,581 +1367,581 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F3FFB2F-BC88-43B7-B5AC-FC5BC58FCAEB}">
   <dimension ref="A1:DH348"/>
-  <sheetFormatPr defaultColWidth="14.46484375" defaultRowHeight="25.75" x14ac:dyDescent="0.9"/>
+  <sheetFormatPr defaultColWidth="14.4609375" defaultRowHeight="17.399999999999999"/>
   <cols>
-    <col min="1" max="1" width="14.46484375" style="37" customWidth="1"/>
-    <col min="2" max="16384" width="14.46484375" style="31"/>
+    <col min="1" max="1" width="14.4609375" style="37" customWidth="1"/>
+    <col min="2" max="16384" width="14.4609375" style="31"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:112" s="39" customFormat="1" ht="23.15" customHeight="1" x14ac:dyDescent="0.9">
+    <row r="1" spans="1:112" s="39" customFormat="1" ht="23.1" customHeight="1">
       <c r="A1" s="38" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="67">
+      <c r="B1" s="44">
         <v>1369</v>
       </c>
-      <c r="C1" s="68"/>
-      <c r="D1" s="68"/>
-      <c r="E1" s="67">
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="44">
         <v>1370</v>
       </c>
-      <c r="F1" s="68"/>
-      <c r="G1" s="68"/>
-      <c r="H1" s="67">
+      <c r="F1" s="45"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="44">
         <v>1371</v>
       </c>
-      <c r="I1" s="68"/>
-      <c r="J1" s="68"/>
-      <c r="K1" s="67">
+      <c r="I1" s="45"/>
+      <c r="J1" s="45"/>
+      <c r="K1" s="44">
         <v>1372</v>
       </c>
-      <c r="L1" s="68"/>
-      <c r="M1" s="68"/>
-      <c r="N1" s="67">
+      <c r="L1" s="45"/>
+      <c r="M1" s="45"/>
+      <c r="N1" s="44">
         <v>1373</v>
       </c>
-      <c r="O1" s="68"/>
-      <c r="P1" s="68"/>
-      <c r="Q1" s="67">
+      <c r="O1" s="45"/>
+      <c r="P1" s="45"/>
+      <c r="Q1" s="44">
         <v>1374</v>
       </c>
-      <c r="R1" s="68"/>
-      <c r="S1" s="68"/>
-      <c r="T1" s="67">
+      <c r="R1" s="45"/>
+      <c r="S1" s="45"/>
+      <c r="T1" s="44">
         <v>1375</v>
       </c>
-      <c r="U1" s="68"/>
-      <c r="V1" s="68"/>
-      <c r="W1" s="67">
+      <c r="U1" s="45"/>
+      <c r="V1" s="45"/>
+      <c r="W1" s="44">
         <v>1376</v>
       </c>
-      <c r="X1" s="68"/>
-      <c r="Y1" s="68"/>
-      <c r="Z1" s="67">
+      <c r="X1" s="45"/>
+      <c r="Y1" s="45"/>
+      <c r="Z1" s="44">
         <v>1377</v>
       </c>
-      <c r="AA1" s="68"/>
-      <c r="AB1" s="68"/>
-      <c r="AC1" s="67">
+      <c r="AA1" s="45"/>
+      <c r="AB1" s="45"/>
+      <c r="AC1" s="44">
         <v>1378</v>
       </c>
-      <c r="AD1" s="68"/>
-      <c r="AE1" s="68"/>
-      <c r="AF1" s="67">
+      <c r="AD1" s="45"/>
+      <c r="AE1" s="45"/>
+      <c r="AF1" s="44">
         <v>1379</v>
       </c>
-      <c r="AG1" s="68"/>
-      <c r="AH1" s="68"/>
-      <c r="AI1" s="67">
+      <c r="AG1" s="45"/>
+      <c r="AH1" s="45"/>
+      <c r="AI1" s="44">
         <v>1380</v>
       </c>
-      <c r="AJ1" s="68"/>
-      <c r="AK1" s="68"/>
-      <c r="AL1" s="67">
+      <c r="AJ1" s="45"/>
+      <c r="AK1" s="45"/>
+      <c r="AL1" s="44">
         <v>1381</v>
       </c>
-      <c r="AM1" s="68"/>
-      <c r="AN1" s="68"/>
-      <c r="AO1" s="67">
+      <c r="AM1" s="45"/>
+      <c r="AN1" s="45"/>
+      <c r="AO1" s="44">
         <v>1382</v>
       </c>
-      <c r="AP1" s="68"/>
-      <c r="AQ1" s="68"/>
-      <c r="AR1" s="67">
+      <c r="AP1" s="45"/>
+      <c r="AQ1" s="45"/>
+      <c r="AR1" s="44">
         <v>1383</v>
       </c>
-      <c r="AS1" s="68"/>
-      <c r="AT1" s="68"/>
-      <c r="AU1" s="67">
+      <c r="AS1" s="45"/>
+      <c r="AT1" s="45"/>
+      <c r="AU1" s="44">
         <v>1384</v>
       </c>
-      <c r="AV1" s="68"/>
-      <c r="AW1" s="68"/>
-      <c r="AX1" s="67">
+      <c r="AV1" s="45"/>
+      <c r="AW1" s="45"/>
+      <c r="AX1" s="44">
         <v>1385</v>
       </c>
-      <c r="AY1" s="68"/>
-      <c r="AZ1" s="68"/>
-      <c r="BA1" s="67">
+      <c r="AY1" s="45"/>
+      <c r="AZ1" s="45"/>
+      <c r="BA1" s="44">
         <v>1386</v>
       </c>
-      <c r="BB1" s="68"/>
-      <c r="BC1" s="68"/>
-      <c r="BD1" s="67">
+      <c r="BB1" s="45"/>
+      <c r="BC1" s="45"/>
+      <c r="BD1" s="44">
         <v>1387</v>
       </c>
-      <c r="BE1" s="68"/>
-      <c r="BF1" s="68"/>
-      <c r="BG1" s="67">
+      <c r="BE1" s="45"/>
+      <c r="BF1" s="45"/>
+      <c r="BG1" s="44">
         <v>1388</v>
       </c>
-      <c r="BH1" s="68"/>
-      <c r="BI1" s="68"/>
-      <c r="BJ1" s="67">
+      <c r="BH1" s="45"/>
+      <c r="BI1" s="45"/>
+      <c r="BJ1" s="44">
         <v>1389</v>
       </c>
-      <c r="BK1" s="68"/>
-      <c r="BL1" s="68"/>
-      <c r="BM1" s="67">
+      <c r="BK1" s="45"/>
+      <c r="BL1" s="45"/>
+      <c r="BM1" s="44">
         <v>1390</v>
       </c>
-      <c r="BN1" s="68"/>
-      <c r="BO1" s="68"/>
-      <c r="BP1" s="67">
+      <c r="BN1" s="45"/>
+      <c r="BO1" s="45"/>
+      <c r="BP1" s="44">
         <v>1391</v>
       </c>
-      <c r="BQ1" s="68"/>
-      <c r="BR1" s="68"/>
-      <c r="BS1" s="67">
+      <c r="BQ1" s="45"/>
+      <c r="BR1" s="45"/>
+      <c r="BS1" s="44">
         <v>1392</v>
       </c>
-      <c r="BT1" s="68"/>
-      <c r="BU1" s="68"/>
-      <c r="BV1" s="67">
+      <c r="BT1" s="45"/>
+      <c r="BU1" s="45"/>
+      <c r="BV1" s="44">
         <v>1393</v>
       </c>
-      <c r="BW1" s="68"/>
-      <c r="BX1" s="68"/>
-      <c r="BY1" s="67">
+      <c r="BW1" s="45"/>
+      <c r="BX1" s="45"/>
+      <c r="BY1" s="44">
         <v>1394</v>
       </c>
-      <c r="BZ1" s="68"/>
-      <c r="CA1" s="68"/>
-      <c r="CB1" s="67">
+      <c r="BZ1" s="45"/>
+      <c r="CA1" s="45"/>
+      <c r="CB1" s="44">
         <v>1395</v>
       </c>
-      <c r="CC1" s="68"/>
-      <c r="CD1" s="68"/>
-      <c r="CE1" s="67">
+      <c r="CC1" s="45"/>
+      <c r="CD1" s="45"/>
+      <c r="CE1" s="44">
         <v>1396</v>
       </c>
-      <c r="CF1" s="68"/>
-      <c r="CG1" s="68"/>
-      <c r="CH1" s="67">
+      <c r="CF1" s="45"/>
+      <c r="CG1" s="45"/>
+      <c r="CH1" s="44">
         <v>1397</v>
       </c>
-      <c r="CI1" s="68"/>
-      <c r="CJ1" s="68"/>
-      <c r="CK1" s="67">
+      <c r="CI1" s="45"/>
+      <c r="CJ1" s="45"/>
+      <c r="CK1" s="44">
         <v>1398</v>
       </c>
-      <c r="CL1" s="68"/>
-      <c r="CM1" s="68"/>
-      <c r="CN1" s="67">
+      <c r="CL1" s="45"/>
+      <c r="CM1" s="45"/>
+      <c r="CN1" s="44">
         <v>1399</v>
       </c>
-      <c r="CO1" s="68"/>
-      <c r="CP1" s="68"/>
-      <c r="CQ1" s="67">
+      <c r="CO1" s="45"/>
+      <c r="CP1" s="45"/>
+      <c r="CQ1" s="44">
         <v>1400</v>
       </c>
-      <c r="CR1" s="68"/>
-      <c r="CS1" s="68"/>
-      <c r="CT1" s="67">
+      <c r="CR1" s="45"/>
+      <c r="CS1" s="45"/>
+      <c r="CT1" s="44">
         <v>1401</v>
       </c>
-      <c r="CU1" s="68"/>
-      <c r="CV1" s="68"/>
-      <c r="CW1" s="67">
+      <c r="CU1" s="45"/>
+      <c r="CV1" s="45"/>
+      <c r="CW1" s="44">
         <v>1402</v>
       </c>
-      <c r="CX1" s="68"/>
-      <c r="CY1" s="68"/>
-      <c r="CZ1" s="67">
+      <c r="CX1" s="45"/>
+      <c r="CY1" s="45"/>
+      <c r="CZ1" s="44">
         <v>1403</v>
       </c>
-      <c r="DA1" s="68"/>
-      <c r="DB1" s="68"/>
-      <c r="DC1" s="67">
+      <c r="DA1" s="45"/>
+      <c r="DB1" s="45"/>
+      <c r="DC1" s="44">
         <v>1404</v>
       </c>
-      <c r="DD1" s="68"/>
-      <c r="DE1" s="68"/>
-      <c r="DF1" s="67">
+      <c r="DD1" s="45"/>
+      <c r="DE1" s="45"/>
+      <c r="DF1" s="44">
         <v>1405</v>
       </c>
-      <c r="DG1" s="68"/>
-      <c r="DH1" s="68"/>
-    </row>
-    <row r="2" spans="1:112" s="41" customFormat="1" ht="31.4" customHeight="1" x14ac:dyDescent="0.9">
+      <c r="DG1" s="45"/>
+      <c r="DH1" s="45"/>
+    </row>
+    <row r="2" spans="1:112" s="41" customFormat="1" ht="31.35" customHeight="1">
       <c r="A2" s="40" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="65">
+      <c r="B2" s="42">
         <v>1.1399999999999999</v>
       </c>
-      <c r="C2" s="65"/>
-      <c r="D2" s="65"/>
-      <c r="E2" s="65">
+      <c r="C2" s="42"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42">
         <v>1.1200000000000001</v>
       </c>
-      <c r="F2" s="65"/>
-      <c r="G2" s="65"/>
-      <c r="H2" s="65">
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42">
         <v>1.101</v>
       </c>
-      <c r="I2" s="65"/>
-      <c r="J2" s="65"/>
-      <c r="K2" s="65">
+      <c r="I2" s="42"/>
+      <c r="J2" s="42"/>
+      <c r="K2" s="42">
         <v>1.1299999999999999</v>
       </c>
-      <c r="L2" s="65"/>
-      <c r="M2" s="65"/>
-      <c r="N2" s="65">
+      <c r="L2" s="42"/>
+      <c r="M2" s="42"/>
+      <c r="N2" s="42">
         <v>1.1499999999999999</v>
       </c>
-      <c r="O2" s="65"/>
-      <c r="P2" s="65"/>
-      <c r="Q2" s="65">
+      <c r="O2" s="42"/>
+      <c r="P2" s="42"/>
+      <c r="Q2" s="42">
         <v>1.26</v>
       </c>
-      <c r="R2" s="65"/>
-      <c r="S2" s="65"/>
-      <c r="T2" s="65">
+      <c r="R2" s="42"/>
+      <c r="S2" s="42"/>
+      <c r="T2" s="42">
         <v>1.38</v>
       </c>
-      <c r="U2" s="65"/>
-      <c r="V2" s="65"/>
-      <c r="W2" s="65">
+      <c r="U2" s="42"/>
+      <c r="V2" s="42"/>
+      <c r="W2" s="42">
         <v>1.21</v>
       </c>
-      <c r="X2" s="65"/>
-      <c r="Y2" s="65"/>
-      <c r="Z2" s="65">
+      <c r="X2" s="42"/>
+      <c r="Y2" s="42"/>
+      <c r="Z2" s="42">
         <v>1.22</v>
       </c>
-      <c r="AA2" s="65"/>
-      <c r="AB2" s="65"/>
-      <c r="AC2" s="65">
+      <c r="AA2" s="42"/>
+      <c r="AB2" s="42"/>
+      <c r="AC2" s="42">
         <v>1.32</v>
       </c>
-      <c r="AD2" s="65"/>
-      <c r="AE2" s="65"/>
-      <c r="AF2" s="65">
+      <c r="AD2" s="42"/>
+      <c r="AE2" s="42"/>
+      <c r="AF2" s="42">
         <v>1.45</v>
       </c>
-      <c r="AG2" s="65"/>
-      <c r="AH2" s="65"/>
-      <c r="AI2" s="65">
+      <c r="AG2" s="42"/>
+      <c r="AH2" s="42"/>
+      <c r="AI2" s="42">
         <v>1.1200000000000001</v>
       </c>
-      <c r="AJ2" s="65"/>
-      <c r="AK2" s="65"/>
-      <c r="AL2" s="65">
+      <c r="AJ2" s="42"/>
+      <c r="AK2" s="42"/>
+      <c r="AL2" s="42">
         <v>1.17</v>
       </c>
-      <c r="AM2" s="65"/>
-      <c r="AN2" s="65"/>
-      <c r="AO2" s="65">
+      <c r="AM2" s="42"/>
+      <c r="AN2" s="42"/>
+      <c r="AO2" s="42">
         <v>1.1399999999999999</v>
       </c>
-      <c r="AP2" s="65"/>
-      <c r="AQ2" s="65"/>
-      <c r="AR2" s="65">
+      <c r="AP2" s="42"/>
+      <c r="AQ2" s="42"/>
+      <c r="AR2" s="42">
         <v>1.1200000000000001</v>
       </c>
-      <c r="AS2" s="65"/>
-      <c r="AT2" s="65"/>
-      <c r="AU2" s="65">
+      <c r="AS2" s="42"/>
+      <c r="AT2" s="42"/>
+      <c r="AU2" s="42">
         <v>1.101</v>
       </c>
-      <c r="AV2" s="65"/>
-      <c r="AW2" s="65"/>
-      <c r="AX2" s="65">
+      <c r="AV2" s="42"/>
+      <c r="AW2" s="42"/>
+      <c r="AX2" s="42">
         <v>1.1299999999999999</v>
       </c>
-      <c r="AY2" s="65"/>
-      <c r="AZ2" s="65"/>
-      <c r="BA2" s="65">
+      <c r="AY2" s="42"/>
+      <c r="AZ2" s="42"/>
+      <c r="BA2" s="42">
         <v>1.1499999999999999</v>
       </c>
-      <c r="BB2" s="65"/>
-      <c r="BC2" s="65"/>
-      <c r="BD2" s="65">
+      <c r="BB2" s="42"/>
+      <c r="BC2" s="42"/>
+      <c r="BD2" s="42">
         <v>1.26</v>
       </c>
-      <c r="BE2" s="65"/>
-      <c r="BF2" s="65"/>
-      <c r="BG2" s="65">
+      <c r="BE2" s="42"/>
+      <c r="BF2" s="42"/>
+      <c r="BG2" s="42">
         <v>1.38</v>
       </c>
-      <c r="BH2" s="65"/>
-      <c r="BI2" s="65"/>
-      <c r="BJ2" s="65">
+      <c r="BH2" s="42"/>
+      <c r="BI2" s="42"/>
+      <c r="BJ2" s="42">
         <v>1.21</v>
       </c>
-      <c r="BK2" s="65"/>
-      <c r="BL2" s="65"/>
-      <c r="BM2" s="65">
+      <c r="BK2" s="42"/>
+      <c r="BL2" s="42"/>
+      <c r="BM2" s="42">
         <v>1.22</v>
       </c>
-      <c r="BN2" s="65"/>
-      <c r="BO2" s="65"/>
-      <c r="BP2" s="65">
+      <c r="BN2" s="42"/>
+      <c r="BO2" s="42"/>
+      <c r="BP2" s="42">
         <v>1.1000000000000001</v>
       </c>
-      <c r="BQ2" s="65"/>
-      <c r="BR2" s="65"/>
-      <c r="BS2" s="65">
+      <c r="BQ2" s="42"/>
+      <c r="BR2" s="42"/>
+      <c r="BS2" s="42">
         <v>1.1000000000000001</v>
       </c>
-      <c r="BT2" s="65"/>
-      <c r="BU2" s="65"/>
-      <c r="BV2" s="65">
+      <c r="BT2" s="42"/>
+      <c r="BU2" s="42"/>
+      <c r="BV2" s="42">
         <v>1.1200000000000001</v>
       </c>
-      <c r="BW2" s="65"/>
-      <c r="BX2" s="65"/>
-      <c r="BY2" s="65">
+      <c r="BW2" s="42"/>
+      <c r="BX2" s="42"/>
+      <c r="BY2" s="42">
         <v>1.17</v>
       </c>
-      <c r="BZ2" s="65"/>
-      <c r="CA2" s="65"/>
-      <c r="CB2" s="65">
+      <c r="BZ2" s="42"/>
+      <c r="CA2" s="42"/>
+      <c r="CB2" s="42">
         <v>1.1399999999999999</v>
       </c>
-      <c r="CC2" s="65"/>
-      <c r="CD2" s="65"/>
-      <c r="CE2" s="65">
+      <c r="CC2" s="42"/>
+      <c r="CD2" s="42"/>
+      <c r="CE2" s="42">
         <v>1.1200000000000001</v>
       </c>
-      <c r="CF2" s="65"/>
-      <c r="CG2" s="65"/>
-      <c r="CH2" s="65">
+      <c r="CF2" s="42"/>
+      <c r="CG2" s="42"/>
+      <c r="CH2" s="42">
         <v>1.101</v>
       </c>
-      <c r="CI2" s="65"/>
-      <c r="CJ2" s="65"/>
-      <c r="CK2" s="65">
+      <c r="CI2" s="42"/>
+      <c r="CJ2" s="42"/>
+      <c r="CK2" s="42">
         <v>1.1299999999999999</v>
       </c>
-      <c r="CL2" s="65"/>
-      <c r="CM2" s="65"/>
-      <c r="CN2" s="65">
+      <c r="CL2" s="42"/>
+      <c r="CM2" s="42"/>
+      <c r="CN2" s="42">
         <v>1.1499999999999999</v>
       </c>
-      <c r="CO2" s="65"/>
-      <c r="CP2" s="65"/>
-      <c r="CQ2" s="65">
+      <c r="CO2" s="42"/>
+      <c r="CP2" s="42"/>
+      <c r="CQ2" s="42">
         <v>1.26</v>
       </c>
-      <c r="CR2" s="65"/>
-      <c r="CS2" s="65"/>
-      <c r="CT2" s="65">
+      <c r="CR2" s="42"/>
+      <c r="CS2" s="42"/>
+      <c r="CT2" s="42">
         <v>1.38</v>
       </c>
-      <c r="CU2" s="65"/>
-      <c r="CV2" s="65"/>
-      <c r="CW2" s="65">
+      <c r="CU2" s="42"/>
+      <c r="CV2" s="42"/>
+      <c r="CW2" s="42">
         <v>1.21</v>
       </c>
-      <c r="CX2" s="65"/>
-      <c r="CY2" s="65"/>
-      <c r="CZ2" s="65">
+      <c r="CX2" s="42"/>
+      <c r="CY2" s="42"/>
+      <c r="CZ2" s="42">
         <v>1.22</v>
       </c>
-      <c r="DA2" s="65"/>
-      <c r="DB2" s="65"/>
-      <c r="DC2" s="65">
+      <c r="DA2" s="42"/>
+      <c r="DB2" s="42"/>
+      <c r="DC2" s="42">
         <v>1.32</v>
       </c>
-      <c r="DD2" s="65"/>
-      <c r="DE2" s="65"/>
-      <c r="DF2" s="65">
+      <c r="DD2" s="42"/>
+      <c r="DE2" s="42"/>
+      <c r="DF2" s="42">
         <v>1.45</v>
       </c>
-      <c r="DG2" s="65"/>
-      <c r="DH2" s="65"/>
-    </row>
-    <row r="3" spans="1:112" s="41" customFormat="1" ht="40.85" customHeight="1" x14ac:dyDescent="0.9">
+      <c r="DG2" s="42"/>
+      <c r="DH2" s="42"/>
+    </row>
+    <row r="3" spans="1:112" s="41" customFormat="1" ht="40.799999999999997" customHeight="1">
       <c r="A3" s="40"/>
-      <c r="B3" s="65" t="s">
+      <c r="B3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="66"/>
-      <c r="D3" s="66"/>
-      <c r="E3" s="65" t="s">
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="F3" s="66"/>
-      <c r="G3" s="66"/>
-      <c r="H3" s="65" t="s">
+      <c r="F3" s="43"/>
+      <c r="G3" s="43"/>
+      <c r="H3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="I3" s="66"/>
-      <c r="J3" s="66"/>
-      <c r="K3" s="65" t="s">
+      <c r="I3" s="43"/>
+      <c r="J3" s="43"/>
+      <c r="K3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="L3" s="66"/>
-      <c r="M3" s="66"/>
-      <c r="N3" s="65" t="s">
+      <c r="L3" s="43"/>
+      <c r="M3" s="43"/>
+      <c r="N3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="O3" s="66"/>
-      <c r="P3" s="66"/>
-      <c r="Q3" s="65" t="s">
+      <c r="O3" s="43"/>
+      <c r="P3" s="43"/>
+      <c r="Q3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="R3" s="66"/>
-      <c r="S3" s="66"/>
-      <c r="T3" s="65" t="s">
+      <c r="R3" s="43"/>
+      <c r="S3" s="43"/>
+      <c r="T3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="U3" s="66"/>
-      <c r="V3" s="66"/>
-      <c r="W3" s="65" t="s">
+      <c r="U3" s="43"/>
+      <c r="V3" s="43"/>
+      <c r="W3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="X3" s="66"/>
-      <c r="Y3" s="66"/>
-      <c r="Z3" s="65" t="s">
+      <c r="X3" s="43"/>
+      <c r="Y3" s="43"/>
+      <c r="Z3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="AA3" s="66"/>
-      <c r="AB3" s="66"/>
-      <c r="AC3" s="65" t="s">
+      <c r="AA3" s="43"/>
+      <c r="AB3" s="43"/>
+      <c r="AC3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="AD3" s="66"/>
-      <c r="AE3" s="66"/>
-      <c r="AF3" s="65" t="s">
+      <c r="AD3" s="43"/>
+      <c r="AE3" s="43"/>
+      <c r="AF3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="AG3" s="66"/>
-      <c r="AH3" s="66"/>
-      <c r="AI3" s="65" t="s">
+      <c r="AG3" s="43"/>
+      <c r="AH3" s="43"/>
+      <c r="AI3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="AJ3" s="66"/>
-      <c r="AK3" s="66"/>
-      <c r="AL3" s="65" t="s">
+      <c r="AJ3" s="43"/>
+      <c r="AK3" s="43"/>
+      <c r="AL3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="AM3" s="66"/>
-      <c r="AN3" s="66"/>
-      <c r="AO3" s="65" t="s">
+      <c r="AM3" s="43"/>
+      <c r="AN3" s="43"/>
+      <c r="AO3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="AP3" s="66"/>
-      <c r="AQ3" s="66"/>
-      <c r="AR3" s="65" t="s">
+      <c r="AP3" s="43"/>
+      <c r="AQ3" s="43"/>
+      <c r="AR3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="AS3" s="66"/>
-      <c r="AT3" s="66"/>
-      <c r="AU3" s="65" t="s">
+      <c r="AS3" s="43"/>
+      <c r="AT3" s="43"/>
+      <c r="AU3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="AV3" s="66"/>
-      <c r="AW3" s="66"/>
-      <c r="AX3" s="65" t="s">
+      <c r="AV3" s="43"/>
+      <c r="AW3" s="43"/>
+      <c r="AX3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="AY3" s="66"/>
-      <c r="AZ3" s="66"/>
-      <c r="BA3" s="65" t="s">
+      <c r="AY3" s="43"/>
+      <c r="AZ3" s="43"/>
+      <c r="BA3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="BB3" s="66"/>
-      <c r="BC3" s="66"/>
-      <c r="BD3" s="65" t="s">
+      <c r="BB3" s="43"/>
+      <c r="BC3" s="43"/>
+      <c r="BD3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="BE3" s="66"/>
-      <c r="BF3" s="66"/>
-      <c r="BG3" s="65" t="s">
+      <c r="BE3" s="43"/>
+      <c r="BF3" s="43"/>
+      <c r="BG3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="BH3" s="66"/>
-      <c r="BI3" s="66"/>
-      <c r="BJ3" s="65" t="s">
+      <c r="BH3" s="43"/>
+      <c r="BI3" s="43"/>
+      <c r="BJ3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="BK3" s="66"/>
-      <c r="BL3" s="66"/>
-      <c r="BM3" s="65" t="s">
+      <c r="BK3" s="43"/>
+      <c r="BL3" s="43"/>
+      <c r="BM3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="BN3" s="66"/>
-      <c r="BO3" s="66"/>
-      <c r="BP3" s="65" t="s">
+      <c r="BN3" s="43"/>
+      <c r="BO3" s="43"/>
+      <c r="BP3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="BQ3" s="66"/>
-      <c r="BR3" s="66"/>
-      <c r="BS3" s="65" t="s">
+      <c r="BQ3" s="43"/>
+      <c r="BR3" s="43"/>
+      <c r="BS3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="BT3" s="66"/>
-      <c r="BU3" s="66"/>
-      <c r="BV3" s="65" t="s">
+      <c r="BT3" s="43"/>
+      <c r="BU3" s="43"/>
+      <c r="BV3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="BW3" s="66"/>
-      <c r="BX3" s="66"/>
-      <c r="BY3" s="65" t="s">
+      <c r="BW3" s="43"/>
+      <c r="BX3" s="43"/>
+      <c r="BY3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="BZ3" s="66"/>
-      <c r="CA3" s="66"/>
-      <c r="CB3" s="65" t="s">
+      <c r="BZ3" s="43"/>
+      <c r="CA3" s="43"/>
+      <c r="CB3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="CC3" s="66"/>
-      <c r="CD3" s="66"/>
-      <c r="CE3" s="65" t="s">
+      <c r="CC3" s="43"/>
+      <c r="CD3" s="43"/>
+      <c r="CE3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="CF3" s="66"/>
-      <c r="CG3" s="66"/>
-      <c r="CH3" s="65" t="s">
+      <c r="CF3" s="43"/>
+      <c r="CG3" s="43"/>
+      <c r="CH3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="CI3" s="66"/>
-      <c r="CJ3" s="66"/>
-      <c r="CK3" s="65" t="s">
+      <c r="CI3" s="43"/>
+      <c r="CJ3" s="43"/>
+      <c r="CK3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="CL3" s="66"/>
-      <c r="CM3" s="66"/>
-      <c r="CN3" s="65" t="s">
+      <c r="CL3" s="43"/>
+      <c r="CM3" s="43"/>
+      <c r="CN3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="CO3" s="66"/>
-      <c r="CP3" s="66"/>
-      <c r="CQ3" s="65" t="s">
+      <c r="CO3" s="43"/>
+      <c r="CP3" s="43"/>
+      <c r="CQ3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="CR3" s="66"/>
-      <c r="CS3" s="66"/>
-      <c r="CT3" s="65" t="s">
+      <c r="CR3" s="43"/>
+      <c r="CS3" s="43"/>
+      <c r="CT3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="CU3" s="66"/>
-      <c r="CV3" s="66"/>
-      <c r="CW3" s="65" t="s">
+      <c r="CU3" s="43"/>
+      <c r="CV3" s="43"/>
+      <c r="CW3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="CX3" s="66"/>
-      <c r="CY3" s="66"/>
-      <c r="CZ3" s="65" t="s">
+      <c r="CX3" s="43"/>
+      <c r="CY3" s="43"/>
+      <c r="CZ3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="DA3" s="66"/>
-      <c r="DB3" s="66"/>
-      <c r="DC3" s="65" t="s">
+      <c r="DA3" s="43"/>
+      <c r="DB3" s="43"/>
+      <c r="DC3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="DD3" s="66"/>
-      <c r="DE3" s="66"/>
-      <c r="DF3" s="65" t="s">
+      <c r="DD3" s="43"/>
+      <c r="DE3" s="43"/>
+      <c r="DF3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="DG3" s="66"/>
-      <c r="DH3" s="66"/>
-    </row>
-    <row r="4" spans="1:112" s="27" customFormat="1" ht="40.85" customHeight="1" x14ac:dyDescent="0.9">
+      <c r="DG3" s="43"/>
+      <c r="DH3" s="43"/>
+    </row>
+    <row r="4" spans="1:112" s="27" customFormat="1" ht="40.799999999999997" customHeight="1">
       <c r="A4" s="32" t="s">
         <v>5</v>
       </c>
@@ -2291,7 +2277,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:112" s="35" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.9">
+    <row r="5" spans="1:112" s="35" customFormat="1" ht="27" customHeight="1">
       <c r="A5" s="33">
         <v>1</v>
       </c>
@@ -2708,7 +2694,7 @@
         <v>289017092.6656388</v>
       </c>
     </row>
-    <row r="6" spans="1:112" x14ac:dyDescent="0.9">
+    <row r="6" spans="1:112">
       <c r="A6" s="34">
         <v>2</v>
       </c>
@@ -3129,7 +3115,7 @@
         <v>289904014.05304569</v>
       </c>
     </row>
-    <row r="7" spans="1:112" x14ac:dyDescent="0.9">
+    <row r="7" spans="1:112">
       <c r="A7" s="34">
         <v>3</v>
       </c>
@@ -3550,7 +3536,7 @@
         <v>289957907.69702905</v>
       </c>
     </row>
-    <row r="8" spans="1:112" x14ac:dyDescent="0.9">
+    <row r="8" spans="1:112">
       <c r="A8" s="34">
         <v>4</v>
       </c>
@@ -3971,7 +3957,7 @@
         <v>290011801.34101248</v>
       </c>
     </row>
-    <row r="9" spans="1:112" x14ac:dyDescent="0.9">
+    <row r="9" spans="1:112">
       <c r="A9" s="34">
         <v>5</v>
       </c>
@@ -4392,7 +4378,7 @@
         <v>290065694.9849959</v>
       </c>
     </row>
-    <row r="10" spans="1:112" x14ac:dyDescent="0.9">
+    <row r="10" spans="1:112">
       <c r="A10" s="34">
         <v>6</v>
       </c>
@@ -4813,7 +4799,7 @@
         <v>290119588.62897927</v>
       </c>
     </row>
-    <row r="11" spans="1:112" x14ac:dyDescent="0.9">
+    <row r="11" spans="1:112">
       <c r="A11" s="34">
         <v>7</v>
       </c>
@@ -5234,7 +5220,7 @@
         <v>290173482.27296269</v>
       </c>
     </row>
-    <row r="12" spans="1:112" x14ac:dyDescent="0.9">
+    <row r="12" spans="1:112">
       <c r="A12" s="34">
         <v>8</v>
       </c>
@@ -5655,7 +5641,7 @@
         <v>290227375.91694611</v>
       </c>
     </row>
-    <row r="13" spans="1:112" x14ac:dyDescent="0.9">
+    <row r="13" spans="1:112">
       <c r="A13" s="34">
         <v>9</v>
       </c>
@@ -6076,7 +6062,7 @@
         <v>290281269.56092954</v>
       </c>
     </row>
-    <row r="14" spans="1:112" x14ac:dyDescent="0.9">
+    <row r="14" spans="1:112">
       <c r="A14" s="34">
         <v>10</v>
       </c>
@@ -6497,7 +6483,7 @@
         <v>290335163.2049129</v>
       </c>
     </row>
-    <row r="15" spans="1:112" x14ac:dyDescent="0.9">
+    <row r="15" spans="1:112">
       <c r="A15" s="34">
         <v>11</v>
       </c>
@@ -6918,7 +6904,7 @@
         <v>290389056.84889632</v>
       </c>
     </row>
-    <row r="16" spans="1:112" x14ac:dyDescent="0.9">
+    <row r="16" spans="1:112">
       <c r="A16" s="34">
         <v>12</v>
       </c>
@@ -7339,7 +7325,7 @@
         <v>290484847.68082577</v>
       </c>
     </row>
-    <row r="17" spans="1:112" x14ac:dyDescent="0.9">
+    <row r="17" spans="1:112">
       <c r="A17" s="34">
         <v>13</v>
       </c>
@@ -7760,7 +7746,7 @@
         <v>290591515.58007014</v>
       </c>
     </row>
-    <row r="18" spans="1:112" x14ac:dyDescent="0.9">
+    <row r="18" spans="1:112">
       <c r="A18" s="34">
         <v>14</v>
       </c>
@@ -8181,7 +8167,7 @@
         <v>290698183.47931457</v>
       </c>
     </row>
-    <row r="19" spans="1:112" x14ac:dyDescent="0.9">
+    <row r="19" spans="1:112">
       <c r="A19" s="34">
         <v>15</v>
       </c>
@@ -8602,7 +8588,7 @@
         <v>290804851.37855899</v>
       </c>
     </row>
-    <row r="20" spans="1:112" x14ac:dyDescent="0.9">
+    <row r="20" spans="1:112">
       <c r="A20" s="34">
         <v>16</v>
       </c>
@@ -9023,7 +9009,7 @@
         <v>290911519.27780336</v>
       </c>
     </row>
-    <row r="21" spans="1:112" x14ac:dyDescent="0.9">
+    <row r="21" spans="1:112">
       <c r="A21" s="34">
         <v>17</v>
       </c>
@@ -9444,7 +9430,7 @@
         <v>291018187.17704779</v>
       </c>
     </row>
-    <row r="22" spans="1:112" x14ac:dyDescent="0.9">
+    <row r="22" spans="1:112">
       <c r="A22" s="34">
         <v>18</v>
       </c>
@@ -9865,7 +9851,7 @@
         <v>291113105.22166628</v>
       </c>
     </row>
-    <row r="23" spans="1:112" x14ac:dyDescent="0.9">
+    <row r="23" spans="1:112">
       <c r="A23" s="34">
         <v>19</v>
       </c>
@@ -10286,7 +10272,7 @@
         <v>291231522.97553647</v>
       </c>
     </row>
-    <row r="24" spans="1:112" x14ac:dyDescent="0.9">
+    <row r="24" spans="1:112">
       <c r="A24" s="34">
         <v>20</v>
       </c>
@@ -10707,322 +10693,322 @@
         <v>291338190.87478095</v>
       </c>
     </row>
-    <row r="33" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="34" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="35" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="36" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="37" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="38" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="39" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="40" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="41" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="42" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="43" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="44" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="45" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="46" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="47" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="48" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="49" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="50" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="51" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="52" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="53" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="54" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="55" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="56" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="57" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="58" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="59" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="60" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="61" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="62" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="63" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="64" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="65" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="66" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="67" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="68" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="69" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="70" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="71" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="72" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="73" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="74" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="75" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="76" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="77" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="78" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="79" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="80" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="81" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="82" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="83" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="84" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="85" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="86" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="87" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="88" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="89" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="90" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="91" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="92" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="93" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="94" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="95" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="96" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="97" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="98" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="99" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="100" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="101" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="102" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="103" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="104" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="105" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="106" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="107" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="108" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="109" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="110" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="111" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="112" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="113" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="114" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="115" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="116" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="117" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="118" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="119" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="120" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="121" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="122" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="123" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="124" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="125" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="126" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="127" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="128" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="129" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="130" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="131" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="132" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="133" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="134" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="135" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="136" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="137" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="138" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="139" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="140" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="141" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="142" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="143" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="144" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="145" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="146" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="147" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="148" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="149" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="150" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="151" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="152" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="153" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="154" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="155" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="156" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="157" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="158" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="159" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="160" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="161" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="162" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="163" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="164" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="165" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="166" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="167" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="168" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="169" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="170" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="171" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="172" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="173" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="174" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="175" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="176" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="177" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="178" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="179" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="180" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="181" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="182" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="183" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="184" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="185" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="186" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="187" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="188" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="189" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="190" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="191" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="192" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="193" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="194" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="195" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="196" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="197" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="198" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="199" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="200" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="201" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="202" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="203" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="204" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="205" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="206" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="207" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="208" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="209" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="210" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="211" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="212" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="213" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="214" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="215" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="216" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="217" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="218" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="219" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="220" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="221" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="222" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="223" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="224" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="225" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="226" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="227" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="228" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="229" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="230" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="231" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="232" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="233" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="234" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="235" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="236" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="237" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="238" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="239" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="240" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="241" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="242" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="243" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="244" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="245" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="246" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="247" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="248" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="249" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="250" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="251" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="252" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="253" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="254" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="255" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="256" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="257" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="258" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="259" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="260" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="261" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="262" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="263" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="264" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="265" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="266" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="267" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="268" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="269" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="270" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="271" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="272" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="273" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="274" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="275" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="276" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="277" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="278" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="279" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="280" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="281" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="282" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="283" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="284" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="285" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="286" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="287" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="288" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="289" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="290" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="291" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="292" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="293" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="294" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="295" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="296" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="297" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="298" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="299" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="300" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="301" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="302" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="303" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="304" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="305" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="306" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="307" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="308" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="309" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="310" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="311" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="312" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="313" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="314" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="315" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="316" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="317" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="318" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="319" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="320" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="321" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="322" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="323" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="324" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="325" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="326" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="327" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="328" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="329" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="330" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="331" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="332" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="333" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="334" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="335" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="336" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="337" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="338" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="339" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="340" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="341" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="342" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="343" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="344" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="345" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="346" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="347" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
-    <row r="348" s="31" customFormat="1" x14ac:dyDescent="0.9"/>
+    <row r="33" s="31" customFormat="1"/>
+    <row r="34" s="31" customFormat="1"/>
+    <row r="35" s="31" customFormat="1"/>
+    <row r="36" s="31" customFormat="1"/>
+    <row r="37" s="31" customFormat="1"/>
+    <row r="38" s="31" customFormat="1"/>
+    <row r="39" s="31" customFormat="1"/>
+    <row r="40" s="31" customFormat="1"/>
+    <row r="41" s="31" customFormat="1"/>
+    <row r="42" s="31" customFormat="1"/>
+    <row r="43" s="31" customFormat="1"/>
+    <row r="44" s="31" customFormat="1"/>
+    <row r="45" s="31" customFormat="1"/>
+    <row r="46" s="31" customFormat="1"/>
+    <row r="47" s="31" customFormat="1"/>
+    <row r="48" s="31" customFormat="1"/>
+    <row r="49" s="31" customFormat="1"/>
+    <row r="50" s="31" customFormat="1"/>
+    <row r="51" s="31" customFormat="1"/>
+    <row r="52" s="31" customFormat="1"/>
+    <row r="53" s="31" customFormat="1"/>
+    <row r="54" s="31" customFormat="1"/>
+    <row r="55" s="31" customFormat="1"/>
+    <row r="56" s="31" customFormat="1"/>
+    <row r="57" s="31" customFormat="1"/>
+    <row r="58" s="31" customFormat="1"/>
+    <row r="59" s="31" customFormat="1"/>
+    <row r="60" s="31" customFormat="1"/>
+    <row r="61" s="31" customFormat="1"/>
+    <row r="62" s="31" customFormat="1"/>
+    <row r="63" s="31" customFormat="1"/>
+    <row r="64" s="31" customFormat="1"/>
+    <row r="65" s="31" customFormat="1"/>
+    <row r="66" s="31" customFormat="1"/>
+    <row r="67" s="31" customFormat="1"/>
+    <row r="68" s="31" customFormat="1"/>
+    <row r="69" s="31" customFormat="1"/>
+    <row r="70" s="31" customFormat="1"/>
+    <row r="71" s="31" customFormat="1"/>
+    <row r="72" s="31" customFormat="1"/>
+    <row r="73" s="31" customFormat="1"/>
+    <row r="74" s="31" customFormat="1"/>
+    <row r="75" s="31" customFormat="1"/>
+    <row r="76" s="31" customFormat="1"/>
+    <row r="77" s="31" customFormat="1"/>
+    <row r="78" s="31" customFormat="1"/>
+    <row r="79" s="31" customFormat="1"/>
+    <row r="80" s="31" customFormat="1"/>
+    <row r="81" s="31" customFormat="1"/>
+    <row r="82" s="31" customFormat="1"/>
+    <row r="83" s="31" customFormat="1"/>
+    <row r="84" s="31" customFormat="1"/>
+    <row r="85" s="31" customFormat="1"/>
+    <row r="86" s="31" customFormat="1"/>
+    <row r="87" s="31" customFormat="1"/>
+    <row r="88" s="31" customFormat="1"/>
+    <row r="89" s="31" customFormat="1"/>
+    <row r="90" s="31" customFormat="1"/>
+    <row r="91" s="31" customFormat="1"/>
+    <row r="92" s="31" customFormat="1"/>
+    <row r="93" s="31" customFormat="1"/>
+    <row r="94" s="31" customFormat="1"/>
+    <row r="95" s="31" customFormat="1"/>
+    <row r="96" s="31" customFormat="1"/>
+    <row r="97" s="31" customFormat="1"/>
+    <row r="98" s="31" customFormat="1"/>
+    <row r="99" s="31" customFormat="1"/>
+    <row r="100" s="31" customFormat="1"/>
+    <row r="101" s="31" customFormat="1"/>
+    <row r="102" s="31" customFormat="1"/>
+    <row r="103" s="31" customFormat="1"/>
+    <row r="104" s="31" customFormat="1"/>
+    <row r="105" s="31" customFormat="1"/>
+    <row r="106" s="31" customFormat="1"/>
+    <row r="107" s="31" customFormat="1"/>
+    <row r="108" s="31" customFormat="1"/>
+    <row r="109" s="31" customFormat="1"/>
+    <row r="110" s="31" customFormat="1"/>
+    <row r="111" s="31" customFormat="1"/>
+    <row r="112" s="31" customFormat="1"/>
+    <row r="113" s="31" customFormat="1"/>
+    <row r="114" s="31" customFormat="1"/>
+    <row r="115" s="31" customFormat="1"/>
+    <row r="116" s="31" customFormat="1"/>
+    <row r="117" s="31" customFormat="1"/>
+    <row r="118" s="31" customFormat="1"/>
+    <row r="119" s="31" customFormat="1"/>
+    <row r="120" s="31" customFormat="1"/>
+    <row r="121" s="31" customFormat="1"/>
+    <row r="122" s="31" customFormat="1"/>
+    <row r="123" s="31" customFormat="1"/>
+    <row r="124" s="31" customFormat="1"/>
+    <row r="125" s="31" customFormat="1"/>
+    <row r="126" s="31" customFormat="1"/>
+    <row r="127" s="31" customFormat="1"/>
+    <row r="128" s="31" customFormat="1"/>
+    <row r="129" s="31" customFormat="1"/>
+    <row r="130" s="31" customFormat="1"/>
+    <row r="131" s="31" customFormat="1"/>
+    <row r="132" s="31" customFormat="1"/>
+    <row r="133" s="31" customFormat="1"/>
+    <row r="134" s="31" customFormat="1"/>
+    <row r="135" s="31" customFormat="1"/>
+    <row r="136" s="31" customFormat="1"/>
+    <row r="137" s="31" customFormat="1"/>
+    <row r="138" s="31" customFormat="1"/>
+    <row r="139" s="31" customFormat="1"/>
+    <row r="140" s="31" customFormat="1"/>
+    <row r="141" s="31" customFormat="1"/>
+    <row r="142" s="31" customFormat="1"/>
+    <row r="143" s="31" customFormat="1"/>
+    <row r="144" s="31" customFormat="1"/>
+    <row r="145" s="31" customFormat="1"/>
+    <row r="146" s="31" customFormat="1"/>
+    <row r="147" s="31" customFormat="1"/>
+    <row r="148" s="31" customFormat="1"/>
+    <row r="149" s="31" customFormat="1"/>
+    <row r="150" s="31" customFormat="1"/>
+    <row r="151" s="31" customFormat="1"/>
+    <row r="152" s="31" customFormat="1"/>
+    <row r="153" s="31" customFormat="1"/>
+    <row r="154" s="31" customFormat="1"/>
+    <row r="155" s="31" customFormat="1"/>
+    <row r="156" s="31" customFormat="1"/>
+    <row r="157" s="31" customFormat="1"/>
+    <row r="158" s="31" customFormat="1"/>
+    <row r="159" s="31" customFormat="1"/>
+    <row r="160" s="31" customFormat="1"/>
+    <row r="161" s="31" customFormat="1"/>
+    <row r="162" s="31" customFormat="1"/>
+    <row r="163" s="31" customFormat="1"/>
+    <row r="164" s="31" customFormat="1"/>
+    <row r="165" s="31" customFormat="1"/>
+    <row r="166" s="31" customFormat="1"/>
+    <row r="167" s="31" customFormat="1"/>
+    <row r="168" s="31" customFormat="1"/>
+    <row r="169" s="31" customFormat="1"/>
+    <row r="170" s="31" customFormat="1"/>
+    <row r="171" s="31" customFormat="1"/>
+    <row r="172" s="31" customFormat="1"/>
+    <row r="173" s="31" customFormat="1"/>
+    <row r="174" s="31" customFormat="1"/>
+    <row r="175" s="31" customFormat="1"/>
+    <row r="176" s="31" customFormat="1"/>
+    <row r="177" s="31" customFormat="1"/>
+    <row r="178" s="31" customFormat="1"/>
+    <row r="179" s="31" customFormat="1"/>
+    <row r="180" s="31" customFormat="1"/>
+    <row r="181" s="31" customFormat="1"/>
+    <row r="182" s="31" customFormat="1"/>
+    <row r="183" s="31" customFormat="1"/>
+    <row r="184" s="31" customFormat="1"/>
+    <row r="185" s="31" customFormat="1"/>
+    <row r="186" s="31" customFormat="1"/>
+    <row r="187" s="31" customFormat="1"/>
+    <row r="188" s="31" customFormat="1"/>
+    <row r="189" s="31" customFormat="1"/>
+    <row r="190" s="31" customFormat="1"/>
+    <row r="191" s="31" customFormat="1"/>
+    <row r="192" s="31" customFormat="1"/>
+    <row r="193" s="31" customFormat="1"/>
+    <row r="194" s="31" customFormat="1"/>
+    <row r="195" s="31" customFormat="1"/>
+    <row r="196" s="31" customFormat="1"/>
+    <row r="197" s="31" customFormat="1"/>
+    <row r="198" s="31" customFormat="1"/>
+    <row r="199" s="31" customFormat="1"/>
+    <row r="200" s="31" customFormat="1"/>
+    <row r="201" s="31" customFormat="1"/>
+    <row r="202" s="31" customFormat="1"/>
+    <row r="203" s="31" customFormat="1"/>
+    <row r="204" s="31" customFormat="1"/>
+    <row r="205" s="31" customFormat="1"/>
+    <row r="206" s="31" customFormat="1"/>
+    <row r="207" s="31" customFormat="1"/>
+    <row r="208" s="31" customFormat="1"/>
+    <row r="209" s="31" customFormat="1"/>
+    <row r="210" s="31" customFormat="1"/>
+    <row r="211" s="31" customFormat="1"/>
+    <row r="212" s="31" customFormat="1"/>
+    <row r="213" s="31" customFormat="1"/>
+    <row r="214" s="31" customFormat="1"/>
+    <row r="215" s="31" customFormat="1"/>
+    <row r="216" s="31" customFormat="1"/>
+    <row r="217" s="31" customFormat="1"/>
+    <row r="218" s="31" customFormat="1"/>
+    <row r="219" s="31" customFormat="1"/>
+    <row r="220" s="31" customFormat="1"/>
+    <row r="221" s="31" customFormat="1"/>
+    <row r="222" s="31" customFormat="1"/>
+    <row r="223" s="31" customFormat="1"/>
+    <row r="224" s="31" customFormat="1"/>
+    <row r="225" s="31" customFormat="1"/>
+    <row r="226" s="31" customFormat="1"/>
+    <row r="227" s="31" customFormat="1"/>
+    <row r="228" s="31" customFormat="1"/>
+    <row r="229" s="31" customFormat="1"/>
+    <row r="230" s="31" customFormat="1"/>
+    <row r="231" s="31" customFormat="1"/>
+    <row r="232" s="31" customFormat="1"/>
+    <row r="233" s="31" customFormat="1"/>
+    <row r="234" s="31" customFormat="1"/>
+    <row r="235" s="31" customFormat="1"/>
+    <row r="236" s="31" customFormat="1"/>
+    <row r="237" s="31" customFormat="1"/>
+    <row r="238" s="31" customFormat="1"/>
+    <row r="239" s="31" customFormat="1"/>
+    <row r="240" s="31" customFormat="1"/>
+    <row r="241" s="31" customFormat="1"/>
+    <row r="242" s="31" customFormat="1"/>
+    <row r="243" s="31" customFormat="1"/>
+    <row r="244" s="31" customFormat="1"/>
+    <row r="245" s="31" customFormat="1"/>
+    <row r="246" s="31" customFormat="1"/>
+    <row r="247" s="31" customFormat="1"/>
+    <row r="248" s="31" customFormat="1"/>
+    <row r="249" s="31" customFormat="1"/>
+    <row r="250" s="31" customFormat="1"/>
+    <row r="251" s="31" customFormat="1"/>
+    <row r="252" s="31" customFormat="1"/>
+    <row r="253" s="31" customFormat="1"/>
+    <row r="254" s="31" customFormat="1"/>
+    <row r="255" s="31" customFormat="1"/>
+    <row r="256" s="31" customFormat="1"/>
+    <row r="257" s="31" customFormat="1"/>
+    <row r="258" s="31" customFormat="1"/>
+    <row r="259" s="31" customFormat="1"/>
+    <row r="260" s="31" customFormat="1"/>
+    <row r="261" s="31" customFormat="1"/>
+    <row r="262" s="31" customFormat="1"/>
+    <row r="263" s="31" customFormat="1"/>
+    <row r="264" s="31" customFormat="1"/>
+    <row r="265" s="31" customFormat="1"/>
+    <row r="266" s="31" customFormat="1"/>
+    <row r="267" s="31" customFormat="1"/>
+    <row r="268" s="31" customFormat="1"/>
+    <row r="269" s="31" customFormat="1"/>
+    <row r="270" s="31" customFormat="1"/>
+    <row r="271" s="31" customFormat="1"/>
+    <row r="272" s="31" customFormat="1"/>
+    <row r="273" s="31" customFormat="1"/>
+    <row r="274" s="31" customFormat="1"/>
+    <row r="275" s="31" customFormat="1"/>
+    <row r="276" s="31" customFormat="1"/>
+    <row r="277" s="31" customFormat="1"/>
+    <row r="278" s="31" customFormat="1"/>
+    <row r="279" s="31" customFormat="1"/>
+    <row r="280" s="31" customFormat="1"/>
+    <row r="281" s="31" customFormat="1"/>
+    <row r="282" s="31" customFormat="1"/>
+    <row r="283" s="31" customFormat="1"/>
+    <row r="284" s="31" customFormat="1"/>
+    <row r="285" s="31" customFormat="1"/>
+    <row r="286" s="31" customFormat="1"/>
+    <row r="287" s="31" customFormat="1"/>
+    <row r="288" s="31" customFormat="1"/>
+    <row r="289" s="31" customFormat="1"/>
+    <row r="290" s="31" customFormat="1"/>
+    <row r="291" s="31" customFormat="1"/>
+    <row r="292" s="31" customFormat="1"/>
+    <row r="293" s="31" customFormat="1"/>
+    <row r="294" s="31" customFormat="1"/>
+    <row r="295" s="31" customFormat="1"/>
+    <row r="296" s="31" customFormat="1"/>
+    <row r="297" s="31" customFormat="1"/>
+    <row r="298" s="31" customFormat="1"/>
+    <row r="299" s="31" customFormat="1"/>
+    <row r="300" s="31" customFormat="1"/>
+    <row r="301" s="31" customFormat="1"/>
+    <row r="302" s="31" customFormat="1"/>
+    <row r="303" s="31" customFormat="1"/>
+    <row r="304" s="31" customFormat="1"/>
+    <row r="305" s="31" customFormat="1"/>
+    <row r="306" s="31" customFormat="1"/>
+    <row r="307" s="31" customFormat="1"/>
+    <row r="308" s="31" customFormat="1"/>
+    <row r="309" s="31" customFormat="1"/>
+    <row r="310" s="31" customFormat="1"/>
+    <row r="311" s="31" customFormat="1"/>
+    <row r="312" s="31" customFormat="1"/>
+    <row r="313" s="31" customFormat="1"/>
+    <row r="314" s="31" customFormat="1"/>
+    <row r="315" s="31" customFormat="1"/>
+    <row r="316" s="31" customFormat="1"/>
+    <row r="317" s="31" customFormat="1"/>
+    <row r="318" s="31" customFormat="1"/>
+    <row r="319" s="31" customFormat="1"/>
+    <row r="320" s="31" customFormat="1"/>
+    <row r="321" s="31" customFormat="1"/>
+    <row r="322" s="31" customFormat="1"/>
+    <row r="323" s="31" customFormat="1"/>
+    <row r="324" s="31" customFormat="1"/>
+    <row r="325" s="31" customFormat="1"/>
+    <row r="326" s="31" customFormat="1"/>
+    <row r="327" s="31" customFormat="1"/>
+    <row r="328" s="31" customFormat="1"/>
+    <row r="329" s="31" customFormat="1"/>
+    <row r="330" s="31" customFormat="1"/>
+    <row r="331" s="31" customFormat="1"/>
+    <row r="332" s="31" customFormat="1"/>
+    <row r="333" s="31" customFormat="1"/>
+    <row r="334" s="31" customFormat="1"/>
+    <row r="335" s="31" customFormat="1"/>
+    <row r="336" s="31" customFormat="1"/>
+    <row r="337" s="31" customFormat="1"/>
+    <row r="338" s="31" customFormat="1"/>
+    <row r="339" s="31" customFormat="1"/>
+    <row r="340" s="31" customFormat="1"/>
+    <row r="341" s="31" customFormat="1"/>
+    <row r="342" s="31" customFormat="1"/>
+    <row r="343" s="31" customFormat="1"/>
+    <row r="344" s="31" customFormat="1"/>
+    <row r="345" s="31" customFormat="1"/>
+    <row r="346" s="31" customFormat="1"/>
+    <row r="347" s="31" customFormat="1"/>
+    <row r="348" s="31" customFormat="1"/>
   </sheetData>
   <mergeCells count="111">
     <mergeCell ref="DF1:DH1"/>
@@ -11145,108 +11131,108 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D65A848-DDAF-4F6A-8445-D8E58599F91D}">
   <dimension ref="A1:AM197"/>
-  <sheetFormatPr defaultColWidth="12" defaultRowHeight="23.6" thickTop="1" thickBottom="1" x14ac:dyDescent="0.95"/>
+  <sheetFormatPr defaultColWidth="12" defaultRowHeight="15" thickTop="1" thickBottom="1"/>
   <cols>
-    <col min="1" max="2" width="8.1328125" style="14" customWidth="1"/>
-    <col min="3" max="3" width="6.73046875" style="14" customWidth="1"/>
-    <col min="4" max="4" width="9.19921875" style="14" customWidth="1"/>
-    <col min="5" max="5" width="12.19921875" style="14" customWidth="1"/>
+    <col min="1" max="2" width="8.15234375" style="14" customWidth="1"/>
+    <col min="3" max="3" width="6.69140625" style="14" customWidth="1"/>
+    <col min="4" max="4" width="9.23046875" style="14" customWidth="1"/>
+    <col min="5" max="5" width="12.23046875" style="14" customWidth="1"/>
     <col min="6" max="8" width="12" style="14"/>
     <col min="9" max="9" width="12" style="25"/>
     <col min="10" max="12" width="12" style="14"/>
     <col min="13" max="13" width="12" style="20"/>
     <col min="14" max="15" width="12" style="14"/>
-    <col min="16" max="18" width="20.19921875" style="14" customWidth="1"/>
-    <col min="19" max="19" width="14.6640625" style="14" customWidth="1"/>
+    <col min="16" max="18" width="20.23046875" style="14" customWidth="1"/>
+    <col min="19" max="19" width="14.69140625" style="14" customWidth="1"/>
     <col min="20" max="20" width="12" style="14"/>
-    <col min="21" max="21" width="20.19921875" style="20" customWidth="1"/>
-    <col min="22" max="22" width="18.1328125" style="14" customWidth="1"/>
-    <col min="23" max="23" width="20.19921875" style="14" customWidth="1"/>
-    <col min="24" max="24" width="19.46484375" style="26" customWidth="1"/>
-    <col min="25" max="26" width="18.3984375" style="14" customWidth="1"/>
-    <col min="27" max="27" width="26.1328125" style="14" customWidth="1"/>
+    <col min="21" max="21" width="20.23046875" style="20" customWidth="1"/>
+    <col min="22" max="22" width="18.15234375" style="14" customWidth="1"/>
+    <col min="23" max="23" width="20.23046875" style="14" customWidth="1"/>
+    <col min="24" max="24" width="19.4609375" style="26" customWidth="1"/>
+    <col min="25" max="26" width="18.3828125" style="14" customWidth="1"/>
+    <col min="27" max="27" width="26.15234375" style="14" customWidth="1"/>
     <col min="28" max="28" width="25" style="14" customWidth="1"/>
     <col min="29" max="30" width="12" style="14"/>
     <col min="31" max="39" width="12" style="15"/>
     <col min="40" max="16384" width="12" style="14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:39" s="1" customFormat="1" ht="72" customHeight="1" thickBot="1" x14ac:dyDescent="0.95">
-      <c r="A1" s="42" t="s">
+    <row r="1" spans="1:39" s="1" customFormat="1" ht="72" customHeight="1" thickBot="1">
+      <c r="A1" s="46" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="42" t="s">
+      <c r="B1" s="46" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="42" t="s">
+      <c r="C1" s="46" t="s">
+        <v>102</v>
+      </c>
+      <c r="D1" s="46" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" s="46" t="s">
         <v>103</v>
       </c>
-      <c r="D1" s="42" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1" s="42" t="s">
-        <v>104</v>
-      </c>
-      <c r="F1" s="42" t="s">
+      <c r="F1" s="46" t="s">
         <v>10</v>
       </c>
-      <c r="G1" s="42" t="s">
+      <c r="G1" s="46" t="s">
         <v>11</v>
       </c>
-      <c r="H1" s="42" t="s">
+      <c r="H1" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="I1" s="46" t="s">
+      <c r="I1" s="50" t="s">
         <v>13</v>
       </c>
-      <c r="J1" s="42" t="s">
+      <c r="J1" s="46" t="s">
         <v>14</v>
       </c>
-      <c r="K1" s="42" t="s">
+      <c r="K1" s="46" t="s">
         <v>15</v>
       </c>
-      <c r="L1" s="44" t="s">
+      <c r="L1" s="48" t="s">
+        <v>25</v>
+      </c>
+      <c r="M1" s="46" t="s">
         <v>16</v>
       </c>
-      <c r="M1" s="42" t="s">
+      <c r="N1" s="46" t="s">
         <v>17</v>
       </c>
-      <c r="N1" s="42" t="s">
+      <c r="O1" s="46" t="s">
         <v>18</v>
       </c>
-      <c r="O1" s="42" t="s">
+      <c r="P1" s="57" t="s">
         <v>19</v>
       </c>
-      <c r="P1" s="53" t="s">
+      <c r="Q1" s="58"/>
+      <c r="R1" s="59"/>
+      <c r="S1" s="52" t="s">
         <v>20</v>
       </c>
-      <c r="Q1" s="54"/>
-      <c r="R1" s="55"/>
-      <c r="S1" s="48" t="s">
+      <c r="T1" s="53"/>
+      <c r="U1" s="52" t="s">
         <v>21</v>
       </c>
-      <c r="T1" s="49"/>
-      <c r="U1" s="48" t="s">
+      <c r="V1" s="54"/>
+      <c r="W1" s="55" t="s">
         <v>22</v>
       </c>
-      <c r="V1" s="50"/>
-      <c r="W1" s="51" t="s">
+      <c r="X1" s="46" t="s">
+        <v>109</v>
+      </c>
+      <c r="Y1" s="46" t="s">
+        <v>107</v>
+      </c>
+      <c r="Z1" s="55" t="s">
+        <v>108</v>
+      </c>
+      <c r="AA1" s="46" t="s">
         <v>23</v>
       </c>
-      <c r="X1" s="42" t="s">
-        <v>110</v>
-      </c>
-      <c r="Y1" s="42" t="s">
-        <v>108</v>
-      </c>
-      <c r="Z1" s="51" t="s">
-        <v>109</v>
-      </c>
-      <c r="AA1" s="42" t="s">
+      <c r="AB1" s="46" t="s">
         <v>24</v>
-      </c>
-      <c r="AB1" s="42" t="s">
-        <v>25</v>
       </c>
       <c r="AE1" s="2"/>
       <c r="AF1" s="2"/>
@@ -11258,57 +11244,57 @@
       <c r="AL1" s="2"/>
       <c r="AM1" s="2"/>
     </row>
-    <row r="2" spans="1:39" s="1" customFormat="1" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.95">
-      <c r="A2" s="43"/>
-      <c r="B2" s="43"/>
-      <c r="C2" s="43"/>
-      <c r="D2" s="43"/>
-      <c r="E2" s="43"/>
-      <c r="F2" s="43"/>
-      <c r="G2" s="43"/>
-      <c r="H2" s="43"/>
-      <c r="I2" s="47" t="s">
+    <row r="2" spans="1:39" s="1" customFormat="1" ht="48" customHeight="1" thickBot="1">
+      <c r="A2" s="47"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
+      <c r="I2" s="51" t="s">
         <v>13</v>
       </c>
-      <c r="J2" s="43" t="s">
+      <c r="J2" s="47" t="s">
         <v>14</v>
       </c>
-      <c r="K2" s="43" t="s">
+      <c r="K2" s="47" t="s">
         <v>15</v>
       </c>
-      <c r="L2" s="45" t="s">
+      <c r="L2" s="49" t="s">
+        <v>25</v>
+      </c>
+      <c r="M2" s="47"/>
+      <c r="N2" s="47"/>
+      <c r="O2" s="47"/>
+      <c r="P2" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="S2" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="M2" s="43"/>
-      <c r="N2" s="43"/>
-      <c r="O2" s="43"/>
-      <c r="P2" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="Q2" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="R2" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="S2" s="4" t="s">
+      <c r="T2" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="T2" s="4" t="s">
-        <v>28</v>
-      </c>
       <c r="U2" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="V2" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="V2" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="W2" s="52"/>
-      <c r="X2" s="43"/>
-      <c r="Y2" s="43"/>
-      <c r="Z2" s="52"/>
-      <c r="AA2" s="43"/>
-      <c r="AB2" s="43"/>
+      <c r="W2" s="56"/>
+      <c r="X2" s="47"/>
+      <c r="Y2" s="47"/>
+      <c r="Z2" s="56"/>
+      <c r="AA2" s="47"/>
+      <c r="AB2" s="47"/>
       <c r="AE2" s="2"/>
       <c r="AF2" s="2"/>
       <c r="AG2" s="2"/>
@@ -11319,7 +11305,7 @@
       <c r="AL2" s="2"/>
       <c r="AM2" s="2"/>
     </row>
-    <row r="3" spans="1:39" s="1" customFormat="1" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.95">
+    <row r="3" spans="1:39" s="1" customFormat="1" ht="42" customHeight="1" thickBot="1">
       <c r="A3" s="5">
         <v>1369</v>
       </c>
@@ -11397,10 +11383,10 @@
         <v>7500</v>
       </c>
       <c r="AA3" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="AB3" s="11" t="s">
         <v>29</v>
-      </c>
-      <c r="AB3" s="11" t="s">
-        <v>30</v>
       </c>
       <c r="AE3" s="2"/>
       <c r="AF3" s="2"/>
@@ -11412,7 +11398,7 @@
       <c r="AL3" s="2"/>
       <c r="AM3" s="2"/>
     </row>
-    <row r="4" spans="1:39" s="1" customFormat="1" ht="38.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
+    <row r="4" spans="1:39" s="1" customFormat="1" ht="38.25" customHeight="1" thickTop="1" thickBot="1">
       <c r="A4" s="5">
         <v>1370</v>
       </c>
@@ -11490,10 +11476,10 @@
         <v>12503</v>
       </c>
       <c r="AA4" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB4" s="13" t="s">
         <v>31</v>
-      </c>
-      <c r="AB4" s="13" t="s">
-        <v>32</v>
       </c>
       <c r="AE4" s="2"/>
       <c r="AF4" s="2"/>
@@ -11505,7 +11491,7 @@
       <c r="AL4" s="2"/>
       <c r="AM4" s="2"/>
     </row>
-    <row r="5" spans="1:39" s="1" customFormat="1" ht="38.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
+    <row r="5" spans="1:39" s="1" customFormat="1" ht="38.25" customHeight="1" thickTop="1" thickBot="1">
       <c r="A5" s="5">
         <v>1371</v>
       </c>
@@ -11583,10 +11569,10 @@
         <v>17003</v>
       </c>
       <c r="AA5" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="AB5" s="13" t="s">
         <v>33</v>
-      </c>
-      <c r="AB5" s="13" t="s">
-        <v>34</v>
       </c>
       <c r="AE5" s="2"/>
       <c r="AF5" s="2"/>
@@ -11598,7 +11584,7 @@
       <c r="AL5" s="2"/>
       <c r="AM5" s="2"/>
     </row>
-    <row r="6" spans="1:39" s="1" customFormat="1" ht="38.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
+    <row r="6" spans="1:39" s="1" customFormat="1" ht="38.25" customHeight="1" thickTop="1" thickBot="1">
       <c r="A6" s="5">
         <v>1372</v>
       </c>
@@ -11676,10 +11662,10 @@
         <v>22455</v>
       </c>
       <c r="AA6" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB6" s="13" t="s">
         <v>35</v>
-      </c>
-      <c r="AB6" s="13" t="s">
-        <v>36</v>
       </c>
       <c r="AE6" s="2"/>
       <c r="AF6" s="2"/>
@@ -11691,7 +11677,7 @@
       <c r="AL6" s="2"/>
       <c r="AM6" s="2"/>
     </row>
-    <row r="7" spans="1:39" s="1" customFormat="1" ht="38.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
+    <row r="7" spans="1:39" s="1" customFormat="1" ht="38.25" customHeight="1" thickTop="1" thickBot="1">
       <c r="A7" s="5">
         <v>1373</v>
       </c>
@@ -11769,10 +11755,10 @@
         <v>29205</v>
       </c>
       <c r="AA7" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="AB7" s="13" t="s">
         <v>37</v>
-      </c>
-      <c r="AB7" s="13" t="s">
-        <v>38</v>
       </c>
       <c r="AE7" s="2"/>
       <c r="AF7" s="2"/>
@@ -11784,7 +11770,7 @@
       <c r="AL7" s="2"/>
       <c r="AM7" s="2"/>
     </row>
-    <row r="8" spans="1:39" s="1" customFormat="1" ht="38.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
+    <row r="8" spans="1:39" s="1" customFormat="1" ht="38.25" customHeight="1" thickTop="1" thickBot="1">
       <c r="A8" s="5">
         <v>1374</v>
       </c>
@@ -11862,10 +11848,10 @@
         <v>39998</v>
       </c>
       <c r="AA8" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB8" s="13" t="s">
         <v>39</v>
-      </c>
-      <c r="AB8" s="13" t="s">
-        <v>40</v>
       </c>
       <c r="AE8" s="2"/>
       <c r="AF8" s="2"/>
@@ -11877,7 +11863,7 @@
       <c r="AL8" s="2"/>
       <c r="AM8" s="2"/>
     </row>
-    <row r="9" spans="1:39" s="1" customFormat="1" ht="38.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
+    <row r="9" spans="1:39" s="1" customFormat="1" ht="38.25" customHeight="1" thickTop="1" thickBot="1">
       <c r="A9" s="5">
         <v>1375</v>
       </c>
@@ -11955,10 +11941,10 @@
         <v>51803</v>
       </c>
       <c r="AA9" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="AB9" s="13" t="s">
         <v>41</v>
-      </c>
-      <c r="AB9" s="13" t="s">
-        <v>42</v>
       </c>
       <c r="AE9" s="2"/>
       <c r="AF9" s="2"/>
@@ -11970,7 +11956,7 @@
       <c r="AL9" s="2"/>
       <c r="AM9" s="2"/>
     </row>
-    <row r="10" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
+    <row r="10" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
       <c r="A10" s="5">
         <v>1376</v>
       </c>
@@ -12048,13 +12034,13 @@
         <v>63615</v>
       </c>
       <c r="AA10" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="AB10" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="AB10" s="13" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="11" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
+    </row>
+    <row r="11" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
       <c r="A11" s="5">
         <v>1377</v>
       </c>
@@ -12132,13 +12118,13 @@
         <v>75383</v>
       </c>
       <c r="AA11" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="AB11" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="AB11" s="13" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="12" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
+    </row>
+    <row r="12" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
       <c r="A12" s="5">
         <v>1378</v>
       </c>
@@ -12216,13 +12202,13 @@
         <v>90458</v>
       </c>
       <c r="AA12" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="AB12" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="AB12" s="13" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="13" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
+    </row>
+    <row r="13" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
       <c r="A13" s="5">
         <v>1379</v>
       </c>
@@ -12300,13 +12286,13 @@
         <v>114503</v>
       </c>
       <c r="AA13" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB13" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="AB13" s="13" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="14" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
+    </row>
+    <row r="14" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
       <c r="A14" s="5">
         <v>1380</v>
       </c>
@@ -12384,13 +12370,13 @@
         <v>141975</v>
       </c>
       <c r="AA14" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="AB14" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="AB14" s="13" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="15" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
+    </row>
+    <row r="15" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
       <c r="A15" s="5">
         <v>1381</v>
       </c>
@@ -12468,13 +12454,13 @@
         <v>174615</v>
       </c>
       <c r="AA15" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="AB15" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="AB15" s="13" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="16" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
+    </row>
+    <row r="16" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
       <c r="A16" s="5">
         <v>1382</v>
       </c>
@@ -12552,13 +12538,13 @@
         <v>213345</v>
       </c>
       <c r="AA16" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="AB16" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="AB16" s="13" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="17" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
+    </row>
+    <row r="17" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
       <c r="A17" s="5">
         <v>1383</v>
       </c>
@@ -12636,13 +12622,13 @@
         <v>266505</v>
       </c>
       <c r="AA17" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="AB17" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="AB17" s="13" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="18" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
+    </row>
+    <row r="18" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
       <c r="A18" s="5">
         <v>1384</v>
       </c>
@@ -12720,13 +12706,13 @@
         <v>306480</v>
       </c>
       <c r="AA18" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="AB18" s="13" t="s">
         <v>59</v>
       </c>
-      <c r="AB18" s="13" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="19" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
+    </row>
+    <row r="19" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
       <c r="A19" s="5">
         <v>1385</v>
       </c>
@@ -12804,13 +12790,13 @@
         <v>375000</v>
       </c>
       <c r="AA19" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="AB19" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="AB19" s="13" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="20" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
+    </row>
+    <row r="20" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
       <c r="A20" s="5">
         <v>1386</v>
       </c>
@@ -12888,13 +12874,13 @@
         <v>457500</v>
       </c>
       <c r="AA20" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="AB20" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="AB20" s="13" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="21" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
+    </row>
+    <row r="21" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
       <c r="A21" s="5">
         <v>1387</v>
       </c>
@@ -12972,13 +12958,13 @@
         <v>549000</v>
       </c>
       <c r="AA21" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="AB21" s="13" t="s">
         <v>65</v>
       </c>
-      <c r="AB21" s="13" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="22" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
+    </row>
+    <row r="22" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
       <c r="A22" s="5">
         <v>1388</v>
       </c>
@@ -13056,13 +13042,13 @@
         <v>658800</v>
       </c>
       <c r="AA22" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="AB22" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="AB22" s="13" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="23" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
+    </row>
+    <row r="23" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
       <c r="A23" s="5">
         <v>1389</v>
       </c>
@@ -13140,13 +13126,13 @@
         <v>757500</v>
       </c>
       <c r="AA23" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="AB23" s="13" t="s">
         <v>69</v>
       </c>
-      <c r="AB23" s="13" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="24" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
+    </row>
+    <row r="24" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
       <c r="A24" s="5">
         <v>1390</v>
       </c>
@@ -13224,13 +13210,13 @@
         <v>825750</v>
       </c>
       <c r="AA24" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="AB24" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="AB24" s="13" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="25" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
+    </row>
+    <row r="25" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
       <c r="A25" s="5">
         <v>1391</v>
       </c>
@@ -13308,14 +13294,14 @@
         <v>974250</v>
       </c>
       <c r="AA25" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="AB25" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="AB25" s="13" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="26" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
-      <c r="A26" s="56">
+    </row>
+    <row r="26" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A26" s="60">
         <v>1392</v>
       </c>
       <c r="B26" s="6">
@@ -13392,14 +13378,14 @@
         <v>1217813</v>
       </c>
       <c r="AA26" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="AB26" s="60" t="s">
         <v>75</v>
       </c>
-      <c r="AB26" s="56" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="27" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
-      <c r="A27" s="57"/>
+    </row>
+    <row r="27" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A27" s="61"/>
       <c r="B27" s="6">
         <v>8</v>
       </c>
@@ -13474,11 +13460,11 @@
         <v>1217813</v>
       </c>
       <c r="AA27" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="AB27" s="57"/>
-    </row>
-    <row r="28" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
+        <v>74</v>
+      </c>
+      <c r="AB27" s="61"/>
+    </row>
+    <row r="28" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
       <c r="A28" s="5">
         <v>1393</v>
       </c>
@@ -13556,13 +13542,13 @@
         <v>1522275</v>
       </c>
       <c r="AA28" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="AB28" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="AB28" s="13" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="29" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
+    </row>
+    <row r="29" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
       <c r="A29" s="5">
         <v>1394</v>
       </c>
@@ -13640,14 +13626,14 @@
         <v>1781063</v>
       </c>
       <c r="AA29" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="AB29" s="13" t="s">
         <v>79</v>
       </c>
-      <c r="AB29" s="13" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="30" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
-      <c r="A30" s="58">
+    </row>
+    <row r="30" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A30" s="62">
         <v>1395</v>
       </c>
       <c r="B30" s="6">
@@ -13724,14 +13710,14 @@
         <v>2030415</v>
       </c>
       <c r="AA30" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="AB30" s="64" t="s">
         <v>81</v>
       </c>
-      <c r="AB30" s="60" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="31" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
-      <c r="A31" s="59"/>
+    </row>
+    <row r="31" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A31" s="63"/>
       <c r="B31" s="6">
         <v>6</v>
       </c>
@@ -13806,11 +13792,11 @@
         <v>2030415</v>
       </c>
       <c r="AA31" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="AB31" s="61"/>
-    </row>
-    <row r="32" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
+        <v>80</v>
+      </c>
+      <c r="AB31" s="65"/>
+    </row>
+    <row r="32" spans="1:28" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
       <c r="A32" s="5">
         <v>1396</v>
       </c>
@@ -13888,13 +13874,13 @@
         <v>2324828</v>
       </c>
       <c r="AA32" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="AB32" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="AB32" s="13" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="33" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
+    </row>
+    <row r="33" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
       <c r="A33" s="5">
         <v>1397</v>
       </c>
@@ -13972,13 +13958,13 @@
         <v>2778173</v>
       </c>
       <c r="AA33" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="AB33" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="AB33" s="13" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="34" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
+    </row>
+    <row r="34" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
       <c r="A34" s="5">
         <v>1398</v>
       </c>
@@ -14056,14 +14042,14 @@
         <v>3792203</v>
       </c>
       <c r="AA34" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="AB34" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="AB34" s="13" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="35" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
-      <c r="A35" s="62">
+    </row>
+    <row r="35" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A35" s="66">
         <v>1399</v>
       </c>
       <c r="B35" s="6">
@@ -14094,7 +14080,7 @@
         <v>187621</v>
       </c>
       <c r="K35" s="20">
-        <v>33333</v>
+        <v>58333</v>
       </c>
       <c r="L35" s="21">
         <v>220957</v>
@@ -14140,14 +14126,14 @@
         <v>4588568</v>
       </c>
       <c r="AA35" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="AB35" s="68" t="s">
         <v>89</v>
       </c>
-      <c r="AB35" s="64" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="36" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
-      <c r="A36" s="63"/>
+    </row>
+    <row r="36" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A36" s="67"/>
       <c r="B36" s="6">
         <v>9</v>
       </c>
@@ -14222,11 +14208,11 @@
         <v>4776068</v>
       </c>
       <c r="AA36" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="AB36" s="61"/>
-    </row>
-    <row r="37" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
+        <v>90</v>
+      </c>
+      <c r="AB36" s="65"/>
+    </row>
+    <row r="37" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
       <c r="A37" s="5">
         <v>1400</v>
       </c>
@@ -14304,13 +14290,13 @@
         <v>6638738</v>
       </c>
       <c r="AA37" s="12" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="AB37" s="13" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="38" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="38" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
       <c r="A38" s="5">
         <v>1401</v>
       </c>
@@ -14388,13 +14374,13 @@
         <v>10449375</v>
       </c>
       <c r="AA38" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="AB38" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="AB38" s="13" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="39" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
+    </row>
+    <row r="39" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
       <c r="A39" s="5">
         <v>1402</v>
       </c>
@@ -14472,13 +14458,13 @@
         <v>13270710</v>
       </c>
       <c r="AA39" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="AB39" s="13" t="s">
         <v>95</v>
       </c>
-      <c r="AB39" s="13" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="40" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
+    </row>
+    <row r="40" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
       <c r="A40" s="5">
         <v>1403</v>
       </c>
@@ -14558,13 +14544,13 @@
         <v>17915460</v>
       </c>
       <c r="AA40" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="AB40" s="13" t="s">
         <v>97</v>
       </c>
-      <c r="AB40" s="13" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="41" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
+    </row>
+    <row r="41" spans="1:39" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
       <c r="A41" s="5">
         <v>1404</v>
       </c>
@@ -14644,13 +14630,13 @@
         <v>25977420</v>
       </c>
       <c r="AA41" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="AB41" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="AB41" s="13" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="42" spans="1:39" s="24" customFormat="1" ht="45.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.95">
+    </row>
+    <row r="42" spans="1:39" s="24" customFormat="1" ht="45.75" customHeight="1" thickTop="1" thickBot="1">
       <c r="A42" s="5">
         <v>1405</v>
       </c>
@@ -14730,10 +14716,10 @@
         <v>41563875</v>
       </c>
       <c r="AA42" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="AB42" s="12" t="s">
         <v>101</v>
-      </c>
-      <c r="AB42" s="12" t="s">
-        <v>102</v>
       </c>
       <c r="AC42" s="22"/>
       <c r="AD42" s="22"/>
@@ -14747,7 +14733,7 @@
       <c r="AL42" s="23"/>
       <c r="AM42" s="23"/>
     </row>
-    <row r="43" spans="1:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="43" spans="1:39" ht="13.8">
       <c r="M43" s="14"/>
       <c r="S43" s="15"/>
       <c r="T43" s="15"/>
@@ -14767,7 +14753,7 @@
       <c r="AL43" s="14"/>
       <c r="AM43" s="14"/>
     </row>
-    <row r="44" spans="1:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="44" spans="1:39" ht="13.8">
       <c r="M44" s="14"/>
       <c r="S44" s="15"/>
       <c r="T44" s="15"/>
@@ -14787,7 +14773,7 @@
       <c r="AL44" s="14"/>
       <c r="AM44" s="14"/>
     </row>
-    <row r="45" spans="1:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="45" spans="1:39" ht="13.8">
       <c r="M45" s="14"/>
       <c r="S45" s="15"/>
       <c r="T45" s="15"/>
@@ -14807,7 +14793,7 @@
       <c r="AL45" s="14"/>
       <c r="AM45" s="14"/>
     </row>
-    <row r="46" spans="1:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="46" spans="1:39" ht="13.8">
       <c r="M46" s="14"/>
       <c r="S46" s="15"/>
       <c r="T46" s="15"/>
@@ -14827,7 +14813,7 @@
       <c r="AL46" s="14"/>
       <c r="AM46" s="14"/>
     </row>
-    <row r="47" spans="1:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="47" spans="1:39" ht="13.8">
       <c r="M47" s="14"/>
       <c r="S47" s="15"/>
       <c r="T47" s="15"/>
@@ -14847,7 +14833,7 @@
       <c r="AL47" s="14"/>
       <c r="AM47" s="14"/>
     </row>
-    <row r="48" spans="1:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="48" spans="1:39" ht="13.8">
       <c r="M48" s="14"/>
       <c r="S48" s="15"/>
       <c r="T48" s="15"/>
@@ -14867,7 +14853,7 @@
       <c r="AL48" s="14"/>
       <c r="AM48" s="14"/>
     </row>
-    <row r="49" spans="13:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="49" spans="13:39" ht="13.8">
       <c r="M49" s="14"/>
       <c r="S49" s="15"/>
       <c r="T49" s="15"/>
@@ -14887,7 +14873,7 @@
       <c r="AL49" s="14"/>
       <c r="AM49" s="14"/>
     </row>
-    <row r="50" spans="13:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="50" spans="13:39" ht="13.8">
       <c r="M50" s="14"/>
       <c r="S50" s="15"/>
       <c r="T50" s="15"/>
@@ -14905,7 +14891,7 @@
       <c r="AL50" s="14"/>
       <c r="AM50" s="14"/>
     </row>
-    <row r="51" spans="13:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="51" spans="13:39" ht="13.8">
       <c r="M51" s="14"/>
       <c r="S51" s="15"/>
       <c r="T51" s="15"/>
@@ -14925,7 +14911,7 @@
       <c r="AL51" s="14"/>
       <c r="AM51" s="14"/>
     </row>
-    <row r="52" spans="13:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="52" spans="13:39" ht="13.8">
       <c r="M52" s="14"/>
       <c r="S52" s="15"/>
       <c r="T52" s="15"/>
@@ -14945,7 +14931,7 @@
       <c r="AL52" s="14"/>
       <c r="AM52" s="14"/>
     </row>
-    <row r="53" spans="13:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="53" spans="13:39" ht="13.8">
       <c r="M53" s="14"/>
       <c r="S53" s="15"/>
       <c r="T53" s="15"/>
@@ -14965,7 +14951,7 @@
       <c r="AL53" s="14"/>
       <c r="AM53" s="14"/>
     </row>
-    <row r="54" spans="13:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="54" spans="13:39" ht="13.8">
       <c r="M54" s="14"/>
       <c r="S54" s="15"/>
       <c r="T54" s="15"/>
@@ -14985,7 +14971,7 @@
       <c r="AL54" s="14"/>
       <c r="AM54" s="14"/>
     </row>
-    <row r="55" spans="13:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="55" spans="13:39" ht="13.8">
       <c r="M55" s="14"/>
       <c r="S55" s="15"/>
       <c r="T55" s="15"/>
@@ -15005,7 +14991,7 @@
       <c r="AL55" s="14"/>
       <c r="AM55" s="14"/>
     </row>
-    <row r="56" spans="13:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="56" spans="13:39" ht="13.8">
       <c r="M56" s="14"/>
       <c r="S56" s="15"/>
       <c r="T56" s="15"/>
@@ -15025,7 +15011,7 @@
       <c r="AL56" s="14"/>
       <c r="AM56" s="14"/>
     </row>
-    <row r="57" spans="13:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="57" spans="13:39" ht="13.8">
       <c r="M57" s="14"/>
       <c r="S57" s="15"/>
       <c r="T57" s="15"/>
@@ -15045,7 +15031,7 @@
       <c r="AL57" s="14"/>
       <c r="AM57" s="14"/>
     </row>
-    <row r="58" spans="13:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="58" spans="13:39" ht="13.8">
       <c r="M58" s="14"/>
       <c r="S58" s="15"/>
       <c r="T58" s="15"/>
@@ -15065,7 +15051,7 @@
       <c r="AL58" s="14"/>
       <c r="AM58" s="14"/>
     </row>
-    <row r="59" spans="13:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="59" spans="13:39" ht="13.8">
       <c r="M59" s="14"/>
       <c r="S59" s="15"/>
       <c r="T59" s="15"/>
@@ -15085,7 +15071,7 @@
       <c r="AL59" s="14"/>
       <c r="AM59" s="14"/>
     </row>
-    <row r="60" spans="13:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="60" spans="13:39" ht="13.8">
       <c r="M60" s="14"/>
       <c r="S60" s="15"/>
       <c r="T60" s="15"/>
@@ -15105,7 +15091,7 @@
       <c r="AL60" s="14"/>
       <c r="AM60" s="14"/>
     </row>
-    <row r="61" spans="13:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="61" spans="13:39" ht="13.8">
       <c r="M61" s="14"/>
       <c r="S61" s="15"/>
       <c r="T61" s="15"/>
@@ -15125,7 +15111,7 @@
       <c r="AL61" s="14"/>
       <c r="AM61" s="14"/>
     </row>
-    <row r="62" spans="13:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="62" spans="13:39" ht="13.8">
       <c r="S62" s="15"/>
       <c r="T62" s="15"/>
       <c r="U62" s="15"/>
@@ -15144,7 +15130,7 @@
       <c r="AL62" s="14"/>
       <c r="AM62" s="14"/>
     </row>
-    <row r="63" spans="13:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="63" spans="13:39" ht="13.8">
       <c r="S63" s="15"/>
       <c r="T63" s="15"/>
       <c r="U63" s="15"/>
@@ -15163,7 +15149,7 @@
       <c r="AL63" s="14"/>
       <c r="AM63" s="14"/>
     </row>
-    <row r="64" spans="13:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="64" spans="13:39" ht="13.8">
       <c r="S64" s="15"/>
       <c r="T64" s="15"/>
       <c r="U64" s="15"/>
@@ -15182,7 +15168,7 @@
       <c r="AL64" s="14"/>
       <c r="AM64" s="14"/>
     </row>
-    <row r="65" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="65" spans="19:39" ht="13.8">
       <c r="S65" s="15"/>
       <c r="T65" s="15"/>
       <c r="U65" s="15"/>
@@ -15201,7 +15187,7 @@
       <c r="AL65" s="14"/>
       <c r="AM65" s="14"/>
     </row>
-    <row r="66" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="66" spans="19:39" ht="13.8">
       <c r="S66" s="15"/>
       <c r="T66" s="15"/>
       <c r="U66" s="15"/>
@@ -15220,7 +15206,7 @@
       <c r="AL66" s="14"/>
       <c r="AM66" s="14"/>
     </row>
-    <row r="67" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="67" spans="19:39" ht="13.8">
       <c r="S67" s="15"/>
       <c r="T67" s="15"/>
       <c r="U67" s="15"/>
@@ -15239,7 +15225,7 @@
       <c r="AL67" s="14"/>
       <c r="AM67" s="14"/>
     </row>
-    <row r="68" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="68" spans="19:39" ht="13.8">
       <c r="S68" s="15"/>
       <c r="T68" s="15"/>
       <c r="U68" s="15"/>
@@ -15258,7 +15244,7 @@
       <c r="AL68" s="14"/>
       <c r="AM68" s="14"/>
     </row>
-    <row r="69" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="69" spans="19:39" ht="13.8">
       <c r="S69" s="15"/>
       <c r="T69" s="15"/>
       <c r="U69" s="15"/>
@@ -15277,7 +15263,7 @@
       <c r="AL69" s="14"/>
       <c r="AM69" s="14"/>
     </row>
-    <row r="70" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="70" spans="19:39" ht="13.8">
       <c r="S70" s="15"/>
       <c r="T70" s="15"/>
       <c r="U70" s="15"/>
@@ -15296,7 +15282,7 @@
       <c r="AL70" s="14"/>
       <c r="AM70" s="14"/>
     </row>
-    <row r="71" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="71" spans="19:39" ht="13.8">
       <c r="S71" s="15"/>
       <c r="T71" s="15"/>
       <c r="U71" s="15"/>
@@ -15315,7 +15301,7 @@
       <c r="AL71" s="14"/>
       <c r="AM71" s="14"/>
     </row>
-    <row r="72" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="72" spans="19:39" ht="13.8">
       <c r="S72" s="15"/>
       <c r="T72" s="15"/>
       <c r="U72" s="15"/>
@@ -15334,7 +15320,7 @@
       <c r="AL72" s="14"/>
       <c r="AM72" s="14"/>
     </row>
-    <row r="73" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="73" spans="19:39" ht="13.8">
       <c r="S73" s="15"/>
       <c r="T73" s="15"/>
       <c r="U73" s="15"/>
@@ -15353,7 +15339,7 @@
       <c r="AL73" s="14"/>
       <c r="AM73" s="14"/>
     </row>
-    <row r="74" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="74" spans="19:39" ht="13.8">
       <c r="S74" s="15"/>
       <c r="T74" s="15"/>
       <c r="U74" s="15"/>
@@ -15372,7 +15358,7 @@
       <c r="AL74" s="14"/>
       <c r="AM74" s="14"/>
     </row>
-    <row r="75" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="75" spans="19:39" ht="13.8">
       <c r="S75" s="15"/>
       <c r="T75" s="15"/>
       <c r="U75" s="15"/>
@@ -15391,7 +15377,7 @@
       <c r="AL75" s="14"/>
       <c r="AM75" s="14"/>
     </row>
-    <row r="76" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="76" spans="19:39" ht="13.8">
       <c r="S76" s="15"/>
       <c r="T76" s="15"/>
       <c r="U76" s="15"/>
@@ -15410,7 +15396,7 @@
       <c r="AL76" s="14"/>
       <c r="AM76" s="14"/>
     </row>
-    <row r="77" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="77" spans="19:39" ht="13.8">
       <c r="S77" s="15"/>
       <c r="T77" s="15"/>
       <c r="U77" s="15"/>
@@ -15429,7 +15415,7 @@
       <c r="AL77" s="14"/>
       <c r="AM77" s="14"/>
     </row>
-    <row r="78" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="78" spans="19:39" ht="13.8">
       <c r="S78" s="15"/>
       <c r="T78" s="15"/>
       <c r="U78" s="15"/>
@@ -15448,7 +15434,7 @@
       <c r="AL78" s="14"/>
       <c r="AM78" s="14"/>
     </row>
-    <row r="79" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="79" spans="19:39" ht="13.8">
       <c r="S79" s="15"/>
       <c r="T79" s="15"/>
       <c r="U79" s="15"/>
@@ -15467,7 +15453,7 @@
       <c r="AL79" s="14"/>
       <c r="AM79" s="14"/>
     </row>
-    <row r="80" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="80" spans="19:39" ht="13.8">
       <c r="S80" s="15"/>
       <c r="T80" s="15"/>
       <c r="U80" s="15"/>
@@ -15486,7 +15472,7 @@
       <c r="AL80" s="14"/>
       <c r="AM80" s="14"/>
     </row>
-    <row r="81" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="81" spans="19:39" ht="13.8">
       <c r="S81" s="15"/>
       <c r="T81" s="15"/>
       <c r="U81" s="15"/>
@@ -15505,7 +15491,7 @@
       <c r="AL81" s="14"/>
       <c r="AM81" s="14"/>
     </row>
-    <row r="82" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="82" spans="19:39" ht="13.8">
       <c r="S82" s="15"/>
       <c r="T82" s="15"/>
       <c r="U82" s="15"/>
@@ -15524,7 +15510,7 @@
       <c r="AL82" s="14"/>
       <c r="AM82" s="14"/>
     </row>
-    <row r="83" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="83" spans="19:39" ht="13.8">
       <c r="S83" s="15"/>
       <c r="T83" s="15"/>
       <c r="U83" s="15"/>
@@ -15543,7 +15529,7 @@
       <c r="AL83" s="14"/>
       <c r="AM83" s="14"/>
     </row>
-    <row r="84" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="84" spans="19:39" ht="13.8">
       <c r="S84" s="15"/>
       <c r="T84" s="15"/>
       <c r="U84" s="15"/>
@@ -15562,7 +15548,7 @@
       <c r="AL84" s="14"/>
       <c r="AM84" s="14"/>
     </row>
-    <row r="85" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="85" spans="19:39" ht="13.8">
       <c r="S85" s="15"/>
       <c r="T85" s="15"/>
       <c r="U85" s="15"/>
@@ -15581,7 +15567,7 @@
       <c r="AL85" s="14"/>
       <c r="AM85" s="14"/>
     </row>
-    <row r="86" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="86" spans="19:39" ht="13.8">
       <c r="S86" s="15"/>
       <c r="T86" s="15"/>
       <c r="U86" s="15"/>
@@ -15600,7 +15586,7 @@
       <c r="AL86" s="14"/>
       <c r="AM86" s="14"/>
     </row>
-    <row r="87" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="87" spans="19:39" ht="13.8">
       <c r="S87" s="15"/>
       <c r="T87" s="15"/>
       <c r="U87" s="15"/>
@@ -15619,7 +15605,7 @@
       <c r="AL87" s="14"/>
       <c r="AM87" s="14"/>
     </row>
-    <row r="88" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="88" spans="19:39" ht="13.8">
       <c r="S88" s="15"/>
       <c r="T88" s="15"/>
       <c r="U88" s="15"/>
@@ -15638,7 +15624,7 @@
       <c r="AL88" s="14"/>
       <c r="AM88" s="14"/>
     </row>
-    <row r="89" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="89" spans="19:39" ht="13.8">
       <c r="S89" s="15"/>
       <c r="T89" s="15"/>
       <c r="U89" s="15"/>
@@ -15657,7 +15643,7 @@
       <c r="AL89" s="14"/>
       <c r="AM89" s="14"/>
     </row>
-    <row r="90" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="90" spans="19:39" ht="13.8">
       <c r="S90" s="15"/>
       <c r="T90" s="15"/>
       <c r="U90" s="15"/>
@@ -15676,7 +15662,7 @@
       <c r="AL90" s="14"/>
       <c r="AM90" s="14"/>
     </row>
-    <row r="91" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="91" spans="19:39" ht="13.8">
       <c r="S91" s="15"/>
       <c r="T91" s="15"/>
       <c r="U91" s="15"/>
@@ -15695,7 +15681,7 @@
       <c r="AL91" s="14"/>
       <c r="AM91" s="14"/>
     </row>
-    <row r="92" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="92" spans="19:39" ht="13.8">
       <c r="S92" s="15"/>
       <c r="T92" s="15"/>
       <c r="U92" s="15"/>
@@ -15714,7 +15700,7 @@
       <c r="AL92" s="14"/>
       <c r="AM92" s="14"/>
     </row>
-    <row r="93" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="93" spans="19:39" ht="13.8">
       <c r="S93" s="15"/>
       <c r="T93" s="15"/>
       <c r="U93" s="15"/>
@@ -15733,7 +15719,7 @@
       <c r="AL93" s="14"/>
       <c r="AM93" s="14"/>
     </row>
-    <row r="94" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="94" spans="19:39" ht="13.8">
       <c r="S94" s="15"/>
       <c r="T94" s="15"/>
       <c r="U94" s="15"/>
@@ -15752,7 +15738,7 @@
       <c r="AL94" s="14"/>
       <c r="AM94" s="14"/>
     </row>
-    <row r="95" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="95" spans="19:39" ht="13.8">
       <c r="S95" s="15"/>
       <c r="T95" s="15"/>
       <c r="U95" s="15"/>
@@ -15771,7 +15757,7 @@
       <c r="AL95" s="14"/>
       <c r="AM95" s="14"/>
     </row>
-    <row r="96" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="96" spans="19:39" ht="13.8">
       <c r="S96" s="15"/>
       <c r="T96" s="15"/>
       <c r="U96" s="15"/>
@@ -15790,7 +15776,7 @@
       <c r="AL96" s="14"/>
       <c r="AM96" s="14"/>
     </row>
-    <row r="97" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="97" spans="19:39" ht="13.8">
       <c r="S97" s="15"/>
       <c r="T97" s="15"/>
       <c r="U97" s="15"/>
@@ -15809,7 +15795,7 @@
       <c r="AL97" s="14"/>
       <c r="AM97" s="14"/>
     </row>
-    <row r="98" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="98" spans="19:39" ht="13.8">
       <c r="S98" s="15"/>
       <c r="T98" s="15"/>
       <c r="U98" s="15"/>
@@ -15828,7 +15814,7 @@
       <c r="AL98" s="14"/>
       <c r="AM98" s="14"/>
     </row>
-    <row r="99" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="99" spans="19:39" ht="13.8">
       <c r="S99" s="15"/>
       <c r="T99" s="15"/>
       <c r="U99" s="15"/>
@@ -15847,7 +15833,7 @@
       <c r="AL99" s="14"/>
       <c r="AM99" s="14"/>
     </row>
-    <row r="100" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="100" spans="19:39" ht="13.8">
       <c r="S100" s="15"/>
       <c r="T100" s="15"/>
       <c r="U100" s="15"/>
@@ -15866,7 +15852,7 @@
       <c r="AL100" s="14"/>
       <c r="AM100" s="14"/>
     </row>
-    <row r="101" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="101" spans="19:39" ht="13.8">
       <c r="S101" s="15"/>
       <c r="T101" s="15"/>
       <c r="U101" s="15"/>
@@ -15885,7 +15871,7 @@
       <c r="AL101" s="14"/>
       <c r="AM101" s="14"/>
     </row>
-    <row r="102" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="102" spans="19:39" ht="13.8">
       <c r="S102" s="15"/>
       <c r="T102" s="15"/>
       <c r="U102" s="15"/>
@@ -15904,7 +15890,7 @@
       <c r="AL102" s="14"/>
       <c r="AM102" s="14"/>
     </row>
-    <row r="103" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="103" spans="19:39" ht="13.8">
       <c r="S103" s="15"/>
       <c r="T103" s="15"/>
       <c r="U103" s="15"/>
@@ -15923,7 +15909,7 @@
       <c r="AL103" s="14"/>
       <c r="AM103" s="14"/>
     </row>
-    <row r="104" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="104" spans="19:39" ht="13.8">
       <c r="S104" s="15"/>
       <c r="T104" s="15"/>
       <c r="U104" s="15"/>
@@ -15942,7 +15928,7 @@
       <c r="AL104" s="14"/>
       <c r="AM104" s="14"/>
     </row>
-    <row r="105" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="105" spans="19:39" ht="13.8">
       <c r="S105" s="15"/>
       <c r="T105" s="15"/>
       <c r="U105" s="15"/>
@@ -15961,7 +15947,7 @@
       <c r="AL105" s="14"/>
       <c r="AM105" s="14"/>
     </row>
-    <row r="106" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="106" spans="19:39" ht="13.8">
       <c r="S106" s="15"/>
       <c r="T106" s="15"/>
       <c r="U106" s="15"/>
@@ -15980,7 +15966,7 @@
       <c r="AL106" s="14"/>
       <c r="AM106" s="14"/>
     </row>
-    <row r="107" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="107" spans="19:39" ht="13.8">
       <c r="S107" s="15"/>
       <c r="T107" s="15"/>
       <c r="U107" s="15"/>
@@ -15999,7 +15985,7 @@
       <c r="AL107" s="14"/>
       <c r="AM107" s="14"/>
     </row>
-    <row r="108" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="108" spans="19:39" ht="13.8">
       <c r="S108" s="15"/>
       <c r="T108" s="15"/>
       <c r="U108" s="15"/>
@@ -16018,7 +16004,7 @@
       <c r="AL108" s="14"/>
       <c r="AM108" s="14"/>
     </row>
-    <row r="109" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="109" spans="19:39" ht="13.8">
       <c r="S109" s="15"/>
       <c r="T109" s="15"/>
       <c r="U109" s="15"/>
@@ -16037,7 +16023,7 @@
       <c r="AL109" s="14"/>
       <c r="AM109" s="14"/>
     </row>
-    <row r="110" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="110" spans="19:39" ht="13.8">
       <c r="S110" s="15"/>
       <c r="T110" s="15"/>
       <c r="U110" s="15"/>
@@ -16056,7 +16042,7 @@
       <c r="AL110" s="14"/>
       <c r="AM110" s="14"/>
     </row>
-    <row r="111" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="111" spans="19:39" ht="13.8">
       <c r="S111" s="15"/>
       <c r="T111" s="15"/>
       <c r="U111" s="15"/>
@@ -16075,7 +16061,7 @@
       <c r="AL111" s="14"/>
       <c r="AM111" s="14"/>
     </row>
-    <row r="112" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="112" spans="19:39" ht="13.8">
       <c r="S112" s="15"/>
       <c r="T112" s="15"/>
       <c r="U112" s="15"/>
@@ -16094,7 +16080,7 @@
       <c r="AL112" s="14"/>
       <c r="AM112" s="14"/>
     </row>
-    <row r="113" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="113" spans="19:39" ht="13.8">
       <c r="S113" s="15"/>
       <c r="T113" s="15"/>
       <c r="U113" s="15"/>
@@ -16113,7 +16099,7 @@
       <c r="AL113" s="14"/>
       <c r="AM113" s="14"/>
     </row>
-    <row r="114" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="114" spans="19:39" ht="13.8">
       <c r="S114" s="15"/>
       <c r="T114" s="15"/>
       <c r="U114" s="15"/>
@@ -16132,7 +16118,7 @@
       <c r="AL114" s="14"/>
       <c r="AM114" s="14"/>
     </row>
-    <row r="115" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="115" spans="19:39" ht="13.8">
       <c r="S115" s="15"/>
       <c r="T115" s="15"/>
       <c r="U115" s="15"/>
@@ -16151,7 +16137,7 @@
       <c r="AL115" s="14"/>
       <c r="AM115" s="14"/>
     </row>
-    <row r="116" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="116" spans="19:39" ht="13.8">
       <c r="S116" s="15"/>
       <c r="T116" s="15"/>
       <c r="U116" s="15"/>
@@ -16170,7 +16156,7 @@
       <c r="AL116" s="14"/>
       <c r="AM116" s="14"/>
     </row>
-    <row r="117" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="117" spans="19:39" ht="13.8">
       <c r="S117" s="15"/>
       <c r="T117" s="15"/>
       <c r="U117" s="15"/>
@@ -16189,7 +16175,7 @@
       <c r="AL117" s="14"/>
       <c r="AM117" s="14"/>
     </row>
-    <row r="118" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="118" spans="19:39" ht="13.8">
       <c r="S118" s="15"/>
       <c r="T118" s="15"/>
       <c r="U118" s="15"/>
@@ -16208,7 +16194,7 @@
       <c r="AL118" s="14"/>
       <c r="AM118" s="14"/>
     </row>
-    <row r="119" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="119" spans="19:39" ht="13.8">
       <c r="S119" s="15"/>
       <c r="T119" s="15"/>
       <c r="U119" s="15"/>
@@ -16227,7 +16213,7 @@
       <c r="AL119" s="14"/>
       <c r="AM119" s="14"/>
     </row>
-    <row r="120" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="120" spans="19:39" ht="13.8">
       <c r="S120" s="15"/>
       <c r="T120" s="15"/>
       <c r="U120" s="15"/>
@@ -16246,7 +16232,7 @@
       <c r="AL120" s="14"/>
       <c r="AM120" s="14"/>
     </row>
-    <row r="121" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="121" spans="19:39" ht="13.8">
       <c r="S121" s="15"/>
       <c r="T121" s="15"/>
       <c r="U121" s="15"/>
@@ -16265,7 +16251,7 @@
       <c r="AL121" s="14"/>
       <c r="AM121" s="14"/>
     </row>
-    <row r="122" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="122" spans="19:39" ht="13.8">
       <c r="S122" s="15"/>
       <c r="T122" s="15"/>
       <c r="U122" s="15"/>
@@ -16284,7 +16270,7 @@
       <c r="AL122" s="14"/>
       <c r="AM122" s="14"/>
     </row>
-    <row r="123" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="123" spans="19:39" ht="13.8">
       <c r="S123" s="15"/>
       <c r="T123" s="15"/>
       <c r="U123" s="15"/>
@@ -16303,7 +16289,7 @@
       <c r="AL123" s="14"/>
       <c r="AM123" s="14"/>
     </row>
-    <row r="124" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="124" spans="19:39" ht="13.8">
       <c r="S124" s="15"/>
       <c r="T124" s="15"/>
       <c r="U124" s="15"/>
@@ -16322,7 +16308,7 @@
       <c r="AL124" s="14"/>
       <c r="AM124" s="14"/>
     </row>
-    <row r="125" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="125" spans="19:39" ht="13.8">
       <c r="S125" s="15"/>
       <c r="T125" s="15"/>
       <c r="U125" s="15"/>
@@ -16341,7 +16327,7 @@
       <c r="AL125" s="14"/>
       <c r="AM125" s="14"/>
     </row>
-    <row r="126" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="126" spans="19:39" ht="13.8">
       <c r="S126" s="15"/>
       <c r="T126" s="15"/>
       <c r="U126" s="15"/>
@@ -16360,7 +16346,7 @@
       <c r="AL126" s="14"/>
       <c r="AM126" s="14"/>
     </row>
-    <row r="127" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="127" spans="19:39" ht="13.8">
       <c r="S127" s="15"/>
       <c r="T127" s="15"/>
       <c r="U127" s="15"/>
@@ -16379,7 +16365,7 @@
       <c r="AL127" s="14"/>
       <c r="AM127" s="14"/>
     </row>
-    <row r="128" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="128" spans="19:39" ht="13.8">
       <c r="S128" s="15"/>
       <c r="T128" s="15"/>
       <c r="U128" s="15"/>
@@ -16398,7 +16384,7 @@
       <c r="AL128" s="14"/>
       <c r="AM128" s="14"/>
     </row>
-    <row r="129" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="129" spans="19:39" ht="13.8">
       <c r="S129" s="15"/>
       <c r="T129" s="15"/>
       <c r="U129" s="15"/>
@@ -16417,7 +16403,7 @@
       <c r="AL129" s="14"/>
       <c r="AM129" s="14"/>
     </row>
-    <row r="130" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="130" spans="19:39" ht="13.8">
       <c r="S130" s="15"/>
       <c r="T130" s="15"/>
       <c r="U130" s="15"/>
@@ -16436,7 +16422,7 @@
       <c r="AL130" s="14"/>
       <c r="AM130" s="14"/>
     </row>
-    <row r="131" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="131" spans="19:39" ht="13.8">
       <c r="S131" s="15"/>
       <c r="T131" s="15"/>
       <c r="U131" s="15"/>
@@ -16455,7 +16441,7 @@
       <c r="AL131" s="14"/>
       <c r="AM131" s="14"/>
     </row>
-    <row r="132" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="132" spans="19:39" ht="13.8">
       <c r="S132" s="15"/>
       <c r="T132" s="15"/>
       <c r="U132" s="15"/>
@@ -16474,7 +16460,7 @@
       <c r="AL132" s="14"/>
       <c r="AM132" s="14"/>
     </row>
-    <row r="133" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="133" spans="19:39" ht="13.8">
       <c r="S133" s="15"/>
       <c r="T133" s="15"/>
       <c r="U133" s="15"/>
@@ -16493,7 +16479,7 @@
       <c r="AL133" s="14"/>
       <c r="AM133" s="14"/>
     </row>
-    <row r="134" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="134" spans="19:39" ht="13.8">
       <c r="S134" s="15"/>
       <c r="T134" s="15"/>
       <c r="U134" s="15"/>
@@ -16512,7 +16498,7 @@
       <c r="AL134" s="14"/>
       <c r="AM134" s="14"/>
     </row>
-    <row r="135" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="135" spans="19:39" ht="13.8">
       <c r="S135" s="15"/>
       <c r="T135" s="15"/>
       <c r="U135" s="15"/>
@@ -16531,7 +16517,7 @@
       <c r="AL135" s="14"/>
       <c r="AM135" s="14"/>
     </row>
-    <row r="136" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="136" spans="19:39" ht="13.8">
       <c r="S136" s="15"/>
       <c r="T136" s="15"/>
       <c r="U136" s="15"/>
@@ -16550,7 +16536,7 @@
       <c r="AL136" s="14"/>
       <c r="AM136" s="14"/>
     </row>
-    <row r="137" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="137" spans="19:39" ht="13.8">
       <c r="S137" s="15"/>
       <c r="T137" s="15"/>
       <c r="U137" s="15"/>
@@ -16569,7 +16555,7 @@
       <c r="AL137" s="14"/>
       <c r="AM137" s="14"/>
     </row>
-    <row r="138" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="138" spans="19:39" ht="13.8">
       <c r="S138" s="15"/>
       <c r="T138" s="15"/>
       <c r="U138" s="15"/>
@@ -16588,7 +16574,7 @@
       <c r="AL138" s="14"/>
       <c r="AM138" s="14"/>
     </row>
-    <row r="139" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="139" spans="19:39" ht="13.8">
       <c r="S139" s="15"/>
       <c r="T139" s="15"/>
       <c r="U139" s="15"/>
@@ -16607,7 +16593,7 @@
       <c r="AL139" s="14"/>
       <c r="AM139" s="14"/>
     </row>
-    <row r="140" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="140" spans="19:39" ht="13.8">
       <c r="S140" s="15"/>
       <c r="T140" s="15"/>
       <c r="U140" s="15"/>
@@ -16626,7 +16612,7 @@
       <c r="AL140" s="14"/>
       <c r="AM140" s="14"/>
     </row>
-    <row r="141" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="141" spans="19:39" ht="13.8">
       <c r="S141" s="15"/>
       <c r="T141" s="15"/>
       <c r="U141" s="15"/>
@@ -16645,7 +16631,7 @@
       <c r="AL141" s="14"/>
       <c r="AM141" s="14"/>
     </row>
-    <row r="142" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="142" spans="19:39" ht="13.8">
       <c r="S142" s="15"/>
       <c r="T142" s="15"/>
       <c r="U142" s="15"/>
@@ -16664,7 +16650,7 @@
       <c r="AL142" s="14"/>
       <c r="AM142" s="14"/>
     </row>
-    <row r="143" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="143" spans="19:39" ht="13.8">
       <c r="S143" s="15"/>
       <c r="T143" s="15"/>
       <c r="U143" s="15"/>
@@ -16683,7 +16669,7 @@
       <c r="AL143" s="14"/>
       <c r="AM143" s="14"/>
     </row>
-    <row r="144" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="144" spans="19:39" ht="13.8">
       <c r="S144" s="15"/>
       <c r="T144" s="15"/>
       <c r="U144" s="15"/>
@@ -16702,7 +16688,7 @@
       <c r="AL144" s="14"/>
       <c r="AM144" s="14"/>
     </row>
-    <row r="145" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="145" spans="19:39" ht="13.8">
       <c r="S145" s="15"/>
       <c r="T145" s="15"/>
       <c r="U145" s="15"/>
@@ -16721,7 +16707,7 @@
       <c r="AL145" s="14"/>
       <c r="AM145" s="14"/>
     </row>
-    <row r="146" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="146" spans="19:39" ht="13.8">
       <c r="S146" s="15"/>
       <c r="T146" s="15"/>
       <c r="U146" s="15"/>
@@ -16740,7 +16726,7 @@
       <c r="AL146" s="14"/>
       <c r="AM146" s="14"/>
     </row>
-    <row r="147" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="147" spans="19:39" ht="13.8">
       <c r="S147" s="15"/>
       <c r="T147" s="15"/>
       <c r="U147" s="15"/>
@@ -16759,7 +16745,7 @@
       <c r="AL147" s="14"/>
       <c r="AM147" s="14"/>
     </row>
-    <row r="148" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="148" spans="19:39" ht="13.8">
       <c r="S148" s="15"/>
       <c r="T148" s="15"/>
       <c r="U148" s="15"/>
@@ -16778,7 +16764,7 @@
       <c r="AL148" s="14"/>
       <c r="AM148" s="14"/>
     </row>
-    <row r="149" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="149" spans="19:39" ht="13.8">
       <c r="S149" s="15"/>
       <c r="T149" s="15"/>
       <c r="U149" s="15"/>
@@ -16797,7 +16783,7 @@
       <c r="AL149" s="14"/>
       <c r="AM149" s="14"/>
     </row>
-    <row r="150" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="150" spans="19:39" ht="13.8">
       <c r="S150" s="15"/>
       <c r="T150" s="15"/>
       <c r="U150" s="15"/>
@@ -16816,7 +16802,7 @@
       <c r="AL150" s="14"/>
       <c r="AM150" s="14"/>
     </row>
-    <row r="151" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="151" spans="19:39" ht="13.8">
       <c r="S151" s="15"/>
       <c r="T151" s="15"/>
       <c r="U151" s="15"/>
@@ -16835,7 +16821,7 @@
       <c r="AL151" s="14"/>
       <c r="AM151" s="14"/>
     </row>
-    <row r="152" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="152" spans="19:39" ht="13.8">
       <c r="S152" s="15"/>
       <c r="T152" s="15"/>
       <c r="U152" s="15"/>
@@ -16854,7 +16840,7 @@
       <c r="AL152" s="14"/>
       <c r="AM152" s="14"/>
     </row>
-    <row r="153" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="153" spans="19:39" ht="13.8">
       <c r="S153" s="15"/>
       <c r="T153" s="15"/>
       <c r="U153" s="15"/>
@@ -16873,7 +16859,7 @@
       <c r="AL153" s="14"/>
       <c r="AM153" s="14"/>
     </row>
-    <row r="154" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="154" spans="19:39" ht="13.8">
       <c r="S154" s="15"/>
       <c r="T154" s="15"/>
       <c r="U154" s="15"/>
@@ -16892,7 +16878,7 @@
       <c r="AL154" s="14"/>
       <c r="AM154" s="14"/>
     </row>
-    <row r="155" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="155" spans="19:39" ht="13.8">
       <c r="S155" s="15"/>
       <c r="T155" s="15"/>
       <c r="U155" s="15"/>
@@ -16911,7 +16897,7 @@
       <c r="AL155" s="14"/>
       <c r="AM155" s="14"/>
     </row>
-    <row r="156" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="156" spans="19:39" ht="13.8">
       <c r="S156" s="15"/>
       <c r="T156" s="15"/>
       <c r="U156" s="15"/>
@@ -16930,7 +16916,7 @@
       <c r="AL156" s="14"/>
       <c r="AM156" s="14"/>
     </row>
-    <row r="157" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="157" spans="19:39" ht="13.8">
       <c r="S157" s="15"/>
       <c r="T157" s="15"/>
       <c r="U157" s="15"/>
@@ -16949,7 +16935,7 @@
       <c r="AL157" s="14"/>
       <c r="AM157" s="14"/>
     </row>
-    <row r="158" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="158" spans="19:39" ht="13.8">
       <c r="S158" s="15"/>
       <c r="T158" s="15"/>
       <c r="U158" s="15"/>
@@ -16968,7 +16954,7 @@
       <c r="AL158" s="14"/>
       <c r="AM158" s="14"/>
     </row>
-    <row r="159" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="159" spans="19:39" ht="13.8">
       <c r="S159" s="15"/>
       <c r="T159" s="15"/>
       <c r="U159" s="15"/>
@@ -16987,7 +16973,7 @@
       <c r="AL159" s="14"/>
       <c r="AM159" s="14"/>
     </row>
-    <row r="160" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="160" spans="19:39" ht="13.8">
       <c r="S160" s="15"/>
       <c r="T160" s="15"/>
       <c r="U160" s="15"/>
@@ -17006,7 +16992,7 @@
       <c r="AL160" s="14"/>
       <c r="AM160" s="14"/>
     </row>
-    <row r="161" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="161" spans="19:39" ht="13.8">
       <c r="S161" s="15"/>
       <c r="T161" s="15"/>
       <c r="U161" s="15"/>
@@ -17025,7 +17011,7 @@
       <c r="AL161" s="14"/>
       <c r="AM161" s="14"/>
     </row>
-    <row r="162" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="162" spans="19:39" ht="13.8">
       <c r="S162" s="15"/>
       <c r="T162" s="15"/>
       <c r="U162" s="15"/>
@@ -17044,7 +17030,7 @@
       <c r="AL162" s="14"/>
       <c r="AM162" s="14"/>
     </row>
-    <row r="163" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="163" spans="19:39" ht="13.8">
       <c r="S163" s="15"/>
       <c r="T163" s="15"/>
       <c r="U163" s="15"/>
@@ -17063,7 +17049,7 @@
       <c r="AL163" s="14"/>
       <c r="AM163" s="14"/>
     </row>
-    <row r="164" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="164" spans="19:39" ht="13.8">
       <c r="S164" s="15"/>
       <c r="T164" s="15"/>
       <c r="U164" s="15"/>
@@ -17082,7 +17068,7 @@
       <c r="AL164" s="14"/>
       <c r="AM164" s="14"/>
     </row>
-    <row r="165" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="165" spans="19:39" ht="13.8">
       <c r="S165" s="15"/>
       <c r="T165" s="15"/>
       <c r="U165" s="15"/>
@@ -17101,7 +17087,7 @@
       <c r="AL165" s="14"/>
       <c r="AM165" s="14"/>
     </row>
-    <row r="166" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="166" spans="19:39" ht="13.8">
       <c r="S166" s="15"/>
       <c r="T166" s="15"/>
       <c r="U166" s="15"/>
@@ -17120,7 +17106,7 @@
       <c r="AL166" s="14"/>
       <c r="AM166" s="14"/>
     </row>
-    <row r="167" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="167" spans="19:39" ht="13.8">
       <c r="S167" s="15"/>
       <c r="T167" s="15"/>
       <c r="U167" s="15"/>
@@ -17139,7 +17125,7 @@
       <c r="AL167" s="14"/>
       <c r="AM167" s="14"/>
     </row>
-    <row r="168" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="168" spans="19:39" ht="13.8">
       <c r="S168" s="15"/>
       <c r="T168" s="15"/>
       <c r="U168" s="15"/>
@@ -17158,7 +17144,7 @@
       <c r="AL168" s="14"/>
       <c r="AM168" s="14"/>
     </row>
-    <row r="169" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="169" spans="19:39" ht="13.8">
       <c r="S169" s="15"/>
       <c r="T169" s="15"/>
       <c r="U169" s="15"/>
@@ -17177,7 +17163,7 @@
       <c r="AL169" s="14"/>
       <c r="AM169" s="14"/>
     </row>
-    <row r="170" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="170" spans="19:39" ht="13.8">
       <c r="S170" s="15"/>
       <c r="T170" s="15"/>
       <c r="U170" s="15"/>
@@ -17196,7 +17182,7 @@
       <c r="AL170" s="14"/>
       <c r="AM170" s="14"/>
     </row>
-    <row r="171" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="171" spans="19:39" ht="13.8">
       <c r="S171" s="15"/>
       <c r="T171" s="15"/>
       <c r="U171" s="15"/>
@@ -17215,7 +17201,7 @@
       <c r="AL171" s="14"/>
       <c r="AM171" s="14"/>
     </row>
-    <row r="172" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="172" spans="19:39" ht="13.8">
       <c r="S172" s="15"/>
       <c r="T172" s="15"/>
       <c r="U172" s="15"/>
@@ -17234,7 +17220,7 @@
       <c r="AL172" s="14"/>
       <c r="AM172" s="14"/>
     </row>
-    <row r="173" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="173" spans="19:39" ht="13.8">
       <c r="S173" s="15"/>
       <c r="T173" s="15"/>
       <c r="U173" s="15"/>
@@ -17253,7 +17239,7 @@
       <c r="AL173" s="14"/>
       <c r="AM173" s="14"/>
     </row>
-    <row r="174" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="174" spans="19:39" ht="13.8">
       <c r="S174" s="15"/>
       <c r="T174" s="15"/>
       <c r="U174" s="15"/>
@@ -17272,7 +17258,7 @@
       <c r="AL174" s="14"/>
       <c r="AM174" s="14"/>
     </row>
-    <row r="175" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="175" spans="19:39" ht="13.8">
       <c r="S175" s="15"/>
       <c r="T175" s="15"/>
       <c r="U175" s="15"/>
@@ -17291,7 +17277,7 @@
       <c r="AL175" s="14"/>
       <c r="AM175" s="14"/>
     </row>
-    <row r="176" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="176" spans="19:39" ht="13.8">
       <c r="S176" s="15"/>
       <c r="T176" s="15"/>
       <c r="U176" s="15"/>
@@ -17310,7 +17296,7 @@
       <c r="AL176" s="14"/>
       <c r="AM176" s="14"/>
     </row>
-    <row r="177" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="177" spans="19:39" ht="13.8">
       <c r="S177" s="15"/>
       <c r="T177" s="15"/>
       <c r="U177" s="15"/>
@@ -17329,7 +17315,7 @@
       <c r="AL177" s="14"/>
       <c r="AM177" s="14"/>
     </row>
-    <row r="178" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="178" spans="19:39" ht="13.8">
       <c r="S178" s="15"/>
       <c r="T178" s="15"/>
       <c r="U178" s="15"/>
@@ -17348,7 +17334,7 @@
       <c r="AL178" s="14"/>
       <c r="AM178" s="14"/>
     </row>
-    <row r="179" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="179" spans="19:39" ht="13.8">
       <c r="S179" s="15"/>
       <c r="T179" s="15"/>
       <c r="U179" s="15"/>
@@ -17367,7 +17353,7 @@
       <c r="AL179" s="14"/>
       <c r="AM179" s="14"/>
     </row>
-    <row r="180" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="180" spans="19:39" ht="13.8">
       <c r="S180" s="15"/>
       <c r="T180" s="15"/>
       <c r="U180" s="15"/>
@@ -17386,7 +17372,7 @@
       <c r="AL180" s="14"/>
       <c r="AM180" s="14"/>
     </row>
-    <row r="181" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="181" spans="19:39" ht="13.8">
       <c r="S181" s="15"/>
       <c r="T181" s="15"/>
       <c r="U181" s="15"/>
@@ -17405,7 +17391,7 @@
       <c r="AL181" s="14"/>
       <c r="AM181" s="14"/>
     </row>
-    <row r="182" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="182" spans="19:39" ht="13.8">
       <c r="S182" s="15"/>
       <c r="T182" s="15"/>
       <c r="U182" s="15"/>
@@ -17424,7 +17410,7 @@
       <c r="AL182" s="14"/>
       <c r="AM182" s="14"/>
     </row>
-    <row r="183" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="183" spans="19:39" ht="13.8">
       <c r="S183" s="15"/>
       <c r="T183" s="15"/>
       <c r="U183" s="15"/>
@@ -17443,7 +17429,7 @@
       <c r="AL183" s="14"/>
       <c r="AM183" s="14"/>
     </row>
-    <row r="184" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="184" spans="19:39" ht="13.8">
       <c r="S184" s="15"/>
       <c r="T184" s="15"/>
       <c r="U184" s="15"/>
@@ -17462,7 +17448,7 @@
       <c r="AL184" s="14"/>
       <c r="AM184" s="14"/>
     </row>
-    <row r="185" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="185" spans="19:39" ht="13.8">
       <c r="S185" s="15"/>
       <c r="T185" s="15"/>
       <c r="U185" s="15"/>
@@ -17481,7 +17467,7 @@
       <c r="AL185" s="14"/>
       <c r="AM185" s="14"/>
     </row>
-    <row r="186" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="186" spans="19:39" ht="13.8">
       <c r="S186" s="15"/>
       <c r="T186" s="15"/>
       <c r="U186" s="15"/>
@@ -17500,7 +17486,7 @@
       <c r="AL186" s="14"/>
       <c r="AM186" s="14"/>
     </row>
-    <row r="187" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="187" spans="19:39" ht="13.8">
       <c r="S187" s="15"/>
       <c r="T187" s="15"/>
       <c r="U187" s="15"/>
@@ -17519,7 +17505,7 @@
       <c r="AL187" s="14"/>
       <c r="AM187" s="14"/>
     </row>
-    <row r="188" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="188" spans="19:39" ht="13.8">
       <c r="S188" s="15"/>
       <c r="T188" s="15"/>
       <c r="U188" s="15"/>
@@ -17538,7 +17524,7 @@
       <c r="AL188" s="14"/>
       <c r="AM188" s="14"/>
     </row>
-    <row r="189" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="189" spans="19:39" ht="13.8">
       <c r="S189" s="15"/>
       <c r="T189" s="15"/>
       <c r="U189" s="15"/>
@@ -17557,7 +17543,7 @@
       <c r="AL189" s="14"/>
       <c r="AM189" s="14"/>
     </row>
-    <row r="190" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="190" spans="19:39" ht="13.8">
       <c r="S190" s="15"/>
       <c r="T190" s="15"/>
       <c r="U190" s="15"/>
@@ -17576,7 +17562,7 @@
       <c r="AL190" s="14"/>
       <c r="AM190" s="14"/>
     </row>
-    <row r="191" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="191" spans="19:39" ht="13.8">
       <c r="S191" s="15"/>
       <c r="T191" s="15"/>
       <c r="U191" s="15"/>
@@ -17595,7 +17581,7 @@
       <c r="AL191" s="14"/>
       <c r="AM191" s="14"/>
     </row>
-    <row r="192" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="192" spans="19:39" ht="13.8">
       <c r="S192" s="15"/>
       <c r="T192" s="15"/>
       <c r="U192" s="15"/>
@@ -17614,7 +17600,7 @@
       <c r="AL192" s="14"/>
       <c r="AM192" s="14"/>
     </row>
-    <row r="193" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="193" spans="19:39" ht="13.8">
       <c r="S193" s="15"/>
       <c r="T193" s="15"/>
       <c r="U193" s="15"/>
@@ -17633,7 +17619,7 @@
       <c r="AL193" s="14"/>
       <c r="AM193" s="14"/>
     </row>
-    <row r="194" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="194" spans="19:39" ht="13.8">
       <c r="S194" s="15"/>
       <c r="T194" s="15"/>
       <c r="U194" s="15"/>
@@ -17652,7 +17638,7 @@
       <c r="AL194" s="14"/>
       <c r="AM194" s="14"/>
     </row>
-    <row r="195" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="195" spans="19:39" ht="13.8">
       <c r="S195" s="15"/>
       <c r="T195" s="15"/>
       <c r="U195" s="15"/>
@@ -17671,7 +17657,7 @@
       <c r="AL195" s="14"/>
       <c r="AM195" s="14"/>
     </row>
-    <row r="196" spans="19:39" ht="22.75" x14ac:dyDescent="0.9">
+    <row r="196" spans="19:39" ht="13.8">
       <c r="S196" s="15"/>
       <c r="T196" s="15"/>
       <c r="U196" s="15"/>
@@ -17690,7 +17676,7 @@
       <c r="AL196" s="14"/>
       <c r="AM196" s="14"/>
     </row>
-    <row r="197" spans="19:39" ht="23.15" thickBot="1" x14ac:dyDescent="0.95">
+    <row r="197" spans="19:39" ht="14.4" thickBot="1">
       <c r="S197" s="15"/>
       <c r="T197" s="15"/>
       <c r="U197" s="15"/>

</xml_diff>

<commit_message>
insert 3 new card
</commit_message>
<xml_diff>
--- a/assets/data-source/data.xlsx
+++ b/assets/data-source/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Venus\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF62AF90-B416-4C44-A40E-9D4817E5C122}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87F33568-1DD1-4D33-BD21-3C9170FDD5E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="736" activeTab="1" xr2:uid="{2E6F1639-AB3B-4860-9C01-087F2448B9B1}"/>
   </bookViews>
@@ -79,7 +79,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="112">
   <si>
     <t>پایه سنوات</t>
   </si>
@@ -88,9 +88,6 @@
   </si>
   <si>
     <t>گذشته</t>
-  </si>
-  <si>
-    <t>استحقاقی</t>
   </si>
   <si>
     <t>سال</t>
@@ -412,6 +409,9 @@
   </si>
   <si>
     <t>(مزد روزانه سال  قبل *1.07)+1200</t>
+  </si>
+  <si>
+    <t>تجمیعی</t>
   </si>
   <si>
     <t>پایه سنواتی  گذشته</t>
@@ -1142,34 +1142,49 @@
     <xf numFmtId="165" fontId="16" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="2" fontId="9" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="4" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="4" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="2" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="2" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="3" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="3" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="2" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="2" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1196,31 +1211,16 @@
     <xf numFmtId="165" fontId="2" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="3" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="4" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="3" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="168" fontId="2" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="15" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="4" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="2" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1536,575 +1536,575 @@
   <sheetData>
     <row r="1" spans="1:112" s="30" customFormat="1" ht="23.1" customHeight="1">
       <c r="A1" s="29" t="s">
-        <v>4</v>
-      </c>
-      <c r="B1" s="62">
+        <v>3</v>
+      </c>
+      <c r="B1" s="60">
         <v>1369</v>
       </c>
-      <c r="C1" s="63"/>
-      <c r="D1" s="63"/>
-      <c r="E1" s="62">
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="60">
         <v>1370</v>
       </c>
-      <c r="F1" s="63"/>
-      <c r="G1" s="63"/>
-      <c r="H1" s="62">
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="60">
         <v>1371</v>
       </c>
-      <c r="I1" s="63"/>
-      <c r="J1" s="63"/>
-      <c r="K1" s="62">
+      <c r="I1" s="61"/>
+      <c r="J1" s="61"/>
+      <c r="K1" s="60">
         <v>1372</v>
       </c>
-      <c r="L1" s="63"/>
-      <c r="M1" s="63"/>
-      <c r="N1" s="62">
+      <c r="L1" s="61"/>
+      <c r="M1" s="61"/>
+      <c r="N1" s="60">
         <v>1373</v>
       </c>
-      <c r="O1" s="63"/>
-      <c r="P1" s="63"/>
-      <c r="Q1" s="62">
+      <c r="O1" s="61"/>
+      <c r="P1" s="61"/>
+      <c r="Q1" s="60">
         <v>1374</v>
       </c>
-      <c r="R1" s="63"/>
-      <c r="S1" s="63"/>
-      <c r="T1" s="62">
+      <c r="R1" s="61"/>
+      <c r="S1" s="61"/>
+      <c r="T1" s="60">
         <v>1375</v>
       </c>
-      <c r="U1" s="63"/>
-      <c r="V1" s="63"/>
-      <c r="W1" s="62">
+      <c r="U1" s="61"/>
+      <c r="V1" s="61"/>
+      <c r="W1" s="60">
         <v>1376</v>
       </c>
-      <c r="X1" s="63"/>
-      <c r="Y1" s="63"/>
-      <c r="Z1" s="62">
+      <c r="X1" s="61"/>
+      <c r="Y1" s="61"/>
+      <c r="Z1" s="60">
         <v>1377</v>
       </c>
-      <c r="AA1" s="63"/>
-      <c r="AB1" s="63"/>
-      <c r="AC1" s="62">
+      <c r="AA1" s="61"/>
+      <c r="AB1" s="61"/>
+      <c r="AC1" s="60">
         <v>1378</v>
       </c>
-      <c r="AD1" s="63"/>
-      <c r="AE1" s="63"/>
-      <c r="AF1" s="62">
+      <c r="AD1" s="61"/>
+      <c r="AE1" s="61"/>
+      <c r="AF1" s="60">
         <v>1379</v>
       </c>
-      <c r="AG1" s="63"/>
-      <c r="AH1" s="63"/>
-      <c r="AI1" s="62">
+      <c r="AG1" s="61"/>
+      <c r="AH1" s="61"/>
+      <c r="AI1" s="60">
         <v>1380</v>
       </c>
-      <c r="AJ1" s="63"/>
-      <c r="AK1" s="63"/>
-      <c r="AL1" s="62">
+      <c r="AJ1" s="61"/>
+      <c r="AK1" s="61"/>
+      <c r="AL1" s="60">
         <v>1381</v>
       </c>
-      <c r="AM1" s="63"/>
-      <c r="AN1" s="63"/>
-      <c r="AO1" s="62">
+      <c r="AM1" s="61"/>
+      <c r="AN1" s="61"/>
+      <c r="AO1" s="60">
         <v>1382</v>
       </c>
-      <c r="AP1" s="63"/>
-      <c r="AQ1" s="63"/>
-      <c r="AR1" s="62">
+      <c r="AP1" s="61"/>
+      <c r="AQ1" s="61"/>
+      <c r="AR1" s="60">
         <v>1383</v>
       </c>
-      <c r="AS1" s="63"/>
-      <c r="AT1" s="63"/>
-      <c r="AU1" s="62">
+      <c r="AS1" s="61"/>
+      <c r="AT1" s="61"/>
+      <c r="AU1" s="60">
         <v>1384</v>
       </c>
-      <c r="AV1" s="63"/>
-      <c r="AW1" s="63"/>
-      <c r="AX1" s="62">
+      <c r="AV1" s="61"/>
+      <c r="AW1" s="61"/>
+      <c r="AX1" s="60">
         <v>1385</v>
       </c>
-      <c r="AY1" s="63"/>
-      <c r="AZ1" s="63"/>
-      <c r="BA1" s="62">
+      <c r="AY1" s="61"/>
+      <c r="AZ1" s="61"/>
+      <c r="BA1" s="60">
         <v>1386</v>
       </c>
-      <c r="BB1" s="63"/>
-      <c r="BC1" s="63"/>
-      <c r="BD1" s="62">
+      <c r="BB1" s="61"/>
+      <c r="BC1" s="61"/>
+      <c r="BD1" s="60">
         <v>1387</v>
       </c>
-      <c r="BE1" s="63"/>
-      <c r="BF1" s="63"/>
-      <c r="BG1" s="62">
+      <c r="BE1" s="61"/>
+      <c r="BF1" s="61"/>
+      <c r="BG1" s="60">
         <v>1388</v>
       </c>
-      <c r="BH1" s="63"/>
-      <c r="BI1" s="63"/>
-      <c r="BJ1" s="62">
+      <c r="BH1" s="61"/>
+      <c r="BI1" s="61"/>
+      <c r="BJ1" s="60">
         <v>1389</v>
       </c>
-      <c r="BK1" s="63"/>
-      <c r="BL1" s="63"/>
-      <c r="BM1" s="62">
+      <c r="BK1" s="61"/>
+      <c r="BL1" s="61"/>
+      <c r="BM1" s="60">
         <v>1390</v>
       </c>
-      <c r="BN1" s="63"/>
-      <c r="BO1" s="63"/>
-      <c r="BP1" s="62">
+      <c r="BN1" s="61"/>
+      <c r="BO1" s="61"/>
+      <c r="BP1" s="60">
         <v>1391</v>
       </c>
-      <c r="BQ1" s="63"/>
-      <c r="BR1" s="63"/>
-      <c r="BS1" s="62">
+      <c r="BQ1" s="61"/>
+      <c r="BR1" s="61"/>
+      <c r="BS1" s="60">
         <v>1392</v>
       </c>
-      <c r="BT1" s="63"/>
-      <c r="BU1" s="63"/>
-      <c r="BV1" s="62">
+      <c r="BT1" s="61"/>
+      <c r="BU1" s="61"/>
+      <c r="BV1" s="60">
         <v>1393</v>
       </c>
-      <c r="BW1" s="63"/>
-      <c r="BX1" s="63"/>
-      <c r="BY1" s="62">
+      <c r="BW1" s="61"/>
+      <c r="BX1" s="61"/>
+      <c r="BY1" s="60">
         <v>1394</v>
       </c>
-      <c r="BZ1" s="63"/>
-      <c r="CA1" s="63"/>
-      <c r="CB1" s="62">
+      <c r="BZ1" s="61"/>
+      <c r="CA1" s="61"/>
+      <c r="CB1" s="60">
         <v>1395</v>
       </c>
-      <c r="CC1" s="63"/>
-      <c r="CD1" s="63"/>
-      <c r="CE1" s="62">
+      <c r="CC1" s="61"/>
+      <c r="CD1" s="61"/>
+      <c r="CE1" s="60">
         <v>1396</v>
       </c>
-      <c r="CF1" s="63"/>
-      <c r="CG1" s="63"/>
-      <c r="CH1" s="62">
+      <c r="CF1" s="61"/>
+      <c r="CG1" s="61"/>
+      <c r="CH1" s="60">
         <v>1397</v>
       </c>
-      <c r="CI1" s="63"/>
-      <c r="CJ1" s="63"/>
-      <c r="CK1" s="62">
+      <c r="CI1" s="61"/>
+      <c r="CJ1" s="61"/>
+      <c r="CK1" s="60">
         <v>1398</v>
       </c>
-      <c r="CL1" s="63"/>
-      <c r="CM1" s="63"/>
-      <c r="CN1" s="62">
+      <c r="CL1" s="61"/>
+      <c r="CM1" s="61"/>
+      <c r="CN1" s="60">
         <v>1399</v>
       </c>
-      <c r="CO1" s="63"/>
-      <c r="CP1" s="63"/>
-      <c r="CQ1" s="62">
+      <c r="CO1" s="61"/>
+      <c r="CP1" s="61"/>
+      <c r="CQ1" s="60">
         <v>1400</v>
       </c>
-      <c r="CR1" s="63"/>
-      <c r="CS1" s="63"/>
-      <c r="CT1" s="62">
+      <c r="CR1" s="61"/>
+      <c r="CS1" s="61"/>
+      <c r="CT1" s="60">
         <v>1401</v>
       </c>
-      <c r="CU1" s="63"/>
-      <c r="CV1" s="63"/>
-      <c r="CW1" s="62">
+      <c r="CU1" s="61"/>
+      <c r="CV1" s="61"/>
+      <c r="CW1" s="60">
         <v>1402</v>
       </c>
-      <c r="CX1" s="63"/>
-      <c r="CY1" s="63"/>
-      <c r="CZ1" s="62">
+      <c r="CX1" s="61"/>
+      <c r="CY1" s="61"/>
+      <c r="CZ1" s="60">
         <v>1403</v>
       </c>
-      <c r="DA1" s="63"/>
-      <c r="DB1" s="63"/>
-      <c r="DC1" s="62">
+      <c r="DA1" s="61"/>
+      <c r="DB1" s="61"/>
+      <c r="DC1" s="60">
         <v>1404</v>
       </c>
-      <c r="DD1" s="63"/>
-      <c r="DE1" s="63"/>
-      <c r="DF1" s="62">
+      <c r="DD1" s="61"/>
+      <c r="DE1" s="61"/>
+      <c r="DF1" s="60">
         <v>1405</v>
       </c>
-      <c r="DG1" s="63"/>
-      <c r="DH1" s="63"/>
+      <c r="DG1" s="61"/>
+      <c r="DH1" s="61"/>
     </row>
     <row r="2" spans="1:112" s="32" customFormat="1" ht="31.35" customHeight="1">
       <c r="A2" s="31" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" s="60">
+        <v>5</v>
+      </c>
+      <c r="B2" s="62">
         <v>1.1399999999999999</v>
       </c>
-      <c r="C2" s="60"/>
-      <c r="D2" s="60"/>
-      <c r="E2" s="60">
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62">
         <v>1.1200000000000001</v>
       </c>
-      <c r="F2" s="60"/>
-      <c r="G2" s="60"/>
-      <c r="H2" s="60">
+      <c r="F2" s="62"/>
+      <c r="G2" s="62"/>
+      <c r="H2" s="62">
         <v>1.101</v>
       </c>
-      <c r="I2" s="60"/>
-      <c r="J2" s="60"/>
-      <c r="K2" s="60">
+      <c r="I2" s="62"/>
+      <c r="J2" s="62"/>
+      <c r="K2" s="62">
         <v>1.1299999999999999</v>
       </c>
-      <c r="L2" s="60"/>
-      <c r="M2" s="60"/>
-      <c r="N2" s="60">
+      <c r="L2" s="62"/>
+      <c r="M2" s="62"/>
+      <c r="N2" s="62">
         <v>1.1499999999999999</v>
       </c>
-      <c r="O2" s="60"/>
-      <c r="P2" s="60"/>
-      <c r="Q2" s="60">
+      <c r="O2" s="62"/>
+      <c r="P2" s="62"/>
+      <c r="Q2" s="62">
         <v>1.26</v>
       </c>
-      <c r="R2" s="60"/>
-      <c r="S2" s="60"/>
-      <c r="T2" s="60">
+      <c r="R2" s="62"/>
+      <c r="S2" s="62"/>
+      <c r="T2" s="62">
         <v>1.38</v>
       </c>
-      <c r="U2" s="60"/>
-      <c r="V2" s="60"/>
-      <c r="W2" s="60">
+      <c r="U2" s="62"/>
+      <c r="V2" s="62"/>
+      <c r="W2" s="62">
         <v>1.21</v>
       </c>
-      <c r="X2" s="60"/>
-      <c r="Y2" s="60"/>
-      <c r="Z2" s="60">
+      <c r="X2" s="62"/>
+      <c r="Y2" s="62"/>
+      <c r="Z2" s="62">
         <v>1.22</v>
       </c>
-      <c r="AA2" s="60"/>
-      <c r="AB2" s="60"/>
-      <c r="AC2" s="60">
+      <c r="AA2" s="62"/>
+      <c r="AB2" s="62"/>
+      <c r="AC2" s="62">
         <v>1.32</v>
       </c>
-      <c r="AD2" s="60"/>
-      <c r="AE2" s="60"/>
-      <c r="AF2" s="60">
+      <c r="AD2" s="62"/>
+      <c r="AE2" s="62"/>
+      <c r="AF2" s="62">
         <v>1.45</v>
       </c>
-      <c r="AG2" s="60"/>
-      <c r="AH2" s="60"/>
-      <c r="AI2" s="60">
+      <c r="AG2" s="62"/>
+      <c r="AH2" s="62"/>
+      <c r="AI2" s="62">
         <v>1.1200000000000001</v>
       </c>
-      <c r="AJ2" s="60"/>
-      <c r="AK2" s="60"/>
-      <c r="AL2" s="60">
+      <c r="AJ2" s="62"/>
+      <c r="AK2" s="62"/>
+      <c r="AL2" s="62">
         <v>1.17</v>
       </c>
-      <c r="AM2" s="60"/>
-      <c r="AN2" s="60"/>
-      <c r="AO2" s="60">
+      <c r="AM2" s="62"/>
+      <c r="AN2" s="62"/>
+      <c r="AO2" s="62">
         <v>1.1399999999999999</v>
       </c>
-      <c r="AP2" s="60"/>
-      <c r="AQ2" s="60"/>
-      <c r="AR2" s="60">
+      <c r="AP2" s="62"/>
+      <c r="AQ2" s="62"/>
+      <c r="AR2" s="62">
         <v>1.1200000000000001</v>
       </c>
-      <c r="AS2" s="60"/>
-      <c r="AT2" s="60"/>
-      <c r="AU2" s="60">
+      <c r="AS2" s="62"/>
+      <c r="AT2" s="62"/>
+      <c r="AU2" s="62">
         <v>1.101</v>
       </c>
-      <c r="AV2" s="60"/>
-      <c r="AW2" s="60"/>
-      <c r="AX2" s="60">
+      <c r="AV2" s="62"/>
+      <c r="AW2" s="62"/>
+      <c r="AX2" s="62">
         <v>1.1299999999999999</v>
       </c>
-      <c r="AY2" s="60"/>
-      <c r="AZ2" s="60"/>
-      <c r="BA2" s="60">
+      <c r="AY2" s="62"/>
+      <c r="AZ2" s="62"/>
+      <c r="BA2" s="62">
         <v>1.1499999999999999</v>
       </c>
-      <c r="BB2" s="60"/>
-      <c r="BC2" s="60"/>
-      <c r="BD2" s="60">
+      <c r="BB2" s="62"/>
+      <c r="BC2" s="62"/>
+      <c r="BD2" s="62">
         <v>1.26</v>
       </c>
-      <c r="BE2" s="60"/>
-      <c r="BF2" s="60"/>
-      <c r="BG2" s="60">
+      <c r="BE2" s="62"/>
+      <c r="BF2" s="62"/>
+      <c r="BG2" s="62">
         <v>1.38</v>
       </c>
-      <c r="BH2" s="60"/>
-      <c r="BI2" s="60"/>
-      <c r="BJ2" s="60">
+      <c r="BH2" s="62"/>
+      <c r="BI2" s="62"/>
+      <c r="BJ2" s="62">
         <v>1.21</v>
       </c>
-      <c r="BK2" s="60"/>
-      <c r="BL2" s="60"/>
-      <c r="BM2" s="60">
+      <c r="BK2" s="62"/>
+      <c r="BL2" s="62"/>
+      <c r="BM2" s="62">
         <v>1.22</v>
       </c>
-      <c r="BN2" s="60"/>
-      <c r="BO2" s="60"/>
-      <c r="BP2" s="60">
+      <c r="BN2" s="62"/>
+      <c r="BO2" s="62"/>
+      <c r="BP2" s="62">
         <v>1.1000000000000001</v>
       </c>
-      <c r="BQ2" s="60"/>
-      <c r="BR2" s="60"/>
-      <c r="BS2" s="60">
+      <c r="BQ2" s="62"/>
+      <c r="BR2" s="62"/>
+      <c r="BS2" s="62">
         <v>1.1000000000000001</v>
       </c>
-      <c r="BT2" s="60"/>
-      <c r="BU2" s="60"/>
-      <c r="BV2" s="60">
+      <c r="BT2" s="62"/>
+      <c r="BU2" s="62"/>
+      <c r="BV2" s="62">
         <v>1.1200000000000001</v>
       </c>
-      <c r="BW2" s="60"/>
-      <c r="BX2" s="60"/>
-      <c r="BY2" s="60">
+      <c r="BW2" s="62"/>
+      <c r="BX2" s="62"/>
+      <c r="BY2" s="62">
         <v>1.17</v>
       </c>
-      <c r="BZ2" s="60"/>
-      <c r="CA2" s="60"/>
-      <c r="CB2" s="60">
+      <c r="BZ2" s="62"/>
+      <c r="CA2" s="62"/>
+      <c r="CB2" s="62">
         <v>1.1399999999999999</v>
       </c>
-      <c r="CC2" s="60"/>
-      <c r="CD2" s="60"/>
-      <c r="CE2" s="60">
+      <c r="CC2" s="62"/>
+      <c r="CD2" s="62"/>
+      <c r="CE2" s="62">
         <v>1.1200000000000001</v>
       </c>
-      <c r="CF2" s="60"/>
-      <c r="CG2" s="60"/>
-      <c r="CH2" s="60">
+      <c r="CF2" s="62"/>
+      <c r="CG2" s="62"/>
+      <c r="CH2" s="62">
         <v>1.101</v>
       </c>
-      <c r="CI2" s="60"/>
-      <c r="CJ2" s="60"/>
-      <c r="CK2" s="60">
+      <c r="CI2" s="62"/>
+      <c r="CJ2" s="62"/>
+      <c r="CK2" s="62">
         <v>1.1299999999999999</v>
       </c>
-      <c r="CL2" s="60"/>
-      <c r="CM2" s="60"/>
-      <c r="CN2" s="60">
+      <c r="CL2" s="62"/>
+      <c r="CM2" s="62"/>
+      <c r="CN2" s="62">
         <v>1.1499999999999999</v>
       </c>
-      <c r="CO2" s="60"/>
-      <c r="CP2" s="60"/>
-      <c r="CQ2" s="60">
+      <c r="CO2" s="62"/>
+      <c r="CP2" s="62"/>
+      <c r="CQ2" s="62">
         <v>1.26</v>
       </c>
-      <c r="CR2" s="60"/>
-      <c r="CS2" s="60"/>
-      <c r="CT2" s="60">
+      <c r="CR2" s="62"/>
+      <c r="CS2" s="62"/>
+      <c r="CT2" s="62">
         <v>1.38</v>
       </c>
-      <c r="CU2" s="60"/>
-      <c r="CV2" s="60"/>
-      <c r="CW2" s="60">
+      <c r="CU2" s="62"/>
+      <c r="CV2" s="62"/>
+      <c r="CW2" s="62">
         <v>1.21</v>
       </c>
-      <c r="CX2" s="60"/>
-      <c r="CY2" s="60"/>
-      <c r="CZ2" s="60">
+      <c r="CX2" s="62"/>
+      <c r="CY2" s="62"/>
+      <c r="CZ2" s="62">
         <v>1.22</v>
       </c>
-      <c r="DA2" s="60"/>
-      <c r="DB2" s="60"/>
-      <c r="DC2" s="60">
+      <c r="DA2" s="62"/>
+      <c r="DB2" s="62"/>
+      <c r="DC2" s="62">
         <v>1.32</v>
       </c>
-      <c r="DD2" s="60"/>
-      <c r="DE2" s="60"/>
-      <c r="DF2" s="60">
+      <c r="DD2" s="62"/>
+      <c r="DE2" s="62"/>
+      <c r="DF2" s="62">
         <v>1.45</v>
       </c>
-      <c r="DG2" s="60"/>
-      <c r="DH2" s="60"/>
+      <c r="DG2" s="62"/>
+      <c r="DH2" s="62"/>
     </row>
     <row r="3" spans="1:112" s="32" customFormat="1" ht="40.799999999999997" customHeight="1">
       <c r="A3" s="31"/>
-      <c r="B3" s="60" t="s">
+      <c r="B3" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="61"/>
-      <c r="D3" s="61"/>
-      <c r="E3" s="60" t="s">
+      <c r="C3" s="63"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="F3" s="61"/>
-      <c r="G3" s="61"/>
-      <c r="H3" s="60" t="s">
+      <c r="F3" s="63"/>
+      <c r="G3" s="63"/>
+      <c r="H3" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="I3" s="61"/>
-      <c r="J3" s="61"/>
-      <c r="K3" s="60" t="s">
+      <c r="I3" s="63"/>
+      <c r="J3" s="63"/>
+      <c r="K3" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="L3" s="61"/>
-      <c r="M3" s="61"/>
-      <c r="N3" s="60" t="s">
+      <c r="L3" s="63"/>
+      <c r="M3" s="63"/>
+      <c r="N3" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="O3" s="61"/>
-      <c r="P3" s="61"/>
-      <c r="Q3" s="60" t="s">
+      <c r="O3" s="63"/>
+      <c r="P3" s="63"/>
+      <c r="Q3" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="R3" s="61"/>
-      <c r="S3" s="61"/>
-      <c r="T3" s="60" t="s">
+      <c r="R3" s="63"/>
+      <c r="S3" s="63"/>
+      <c r="T3" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="U3" s="61"/>
-      <c r="V3" s="61"/>
-      <c r="W3" s="60" t="s">
+      <c r="U3" s="63"/>
+      <c r="V3" s="63"/>
+      <c r="W3" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="X3" s="61"/>
-      <c r="Y3" s="61"/>
-      <c r="Z3" s="60" t="s">
+      <c r="X3" s="63"/>
+      <c r="Y3" s="63"/>
+      <c r="Z3" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="AA3" s="61"/>
-      <c r="AB3" s="61"/>
-      <c r="AC3" s="60" t="s">
+      <c r="AA3" s="63"/>
+      <c r="AB3" s="63"/>
+      <c r="AC3" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="AD3" s="61"/>
-      <c r="AE3" s="61"/>
-      <c r="AF3" s="60" t="s">
+      <c r="AD3" s="63"/>
+      <c r="AE3" s="63"/>
+      <c r="AF3" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="AG3" s="61"/>
-      <c r="AH3" s="61"/>
-      <c r="AI3" s="60" t="s">
+      <c r="AG3" s="63"/>
+      <c r="AH3" s="63"/>
+      <c r="AI3" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="AJ3" s="61"/>
-      <c r="AK3" s="61"/>
-      <c r="AL3" s="60" t="s">
+      <c r="AJ3" s="63"/>
+      <c r="AK3" s="63"/>
+      <c r="AL3" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="AM3" s="61"/>
-      <c r="AN3" s="61"/>
-      <c r="AO3" s="60" t="s">
+      <c r="AM3" s="63"/>
+      <c r="AN3" s="63"/>
+      <c r="AO3" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="AP3" s="61"/>
-      <c r="AQ3" s="61"/>
-      <c r="AR3" s="60" t="s">
+      <c r="AP3" s="63"/>
+      <c r="AQ3" s="63"/>
+      <c r="AR3" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="AS3" s="61"/>
-      <c r="AT3" s="61"/>
-      <c r="AU3" s="60" t="s">
+      <c r="AS3" s="63"/>
+      <c r="AT3" s="63"/>
+      <c r="AU3" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="AV3" s="61"/>
-      <c r="AW3" s="61"/>
-      <c r="AX3" s="60" t="s">
+      <c r="AV3" s="63"/>
+      <c r="AW3" s="63"/>
+      <c r="AX3" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="AY3" s="61"/>
-      <c r="AZ3" s="61"/>
-      <c r="BA3" s="60" t="s">
+      <c r="AY3" s="63"/>
+      <c r="AZ3" s="63"/>
+      <c r="BA3" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="BB3" s="61"/>
-      <c r="BC3" s="61"/>
-      <c r="BD3" s="60" t="s">
+      <c r="BB3" s="63"/>
+      <c r="BC3" s="63"/>
+      <c r="BD3" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="BE3" s="61"/>
-      <c r="BF3" s="61"/>
-      <c r="BG3" s="60" t="s">
+      <c r="BE3" s="63"/>
+      <c r="BF3" s="63"/>
+      <c r="BG3" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="BH3" s="61"/>
-      <c r="BI3" s="61"/>
-      <c r="BJ3" s="60" t="s">
+      <c r="BH3" s="63"/>
+      <c r="BI3" s="63"/>
+      <c r="BJ3" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="BK3" s="61"/>
-      <c r="BL3" s="61"/>
-      <c r="BM3" s="60" t="s">
+      <c r="BK3" s="63"/>
+      <c r="BL3" s="63"/>
+      <c r="BM3" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="BN3" s="61"/>
-      <c r="BO3" s="61"/>
-      <c r="BP3" s="60" t="s">
+      <c r="BN3" s="63"/>
+      <c r="BO3" s="63"/>
+      <c r="BP3" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="BQ3" s="61"/>
-      <c r="BR3" s="61"/>
-      <c r="BS3" s="60" t="s">
+      <c r="BQ3" s="63"/>
+      <c r="BR3" s="63"/>
+      <c r="BS3" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="BT3" s="61"/>
-      <c r="BU3" s="61"/>
-      <c r="BV3" s="60" t="s">
+      <c r="BT3" s="63"/>
+      <c r="BU3" s="63"/>
+      <c r="BV3" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="BW3" s="61"/>
-      <c r="BX3" s="61"/>
-      <c r="BY3" s="60" t="s">
+      <c r="BW3" s="63"/>
+      <c r="BX3" s="63"/>
+      <c r="BY3" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="BZ3" s="61"/>
-      <c r="CA3" s="61"/>
-      <c r="CB3" s="60" t="s">
+      <c r="BZ3" s="63"/>
+      <c r="CA3" s="63"/>
+      <c r="CB3" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="CC3" s="61"/>
-      <c r="CD3" s="61"/>
-      <c r="CE3" s="60" t="s">
+      <c r="CC3" s="63"/>
+      <c r="CD3" s="63"/>
+      <c r="CE3" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="CF3" s="61"/>
-      <c r="CG3" s="61"/>
-      <c r="CH3" s="60" t="s">
+      <c r="CF3" s="63"/>
+      <c r="CG3" s="63"/>
+      <c r="CH3" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="CI3" s="61"/>
-      <c r="CJ3" s="61"/>
-      <c r="CK3" s="60" t="s">
+      <c r="CI3" s="63"/>
+      <c r="CJ3" s="63"/>
+      <c r="CK3" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="CL3" s="61"/>
-      <c r="CM3" s="61"/>
-      <c r="CN3" s="60" t="s">
+      <c r="CL3" s="63"/>
+      <c r="CM3" s="63"/>
+      <c r="CN3" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="CO3" s="61"/>
-      <c r="CP3" s="61"/>
-      <c r="CQ3" s="60" t="s">
+      <c r="CO3" s="63"/>
+      <c r="CP3" s="63"/>
+      <c r="CQ3" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="CR3" s="61"/>
-      <c r="CS3" s="61"/>
-      <c r="CT3" s="60" t="s">
+      <c r="CR3" s="63"/>
+      <c r="CS3" s="63"/>
+      <c r="CT3" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="CU3" s="61"/>
-      <c r="CV3" s="61"/>
-      <c r="CW3" s="60" t="s">
+      <c r="CU3" s="63"/>
+      <c r="CV3" s="63"/>
+      <c r="CW3" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="CX3" s="61"/>
-      <c r="CY3" s="61"/>
-      <c r="CZ3" s="60" t="s">
+      <c r="CX3" s="63"/>
+      <c r="CY3" s="63"/>
+      <c r="CZ3" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="DA3" s="61"/>
-      <c r="DB3" s="61"/>
-      <c r="DC3" s="60" t="s">
+      <c r="DA3" s="63"/>
+      <c r="DB3" s="63"/>
+      <c r="DC3" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="DD3" s="61"/>
-      <c r="DE3" s="61"/>
-      <c r="DF3" s="60" t="s">
+      <c r="DD3" s="63"/>
+      <c r="DE3" s="63"/>
+      <c r="DF3" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="DG3" s="61"/>
-      <c r="DH3" s="61"/>
+      <c r="DG3" s="63"/>
+      <c r="DH3" s="63"/>
     </row>
     <row r="4" spans="1:112" s="18" customFormat="1" ht="40.799999999999997" customHeight="1">
       <c r="A4" s="23" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B4" s="19" t="s">
         <v>2</v>
@@ -2113,7 +2113,7 @@
         <v>1</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>3</v>
+        <v>110</v>
       </c>
       <c r="E4" s="19" t="s">
         <v>2</v>
@@ -2122,7 +2122,7 @@
         <v>1</v>
       </c>
       <c r="G4" s="19" t="s">
-        <v>3</v>
+        <v>110</v>
       </c>
       <c r="H4" s="19" t="s">
         <v>2</v>
@@ -2131,7 +2131,7 @@
         <v>1</v>
       </c>
       <c r="J4" s="19" t="s">
-        <v>3</v>
+        <v>110</v>
       </c>
       <c r="K4" s="19" t="s">
         <v>2</v>
@@ -2140,7 +2140,7 @@
         <v>1</v>
       </c>
       <c r="M4" s="19" t="s">
-        <v>3</v>
+        <v>110</v>
       </c>
       <c r="N4" s="19" t="s">
         <v>2</v>
@@ -2149,7 +2149,7 @@
         <v>1</v>
       </c>
       <c r="P4" s="19" t="s">
-        <v>3</v>
+        <v>110</v>
       </c>
       <c r="Q4" s="19" t="s">
         <v>2</v>
@@ -2158,7 +2158,7 @@
         <v>1</v>
       </c>
       <c r="S4" s="19" t="s">
-        <v>3</v>
+        <v>110</v>
       </c>
       <c r="T4" s="19" t="s">
         <v>2</v>
@@ -2167,7 +2167,7 @@
         <v>1</v>
       </c>
       <c r="V4" s="19" t="s">
-        <v>3</v>
+        <v>110</v>
       </c>
       <c r="W4" s="19" t="s">
         <v>2</v>
@@ -2176,7 +2176,7 @@
         <v>1</v>
       </c>
       <c r="Y4" s="19" t="s">
-        <v>3</v>
+        <v>110</v>
       </c>
       <c r="Z4" s="19" t="s">
         <v>2</v>
@@ -2185,7 +2185,7 @@
         <v>1</v>
       </c>
       <c r="AB4" s="19" t="s">
-        <v>3</v>
+        <v>110</v>
       </c>
       <c r="AC4" s="19" t="s">
         <v>2</v>
@@ -2194,7 +2194,7 @@
         <v>1</v>
       </c>
       <c r="AE4" s="19" t="s">
-        <v>3</v>
+        <v>110</v>
       </c>
       <c r="AF4" s="19" t="s">
         <v>2</v>
@@ -2202,7 +2202,9 @@
       <c r="AG4" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="AH4" s="19"/>
+      <c r="AH4" s="19" t="s">
+        <v>110</v>
+      </c>
       <c r="AI4" s="19" t="s">
         <v>2</v>
       </c>
@@ -2210,7 +2212,7 @@
         <v>1</v>
       </c>
       <c r="AK4" s="19" t="s">
-        <v>3</v>
+        <v>110</v>
       </c>
       <c r="AL4" s="19" t="s">
         <v>2</v>
@@ -2219,7 +2221,7 @@
         <v>1</v>
       </c>
       <c r="AN4" s="19" t="s">
-        <v>3</v>
+        <v>110</v>
       </c>
       <c r="AO4" s="19" t="s">
         <v>2</v>
@@ -2228,7 +2230,7 @@
         <v>1</v>
       </c>
       <c r="AQ4" s="19" t="s">
-        <v>3</v>
+        <v>110</v>
       </c>
       <c r="AR4" s="19" t="s">
         <v>2</v>
@@ -2237,7 +2239,7 @@
         <v>1</v>
       </c>
       <c r="AT4" s="19" t="s">
-        <v>3</v>
+        <v>110</v>
       </c>
       <c r="AU4" s="19" t="s">
         <v>2</v>
@@ -2246,7 +2248,7 @@
         <v>1</v>
       </c>
       <c r="AW4" s="19" t="s">
-        <v>3</v>
+        <v>110</v>
       </c>
       <c r="AX4" s="19" t="s">
         <v>2</v>
@@ -2255,7 +2257,7 @@
         <v>1</v>
       </c>
       <c r="AZ4" s="19" t="s">
-        <v>3</v>
+        <v>110</v>
       </c>
       <c r="BA4" s="19" t="s">
         <v>2</v>
@@ -2264,7 +2266,7 @@
         <v>1</v>
       </c>
       <c r="BC4" s="19" t="s">
-        <v>3</v>
+        <v>110</v>
       </c>
       <c r="BD4" s="19" t="s">
         <v>2</v>
@@ -2273,7 +2275,7 @@
         <v>1</v>
       </c>
       <c r="BF4" s="19" t="s">
-        <v>3</v>
+        <v>110</v>
       </c>
       <c r="BG4" s="19" t="s">
         <v>2</v>
@@ -2282,7 +2284,7 @@
         <v>1</v>
       </c>
       <c r="BI4" s="19" t="s">
-        <v>3</v>
+        <v>110</v>
       </c>
       <c r="BJ4" s="19" t="s">
         <v>2</v>
@@ -2291,7 +2293,7 @@
         <v>1</v>
       </c>
       <c r="BL4" s="19" t="s">
-        <v>3</v>
+        <v>110</v>
       </c>
       <c r="BM4" s="19" t="s">
         <v>2</v>
@@ -2300,7 +2302,7 @@
         <v>1</v>
       </c>
       <c r="BO4" s="19" t="s">
-        <v>3</v>
+        <v>110</v>
       </c>
       <c r="BP4" s="19" t="s">
         <v>2</v>
@@ -2309,7 +2311,7 @@
         <v>1</v>
       </c>
       <c r="BR4" s="19" t="s">
-        <v>3</v>
+        <v>110</v>
       </c>
       <c r="BS4" s="19" t="s">
         <v>2</v>
@@ -2318,7 +2320,7 @@
         <v>1</v>
       </c>
       <c r="BU4" s="19" t="s">
-        <v>3</v>
+        <v>110</v>
       </c>
       <c r="BV4" s="19" t="s">
         <v>2</v>
@@ -2327,7 +2329,7 @@
         <v>1</v>
       </c>
       <c r="BX4" s="19" t="s">
-        <v>3</v>
+        <v>110</v>
       </c>
       <c r="BY4" s="19" t="s">
         <v>2</v>
@@ -2336,7 +2338,7 @@
         <v>1</v>
       </c>
       <c r="CA4" s="19" t="s">
-        <v>3</v>
+        <v>110</v>
       </c>
       <c r="CB4" s="19" t="s">
         <v>2</v>
@@ -2345,7 +2347,7 @@
         <v>1</v>
       </c>
       <c r="CD4" s="19" t="s">
-        <v>3</v>
+        <v>110</v>
       </c>
       <c r="CE4" s="19" t="s">
         <v>2</v>
@@ -2354,7 +2356,7 @@
         <v>1</v>
       </c>
       <c r="CG4" s="19" t="s">
-        <v>3</v>
+        <v>110</v>
       </c>
       <c r="CH4" s="19" t="s">
         <v>2</v>
@@ -2363,7 +2365,7 @@
         <v>1</v>
       </c>
       <c r="CJ4" s="19" t="s">
-        <v>3</v>
+        <v>110</v>
       </c>
       <c r="CK4" s="19" t="s">
         <v>2</v>
@@ -2372,7 +2374,7 @@
         <v>1</v>
       </c>
       <c r="CM4" s="19" t="s">
-        <v>3</v>
+        <v>110</v>
       </c>
       <c r="CN4" s="19" t="s">
         <v>2</v>
@@ -2381,7 +2383,7 @@
         <v>1</v>
       </c>
       <c r="CP4" s="19" t="s">
-        <v>3</v>
+        <v>110</v>
       </c>
       <c r="CQ4" s="19" t="s">
         <v>2</v>
@@ -2390,7 +2392,7 @@
         <v>1</v>
       </c>
       <c r="CS4" s="19" t="s">
-        <v>3</v>
+        <v>110</v>
       </c>
       <c r="CT4" s="19" t="s">
         <v>2</v>
@@ -2399,7 +2401,7 @@
         <v>1</v>
       </c>
       <c r="CV4" s="19" t="s">
-        <v>3</v>
+        <v>110</v>
       </c>
       <c r="CW4" s="19" t="s">
         <v>2</v>
@@ -2408,7 +2410,7 @@
         <v>1</v>
       </c>
       <c r="CY4" s="19" t="s">
-        <v>3</v>
+        <v>110</v>
       </c>
       <c r="CZ4" s="19" t="s">
         <v>2</v>
@@ -2417,7 +2419,7 @@
         <v>1</v>
       </c>
       <c r="DB4" s="19" t="s">
-        <v>3</v>
+        <v>110</v>
       </c>
       <c r="DC4" s="19" t="s">
         <v>2</v>
@@ -2426,7 +2428,7 @@
         <v>1</v>
       </c>
       <c r="DE4" s="19" t="s">
-        <v>3</v>
+        <v>110</v>
       </c>
       <c r="DF4" s="19" t="s">
         <v>2</v>
@@ -2435,7 +2437,7 @@
         <v>1</v>
       </c>
       <c r="DH4" s="19" t="s">
-        <v>3</v>
+        <v>110</v>
       </c>
     </row>
     <row r="5" spans="1:112" s="26" customFormat="1" ht="27" customHeight="1">
@@ -11172,6 +11174,93 @@
     <row r="348" s="22" customFormat="1"/>
   </sheetData>
   <mergeCells count="111">
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="E3:G3"/>
+    <mergeCell ref="Z3:AB3"/>
+    <mergeCell ref="AC3:AE3"/>
+    <mergeCell ref="AF3:AH3"/>
+    <mergeCell ref="H3:J3"/>
+    <mergeCell ref="K3:M3"/>
+    <mergeCell ref="N3:P3"/>
+    <mergeCell ref="Q3:S3"/>
+    <mergeCell ref="T3:V3"/>
+    <mergeCell ref="W3:Y3"/>
+    <mergeCell ref="CB1:CD1"/>
+    <mergeCell ref="B1:D1"/>
+    <mergeCell ref="E1:G1"/>
+    <mergeCell ref="H1:J1"/>
+    <mergeCell ref="K1:M1"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="K2:M2"/>
+    <mergeCell ref="N2:P2"/>
+    <mergeCell ref="BG2:BI2"/>
+    <mergeCell ref="W1:Y1"/>
+    <mergeCell ref="Z1:AB1"/>
+    <mergeCell ref="AC1:AE1"/>
+    <mergeCell ref="AF1:AH1"/>
+    <mergeCell ref="W2:Y2"/>
+    <mergeCell ref="Z2:AB2"/>
+    <mergeCell ref="AC2:AE2"/>
+    <mergeCell ref="AF2:AH2"/>
+    <mergeCell ref="AI2:AK2"/>
+    <mergeCell ref="AL2:AN2"/>
+    <mergeCell ref="AO2:AQ2"/>
+    <mergeCell ref="AR2:AT2"/>
+    <mergeCell ref="AU2:AW2"/>
+    <mergeCell ref="BY1:CA1"/>
+    <mergeCell ref="Q2:S2"/>
+    <mergeCell ref="N1:P1"/>
+    <mergeCell ref="Q1:S1"/>
+    <mergeCell ref="T1:V1"/>
+    <mergeCell ref="T2:V2"/>
+    <mergeCell ref="BP1:BR1"/>
+    <mergeCell ref="BP2:BR2"/>
+    <mergeCell ref="BP3:BR3"/>
+    <mergeCell ref="BG3:BI3"/>
+    <mergeCell ref="BJ3:BL3"/>
+    <mergeCell ref="BM3:BO3"/>
+    <mergeCell ref="AI3:AK3"/>
+    <mergeCell ref="AL3:AN3"/>
+    <mergeCell ref="AO3:AQ3"/>
+    <mergeCell ref="AR3:AT3"/>
+    <mergeCell ref="BM1:BO1"/>
+    <mergeCell ref="BJ2:BL2"/>
+    <mergeCell ref="BM2:BO2"/>
+    <mergeCell ref="AX2:AZ2"/>
+    <mergeCell ref="BA2:BC2"/>
+    <mergeCell ref="BD2:BF2"/>
+    <mergeCell ref="BV3:BX3"/>
+    <mergeCell ref="BS1:BU1"/>
+    <mergeCell ref="BV1:BX1"/>
+    <mergeCell ref="AU1:AW1"/>
+    <mergeCell ref="AX1:AZ1"/>
+    <mergeCell ref="BA1:BC1"/>
+    <mergeCell ref="BD1:BF1"/>
+    <mergeCell ref="BG1:BI1"/>
+    <mergeCell ref="BJ1:BL1"/>
+    <mergeCell ref="AU3:AW3"/>
+    <mergeCell ref="AX3:AZ3"/>
+    <mergeCell ref="BA3:BC3"/>
+    <mergeCell ref="BD3:BF3"/>
+    <mergeCell ref="DF3:DH3"/>
+    <mergeCell ref="BS2:BU2"/>
+    <mergeCell ref="BV2:BX2"/>
+    <mergeCell ref="BY2:CA2"/>
+    <mergeCell ref="CB2:CD2"/>
+    <mergeCell ref="CE2:CG2"/>
+    <mergeCell ref="CH2:CJ2"/>
+    <mergeCell ref="CK2:CM2"/>
+    <mergeCell ref="CN2:CP2"/>
+    <mergeCell ref="CQ2:CS2"/>
+    <mergeCell ref="CZ2:DB2"/>
+    <mergeCell ref="DC2:DE2"/>
+    <mergeCell ref="CE3:CG3"/>
+    <mergeCell ref="CH3:CJ3"/>
+    <mergeCell ref="CK3:CM3"/>
+    <mergeCell ref="CQ3:CS3"/>
+    <mergeCell ref="CB3:CD3"/>
     <mergeCell ref="DF1:DH1"/>
     <mergeCell ref="DF2:DH2"/>
     <mergeCell ref="BY3:CA3"/>
@@ -11196,93 +11285,6 @@
     <mergeCell ref="CZ3:DB3"/>
     <mergeCell ref="CN3:CP3"/>
     <mergeCell ref="BS3:BU3"/>
-    <mergeCell ref="DF3:DH3"/>
-    <mergeCell ref="BS2:BU2"/>
-    <mergeCell ref="BV2:BX2"/>
-    <mergeCell ref="BY2:CA2"/>
-    <mergeCell ref="CB2:CD2"/>
-    <mergeCell ref="CE2:CG2"/>
-    <mergeCell ref="CH2:CJ2"/>
-    <mergeCell ref="CK2:CM2"/>
-    <mergeCell ref="CN2:CP2"/>
-    <mergeCell ref="CQ2:CS2"/>
-    <mergeCell ref="CZ2:DB2"/>
-    <mergeCell ref="DC2:DE2"/>
-    <mergeCell ref="CE3:CG3"/>
-    <mergeCell ref="CH3:CJ3"/>
-    <mergeCell ref="CK3:CM3"/>
-    <mergeCell ref="CQ3:CS3"/>
-    <mergeCell ref="CB3:CD3"/>
-    <mergeCell ref="BV1:BX1"/>
-    <mergeCell ref="AU1:AW1"/>
-    <mergeCell ref="AX1:AZ1"/>
-    <mergeCell ref="BA1:BC1"/>
-    <mergeCell ref="BD1:BF1"/>
-    <mergeCell ref="BG1:BI1"/>
-    <mergeCell ref="BJ1:BL1"/>
-    <mergeCell ref="AU3:AW3"/>
-    <mergeCell ref="AX3:AZ3"/>
-    <mergeCell ref="BA3:BC3"/>
-    <mergeCell ref="BD3:BF3"/>
-    <mergeCell ref="BY1:CA1"/>
-    <mergeCell ref="Q2:S2"/>
-    <mergeCell ref="N1:P1"/>
-    <mergeCell ref="Q1:S1"/>
-    <mergeCell ref="T1:V1"/>
-    <mergeCell ref="T2:V2"/>
-    <mergeCell ref="BP1:BR1"/>
-    <mergeCell ref="BP2:BR2"/>
-    <mergeCell ref="BP3:BR3"/>
-    <mergeCell ref="BG3:BI3"/>
-    <mergeCell ref="BJ3:BL3"/>
-    <mergeCell ref="BM3:BO3"/>
-    <mergeCell ref="AI3:AK3"/>
-    <mergeCell ref="AL3:AN3"/>
-    <mergeCell ref="AO3:AQ3"/>
-    <mergeCell ref="AR3:AT3"/>
-    <mergeCell ref="BM1:BO1"/>
-    <mergeCell ref="BJ2:BL2"/>
-    <mergeCell ref="BM2:BO2"/>
-    <mergeCell ref="AX2:AZ2"/>
-    <mergeCell ref="BA2:BC2"/>
-    <mergeCell ref="BD2:BF2"/>
-    <mergeCell ref="BV3:BX3"/>
-    <mergeCell ref="BS1:BU1"/>
-    <mergeCell ref="CB1:CD1"/>
-    <mergeCell ref="B1:D1"/>
-    <mergeCell ref="E1:G1"/>
-    <mergeCell ref="H1:J1"/>
-    <mergeCell ref="K1:M1"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="K2:M2"/>
-    <mergeCell ref="N2:P2"/>
-    <mergeCell ref="BG2:BI2"/>
-    <mergeCell ref="W1:Y1"/>
-    <mergeCell ref="Z1:AB1"/>
-    <mergeCell ref="AC1:AE1"/>
-    <mergeCell ref="AF1:AH1"/>
-    <mergeCell ref="W2:Y2"/>
-    <mergeCell ref="Z2:AB2"/>
-    <mergeCell ref="AC2:AE2"/>
-    <mergeCell ref="AF2:AH2"/>
-    <mergeCell ref="AI2:AK2"/>
-    <mergeCell ref="AL2:AN2"/>
-    <mergeCell ref="AO2:AQ2"/>
-    <mergeCell ref="AR2:AT2"/>
-    <mergeCell ref="AU2:AW2"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="E3:G3"/>
-    <mergeCell ref="Z3:AB3"/>
-    <mergeCell ref="AC3:AE3"/>
-    <mergeCell ref="AF3:AH3"/>
-    <mergeCell ref="H3:J3"/>
-    <mergeCell ref="K3:M3"/>
-    <mergeCell ref="N3:P3"/>
-    <mergeCell ref="Q3:S3"/>
-    <mergeCell ref="T3:V3"/>
-    <mergeCell ref="W3:Y3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -11319,81 +11321,81 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:39" s="1" customFormat="1" ht="72" customHeight="1" thickBot="1">
-      <c r="A1" s="64" t="s">
+      <c r="A1" s="73" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="73" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="64" t="s">
+      <c r="C1" s="73" t="s">
+        <v>98</v>
+      </c>
+      <c r="D1" s="73" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="64" t="s">
+      <c r="E1" s="73" t="s">
         <v>99</v>
       </c>
-      <c r="D1" s="64" t="s">
+      <c r="F1" s="73" t="s">
         <v>9</v>
       </c>
-      <c r="E1" s="64" t="s">
-        <v>100</v>
-      </c>
-      <c r="F1" s="64" t="s">
+      <c r="G1" s="73" t="s">
         <v>10</v>
       </c>
-      <c r="G1" s="64" t="s">
+      <c r="H1" s="73" t="s">
         <v>11</v>
       </c>
-      <c r="H1" s="64" t="s">
+      <c r="I1" s="85" t="s">
         <v>12</v>
       </c>
-      <c r="I1" s="68" t="s">
-        <v>13</v>
-      </c>
-      <c r="J1" s="64" t="s">
+      <c r="J1" s="73" t="s">
         <v>111</v>
       </c>
-      <c r="K1" s="64" t="s">
+      <c r="K1" s="73" t="s">
+        <v>14</v>
+      </c>
+      <c r="L1" s="83" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1" s="73" t="s">
         <v>15</v>
       </c>
-      <c r="L1" s="66" t="s">
-        <v>25</v>
-      </c>
-      <c r="M1" s="64" t="s">
+      <c r="N1" s="73" t="s">
         <v>16</v>
       </c>
-      <c r="N1" s="64" t="s">
+      <c r="O1" s="73" t="s">
         <v>17</v>
       </c>
-      <c r="O1" s="64" t="s">
+      <c r="P1" s="80" t="s">
         <v>18</v>
       </c>
-      <c r="P1" s="75" t="s">
+      <c r="Q1" s="81"/>
+      <c r="R1" s="82"/>
+      <c r="S1" s="75" t="s">
         <v>19</v>
       </c>
-      <c r="Q1" s="76"/>
-      <c r="R1" s="77"/>
-      <c r="S1" s="70" t="s">
+      <c r="T1" s="76"/>
+      <c r="U1" s="75" t="s">
         <v>20</v>
       </c>
-      <c r="T1" s="71"/>
-      <c r="U1" s="70" t="s">
+      <c r="V1" s="77"/>
+      <c r="W1" s="78" t="s">
         <v>21</v>
       </c>
-      <c r="V1" s="72"/>
-      <c r="W1" s="73" t="s">
+      <c r="X1" s="73" t="s">
+        <v>105</v>
+      </c>
+      <c r="Y1" s="73" t="s">
+        <v>103</v>
+      </c>
+      <c r="Z1" s="78" t="s">
+        <v>104</v>
+      </c>
+      <c r="AA1" s="73" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="64" t="s">
-        <v>106</v>
-      </c>
-      <c r="Y1" s="64" t="s">
-        <v>104</v>
-      </c>
-      <c r="Z1" s="73" t="s">
-        <v>105</v>
-      </c>
-      <c r="AA1" s="64" t="s">
+      <c r="AB1" s="73" t="s">
         <v>23</v>
-      </c>
-      <c r="AB1" s="64" t="s">
-        <v>24</v>
       </c>
       <c r="AE1" s="2"/>
       <c r="AF1" s="2"/>
@@ -11406,56 +11408,56 @@
       <c r="AM1" s="2"/>
     </row>
     <row r="2" spans="1:39" s="1" customFormat="1" ht="48" customHeight="1" thickBot="1">
-      <c r="A2" s="65"/>
-      <c r="B2" s="65"/>
-      <c r="C2" s="65"/>
-      <c r="D2" s="65"/>
-      <c r="E2" s="65"/>
-      <c r="F2" s="65"/>
-      <c r="G2" s="65"/>
-      <c r="H2" s="65"/>
-      <c r="I2" s="69" t="s">
+      <c r="A2" s="74"/>
+      <c r="B2" s="74"/>
+      <c r="C2" s="74"/>
+      <c r="D2" s="74"/>
+      <c r="E2" s="74"/>
+      <c r="F2" s="74"/>
+      <c r="G2" s="74"/>
+      <c r="H2" s="74"/>
+      <c r="I2" s="86" t="s">
+        <v>12</v>
+      </c>
+      <c r="J2" s="74" t="s">
         <v>13</v>
       </c>
-      <c r="J2" s="65" t="s">
+      <c r="K2" s="74" t="s">
         <v>14</v>
       </c>
-      <c r="K2" s="65" t="s">
-        <v>15</v>
-      </c>
-      <c r="L2" s="67" t="s">
+      <c r="L2" s="84" t="s">
+        <v>24</v>
+      </c>
+      <c r="M2" s="74"/>
+      <c r="N2" s="74"/>
+      <c r="O2" s="74"/>
+      <c r="P2" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="S2" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="M2" s="65"/>
-      <c r="N2" s="65"/>
-      <c r="O2" s="65"/>
-      <c r="P2" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="Q2" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="R2" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="S2" s="4" t="s">
+      <c r="T2" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="T2" s="4" t="s">
-        <v>27</v>
-      </c>
       <c r="U2" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="V2" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="V2" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="W2" s="74"/>
-      <c r="X2" s="65"/>
-      <c r="Y2" s="65"/>
-      <c r="Z2" s="74"/>
-      <c r="AA2" s="65"/>
-      <c r="AB2" s="65"/>
+      <c r="W2" s="79"/>
+      <c r="X2" s="74"/>
+      <c r="Y2" s="74"/>
+      <c r="Z2" s="79"/>
+      <c r="AA2" s="74"/>
+      <c r="AB2" s="74"/>
       <c r="AE2" s="2"/>
       <c r="AF2" s="2"/>
       <c r="AG2" s="2"/>
@@ -11544,10 +11546,10 @@
         <v>7500</v>
       </c>
       <c r="AA3" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB3" s="11" t="s">
         <v>28</v>
-      </c>
-      <c r="AB3" s="11" t="s">
-        <v>29</v>
       </c>
       <c r="AE3" s="2"/>
       <c r="AF3" s="2"/>
@@ -11637,10 +11639,10 @@
         <v>12503</v>
       </c>
       <c r="AA4" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="AB4" s="13" t="s">
         <v>30</v>
-      </c>
-      <c r="AB4" s="13" t="s">
-        <v>31</v>
       </c>
       <c r="AE4" s="2"/>
       <c r="AF4" s="2"/>
@@ -11730,10 +11732,10 @@
         <v>17003</v>
       </c>
       <c r="AA5" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="AB5" s="13" t="s">
         <v>32</v>
-      </c>
-      <c r="AB5" s="13" t="s">
-        <v>33</v>
       </c>
       <c r="AE5" s="2"/>
       <c r="AF5" s="2"/>
@@ -11823,10 +11825,10 @@
         <v>22455</v>
       </c>
       <c r="AA6" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB6" s="13" t="s">
         <v>34</v>
-      </c>
-      <c r="AB6" s="13" t="s">
-        <v>35</v>
       </c>
       <c r="AE6" s="2"/>
       <c r="AF6" s="2"/>
@@ -11916,10 +11918,10 @@
         <v>29205</v>
       </c>
       <c r="AA7" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="AB7" s="13" t="s">
         <v>36</v>
-      </c>
-      <c r="AB7" s="13" t="s">
-        <v>37</v>
       </c>
       <c r="AE7" s="2"/>
       <c r="AF7" s="2"/>
@@ -12009,10 +12011,10 @@
         <v>39998</v>
       </c>
       <c r="AA8" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="AB8" s="13" t="s">
         <v>38</v>
-      </c>
-      <c r="AB8" s="13" t="s">
-        <v>39</v>
       </c>
       <c r="AE8" s="2"/>
       <c r="AF8" s="2"/>
@@ -12102,10 +12104,10 @@
         <v>51803</v>
       </c>
       <c r="AA9" s="41" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="AB9" s="42" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="AE9" s="59"/>
       <c r="AF9" s="59"/>
@@ -12195,10 +12197,10 @@
         <v>63615</v>
       </c>
       <c r="AA10" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="AB10" s="13" t="s">
         <v>41</v>
-      </c>
-      <c r="AB10" s="13" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="11" spans="1:39" s="43" customFormat="1" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
@@ -12279,10 +12281,10 @@
         <v>75383</v>
       </c>
       <c r="AA11" s="41" t="s">
+        <v>42</v>
+      </c>
+      <c r="AB11" s="42" t="s">
         <v>43</v>
-      </c>
-      <c r="AB11" s="42" t="s">
-        <v>44</v>
       </c>
       <c r="AE11" s="44"/>
       <c r="AF11" s="44"/>
@@ -12372,10 +12374,10 @@
         <v>90458</v>
       </c>
       <c r="AA12" s="41" t="s">
+        <v>44</v>
+      </c>
+      <c r="AB12" s="42" t="s">
         <v>45</v>
-      </c>
-      <c r="AB12" s="42" t="s">
-        <v>46</v>
       </c>
       <c r="AE12" s="44"/>
       <c r="AF12" s="44"/>
@@ -12465,10 +12467,10 @@
         <v>114503</v>
       </c>
       <c r="AA13" s="41" t="s">
+        <v>46</v>
+      </c>
+      <c r="AB13" s="42" t="s">
         <v>47</v>
-      </c>
-      <c r="AB13" s="42" t="s">
-        <v>48</v>
       </c>
       <c r="AE13" s="44"/>
       <c r="AF13" s="44"/>
@@ -12558,10 +12560,10 @@
         <v>141975</v>
       </c>
       <c r="AA14" s="41" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB14" s="42" t="s">
         <v>49</v>
-      </c>
-      <c r="AB14" s="42" t="s">
-        <v>50</v>
       </c>
       <c r="AE14" s="44"/>
       <c r="AF14" s="44"/>
@@ -12651,10 +12653,10 @@
         <v>174615</v>
       </c>
       <c r="AA15" s="41" t="s">
+        <v>50</v>
+      </c>
+      <c r="AB15" s="42" t="s">
         <v>51</v>
-      </c>
-      <c r="AB15" s="42" t="s">
-        <v>52</v>
       </c>
       <c r="AE15" s="44"/>
       <c r="AF15" s="44"/>
@@ -12744,10 +12746,10 @@
         <v>213345</v>
       </c>
       <c r="AA16" s="41" t="s">
+        <v>52</v>
+      </c>
+      <c r="AB16" s="42" t="s">
         <v>53</v>
-      </c>
-      <c r="AB16" s="42" t="s">
-        <v>54</v>
       </c>
       <c r="AE16" s="44"/>
       <c r="AF16" s="44"/>
@@ -12837,10 +12839,10 @@
         <v>266505</v>
       </c>
       <c r="AA17" s="41" t="s">
+        <v>54</v>
+      </c>
+      <c r="AB17" s="42" t="s">
         <v>55</v>
-      </c>
-      <c r="AB17" s="42" t="s">
-        <v>56</v>
       </c>
       <c r="AE17" s="44"/>
       <c r="AF17" s="44"/>
@@ -12930,10 +12932,10 @@
         <v>306480</v>
       </c>
       <c r="AA18" s="41" t="s">
+        <v>56</v>
+      </c>
+      <c r="AB18" s="42" t="s">
         <v>57</v>
-      </c>
-      <c r="AB18" s="42" t="s">
-        <v>58</v>
       </c>
       <c r="AE18" s="44"/>
       <c r="AF18" s="44"/>
@@ -13023,10 +13025,10 @@
         <v>375000</v>
       </c>
       <c r="AA19" s="41" t="s">
+        <v>58</v>
+      </c>
+      <c r="AB19" s="42" t="s">
         <v>59</v>
-      </c>
-      <c r="AB19" s="42" t="s">
-        <v>60</v>
       </c>
       <c r="AE19" s="44"/>
       <c r="AF19" s="44"/>
@@ -13116,10 +13118,10 @@
         <v>457500</v>
       </c>
       <c r="AA20" s="41" t="s">
+        <v>60</v>
+      </c>
+      <c r="AB20" s="42" t="s">
         <v>61</v>
-      </c>
-      <c r="AB20" s="42" t="s">
-        <v>62</v>
       </c>
       <c r="AE20" s="44"/>
       <c r="AF20" s="44"/>
@@ -13209,10 +13211,10 @@
         <v>549000</v>
       </c>
       <c r="AA21" s="41" t="s">
+        <v>62</v>
+      </c>
+      <c r="AB21" s="42" t="s">
         <v>63</v>
-      </c>
-      <c r="AB21" s="42" t="s">
-        <v>64</v>
       </c>
       <c r="AE21" s="44"/>
       <c r="AF21" s="44"/>
@@ -13302,10 +13304,10 @@
         <v>658800</v>
       </c>
       <c r="AA22" s="41" t="s">
+        <v>64</v>
+      </c>
+      <c r="AB22" s="42" t="s">
         <v>65</v>
-      </c>
-      <c r="AB22" s="42" t="s">
-        <v>66</v>
       </c>
       <c r="AE22" s="44"/>
       <c r="AF22" s="44"/>
@@ -13395,10 +13397,10 @@
         <v>757500</v>
       </c>
       <c r="AA23" s="41" t="s">
+        <v>66</v>
+      </c>
+      <c r="AB23" s="42" t="s">
         <v>67</v>
-      </c>
-      <c r="AB23" s="42" t="s">
-        <v>68</v>
       </c>
       <c r="AE23" s="44"/>
       <c r="AF23" s="44"/>
@@ -13488,10 +13490,10 @@
         <v>825750</v>
       </c>
       <c r="AA24" s="41" t="s">
+        <v>68</v>
+      </c>
+      <c r="AB24" s="42" t="s">
         <v>69</v>
-      </c>
-      <c r="AB24" s="42" t="s">
-        <v>70</v>
       </c>
       <c r="AE24" s="44"/>
       <c r="AF24" s="44"/>
@@ -13581,10 +13583,10 @@
         <v>974250</v>
       </c>
       <c r="AA25" s="41" t="s">
+        <v>70</v>
+      </c>
+      <c r="AB25" s="42" t="s">
         <v>71</v>
-      </c>
-      <c r="AB25" s="42" t="s">
-        <v>72</v>
       </c>
       <c r="AE25" s="44"/>
       <c r="AF25" s="44"/>
@@ -13597,7 +13599,7 @@
       <c r="AM25" s="44"/>
     </row>
     <row r="26" spans="1:39" s="43" customFormat="1" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
-      <c r="A26" s="78">
+      <c r="A26" s="64">
         <v>1392</v>
       </c>
       <c r="B26" s="36">
@@ -13674,10 +13676,10 @@
         <v>1217813</v>
       </c>
       <c r="AA26" s="41" t="s">
+        <v>72</v>
+      </c>
+      <c r="AB26" s="64" t="s">
         <v>73</v>
-      </c>
-      <c r="AB26" s="78" t="s">
-        <v>74</v>
       </c>
       <c r="AE26" s="44"/>
       <c r="AF26" s="44"/>
@@ -13690,7 +13692,7 @@
       <c r="AM26" s="44"/>
     </row>
     <row r="27" spans="1:39" s="43" customFormat="1" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
-      <c r="A27" s="79"/>
+      <c r="A27" s="65"/>
       <c r="B27" s="36">
         <v>8</v>
       </c>
@@ -13765,9 +13767,9 @@
         <v>1217813</v>
       </c>
       <c r="AA27" s="41" t="s">
-        <v>73</v>
-      </c>
-      <c r="AB27" s="79"/>
+        <v>72</v>
+      </c>
+      <c r="AB27" s="65"/>
       <c r="AE27" s="44"/>
       <c r="AF27" s="44"/>
       <c r="AG27" s="44"/>
@@ -13856,10 +13858,10 @@
         <v>1522275</v>
       </c>
       <c r="AA28" s="41" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="AB28" s="42" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="AE28" s="44"/>
       <c r="AF28" s="44"/>
@@ -13949,10 +13951,10 @@
         <v>1781063</v>
       </c>
       <c r="AA29" s="41" t="s">
+        <v>75</v>
+      </c>
+      <c r="AB29" s="42" t="s">
         <v>76</v>
-      </c>
-      <c r="AB29" s="42" t="s">
-        <v>77</v>
       </c>
       <c r="AE29" s="44"/>
       <c r="AF29" s="44"/>
@@ -13965,7 +13967,7 @@
       <c r="AM29" s="44"/>
     </row>
     <row r="30" spans="1:39" s="43" customFormat="1" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
-      <c r="A30" s="80">
+      <c r="A30" s="66">
         <v>1395</v>
       </c>
       <c r="B30" s="36">
@@ -14042,10 +14044,10 @@
         <v>2030415</v>
       </c>
       <c r="AA30" s="41" t="s">
+        <v>77</v>
+      </c>
+      <c r="AB30" s="68" t="s">
         <v>78</v>
-      </c>
-      <c r="AB30" s="82" t="s">
-        <v>79</v>
       </c>
       <c r="AE30" s="44"/>
       <c r="AF30" s="44"/>
@@ -14058,7 +14060,7 @@
       <c r="AM30" s="44"/>
     </row>
     <row r="31" spans="1:39" s="43" customFormat="1" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
-      <c r="A31" s="81"/>
+      <c r="A31" s="67"/>
       <c r="B31" s="36">
         <v>6</v>
       </c>
@@ -14133,9 +14135,9 @@
         <v>2030415</v>
       </c>
       <c r="AA31" s="41" t="s">
-        <v>78</v>
-      </c>
-      <c r="AB31" s="83"/>
+        <v>77</v>
+      </c>
+      <c r="AB31" s="69"/>
       <c r="AE31" s="44"/>
       <c r="AF31" s="44"/>
       <c r="AG31" s="44"/>
@@ -14224,10 +14226,10 @@
         <v>2324828</v>
       </c>
       <c r="AA32" s="41" t="s">
+        <v>79</v>
+      </c>
+      <c r="AB32" s="42" t="s">
         <v>80</v>
-      </c>
-      <c r="AB32" s="42" t="s">
-        <v>81</v>
       </c>
       <c r="AE32" s="44"/>
       <c r="AF32" s="44"/>
@@ -14317,10 +14319,10 @@
         <v>2778173</v>
       </c>
       <c r="AA33" s="41" t="s">
+        <v>81</v>
+      </c>
+      <c r="AB33" s="42" t="s">
         <v>82</v>
-      </c>
-      <c r="AB33" s="42" t="s">
-        <v>83</v>
       </c>
       <c r="AE33" s="44"/>
       <c r="AF33" s="44"/>
@@ -14410,10 +14412,10 @@
         <v>3792203</v>
       </c>
       <c r="AA34" s="41" t="s">
+        <v>83</v>
+      </c>
+      <c r="AB34" s="42" t="s">
         <v>84</v>
-      </c>
-      <c r="AB34" s="42" t="s">
-        <v>85</v>
       </c>
       <c r="AE34" s="44"/>
       <c r="AF34" s="44"/>
@@ -14426,7 +14428,7 @@
       <c r="AM34" s="44"/>
     </row>
     <row r="35" spans="1:39" s="43" customFormat="1" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
-      <c r="A35" s="84">
+      <c r="A35" s="70">
         <v>1399</v>
       </c>
       <c r="B35" s="36">
@@ -14503,10 +14505,10 @@
         <v>4588568</v>
       </c>
       <c r="AA35" s="41" t="s">
+        <v>85</v>
+      </c>
+      <c r="AB35" s="72" t="s">
         <v>86</v>
-      </c>
-      <c r="AB35" s="86" t="s">
-        <v>87</v>
       </c>
       <c r="AE35" s="44"/>
       <c r="AF35" s="44"/>
@@ -14519,7 +14521,7 @@
       <c r="AM35" s="44"/>
     </row>
     <row r="36" spans="1:39" s="43" customFormat="1" ht="32.25" customHeight="1" thickTop="1" thickBot="1">
-      <c r="A36" s="85"/>
+      <c r="A36" s="71"/>
       <c r="B36" s="36">
         <v>9</v>
       </c>
@@ -14594,9 +14596,9 @@
         <v>4776068</v>
       </c>
       <c r="AA36" s="41" t="s">
-        <v>88</v>
-      </c>
-      <c r="AB36" s="83"/>
+        <v>87</v>
+      </c>
+      <c r="AB36" s="69"/>
       <c r="AE36" s="44"/>
       <c r="AF36" s="44"/>
       <c r="AG36" s="44"/>
@@ -14685,10 +14687,10 @@
         <v>6638738</v>
       </c>
       <c r="AA37" s="41" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="AB37" s="42" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="AE37" s="44"/>
       <c r="AF37" s="44"/>
@@ -14778,10 +14780,10 @@
         <v>10449375</v>
       </c>
       <c r="AA38" s="41" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="AB38" s="42" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="AE38" s="44"/>
       <c r="AF38" s="44"/>
@@ -14871,10 +14873,10 @@
         <v>13270710</v>
       </c>
       <c r="AA39" s="41" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="AB39" s="42" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="AE39" s="44"/>
       <c r="AF39" s="44"/>
@@ -14966,10 +14968,10 @@
         <v>17915460</v>
       </c>
       <c r="AA40" s="41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="AB40" s="42" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="AE40" s="44"/>
       <c r="AF40" s="44"/>
@@ -15061,10 +15063,10 @@
         <v>25977420</v>
       </c>
       <c r="AA41" s="41" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AB41" s="42" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AE41" s="44"/>
       <c r="AF41" s="44"/>
@@ -15156,10 +15158,10 @@
         <v>41563875</v>
       </c>
       <c r="AA42" s="41" t="s">
+        <v>96</v>
+      </c>
+      <c r="AB42" s="41" t="s">
         <v>97</v>
-      </c>
-      <c r="AB42" s="41" t="s">
-        <v>98</v>
       </c>
       <c r="AC42" s="55"/>
       <c r="AD42" s="55"/>
@@ -18137,12 +18139,18 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="A26:A27"/>
-    <mergeCell ref="AB26:AB27"/>
-    <mergeCell ref="A30:A31"/>
-    <mergeCell ref="AB30:AB31"/>
-    <mergeCell ref="A35:A36"/>
-    <mergeCell ref="AB35:AB36"/>
+    <mergeCell ref="K1:K2"/>
+    <mergeCell ref="L1:L2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="I1:I2"/>
+    <mergeCell ref="J1:J2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:E2"/>
     <mergeCell ref="AB1:AB2"/>
     <mergeCell ref="M1:M2"/>
     <mergeCell ref="N1:N2"/>
@@ -18155,18 +18163,12 @@
     <mergeCell ref="Z1:Z2"/>
     <mergeCell ref="AA1:AA2"/>
     <mergeCell ref="P1:R1"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="K1:K2"/>
-    <mergeCell ref="L1:L2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="G1:G2"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="I1:I2"/>
-    <mergeCell ref="J1:J2"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="AB26:AB27"/>
+    <mergeCell ref="A30:A31"/>
+    <mergeCell ref="AB30:AB31"/>
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="AB35:AB36"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>

</xml_diff>